<commit_message>
Tracker: weekdays only, start trading from 26 Sep 2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USJ2QdZK7Rdpo1YWsPGJTB
</commit_message>
<xml_diff>
--- a/Trading_PnL_Tracker.xlsx
+++ b/Trading_PnL_Tracker.xlsx
@@ -37,7 +37,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Provided by you: Day 1 = 25 Sep 2026. Each row is one calendar day.</t>
+          <t xml:space="preserve">Provided by you: you start trading tomorrow (26 Sep 2026). If this falls on a weekend, Day 1 moves to the next Monday. Only weekdays (Mon–Fri) get rows.</t>
         </r>
       </text>
     </comment>
@@ -106,7 +106,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t xml:space="preserve">Daily Trading P/L Tracker — ₹4,230 → ₹1,00,000 Goal</t>
   </si>
@@ -120,7 +120,7 @@
     <t xml:space="preserve">DASHBOARD  (all calculated)</t>
   </si>
   <si>
-    <t xml:space="preserve">Start date (Day 1)</t>
+    <t xml:space="preserve">Start trading from</t>
   </si>
   <si>
     <t xml:space="preserve">Current balance</t>
@@ -162,7 +162,7 @@
     <t xml:space="preserve">Projected goal date*</t>
   </si>
   <si>
-    <t xml:space="preserve">Legend:  Yellow cells with blue text = your inputs (Settings, Actual P/L, Done?, Notes).  All other cells are formulas — don't overwrite them.  Grey italic rows = Projection (target assumed met), white rows = Actual.   *Projection-based figures.</t>
+    <t xml:space="preserve">Rows = trading days only (Mon–Fri, weekends skipped).  Legend:  Yellow cells with blue text = your inputs (Settings, Actual P/L, Done?, Notes).  All other cells are formulas — don't overwrite them.  Grey italic rows = Projection (target assumed met), white rows = Actual.   *Projection-based figures.</t>
   </si>
   <si>
     <t xml:space="preserve">Day</t>
@@ -240,7 +240,7 @@
     <t xml:space="preserve">   • Rows marked "Projection" (grey italic) assume every daily profit target is hit. This is an illustration, not a prediction or guarantee.</t>
   </si>
   <si>
-    <t xml:space="preserve">   • With no losses at all, reaching ₹1,00,000 from ₹4,230 at 3%/day takes about 108 days (with paisa rounding). Any loss or no-trade day extends the timeline.</t>
+    <t xml:space="preserve">   • With no losses at all, reaching ₹1,00,000 from ₹4,230 at 3%/day takes about 108 trading days (with paisa rounding). Any loss or no-trade day extends the timeline.</t>
   </si>
   <si>
     <t xml:space="preserve">   • The table stops at the first day whose projected (or actual) close reaches the goal, and extends automatically after losses (up to 500 days).</t>
@@ -249,7 +249,13 @@
     <t xml:space="preserve">Other notes</t>
   </si>
   <si>
-    <t xml:space="preserve">   • Dates are consecutive calendar days from 25-Sep-2026 (Day 1). Enter 0 for weekends/holidays you don't trade.</t>
+    <t xml:space="preserve">   • Only trading days (Monday–Friday) get rows — Saturdays and Sundays are skipped automatically.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • Start date is 26-Sep-2026 (Sat), so Day 1 is Monday 28-Sep-2026. Change the "Start trading from" setting to move everything.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • Market holidays on weekdays still get a row — enter 0 on those days.</t>
   </si>
   <si>
     <t xml:space="preserve">   • Amounts are rounded to the paisa (2 decimals). Targets and limits = ROUND(opening capital × 3%, 2).</t>
@@ -1023,7 +1029,7 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="5" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>5</v>
@@ -1131,8 +1137,8 @@
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="14" t="n">
-        <f aca="false">$C$5+$J$6</f>
-        <v>46290</v>
+        <f aca="false">WORKDAY($C$5-1,$J$6+1)</f>
+        <v>46293</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>17</v>
@@ -1140,7 +1146,7 @@
       <c r="I9" s="6"/>
       <c r="J9" s="14" t="n">
         <f aca="false">IF($G$5&gt;=$C$7,"Goal reached",IF(AND($C$512&lt;&gt;"",N($F$512)&lt;$C$7),"Beyond 500 rows",MAX($B$13:$B$512)))</f>
-        <v>46397</v>
+        <v>46442</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1199,8 +1205,8 @@
         <v>1</v>
       </c>
       <c r="B13" s="19" t="n">
-        <f aca="false">IF(C13="","",$C$5+A13-1)</f>
-        <v>46290</v>
+        <f aca="false">IF(C13="","",WORKDAY($C$5-1,A13))</f>
+        <v>46293</v>
       </c>
       <c r="C13" s="20" t="n">
         <f aca="false">$C$6</f>
@@ -1236,8 +1242,8 @@
         <v>2</v>
       </c>
       <c r="B14" s="19" t="n">
-        <f aca="false">IF(C14="","",$C$5+A14-1)</f>
-        <v>46291</v>
+        <f aca="false">IF(C14="","",WORKDAY($C$5-1,A14))</f>
+        <v>46294</v>
       </c>
       <c r="C14" s="20" t="n">
         <f aca="false">IF(C13="","",IF(OR(IF(ISNUMBER(G13),H13,F13)&gt;=$C$7,IF(ISNUMBER(G13),H13,F13)&lt;=0),"",IF(ISNUMBER(G13),H13,F13)))</f>
@@ -1273,8 +1279,8 @@
         <v>3</v>
       </c>
       <c r="B15" s="19" t="n">
-        <f aca="false">IF(C15="","",$C$5+A15-1)</f>
-        <v>46292</v>
+        <f aca="false">IF(C15="","",WORKDAY($C$5-1,A15))</f>
+        <v>46295</v>
       </c>
       <c r="C15" s="20" t="n">
         <f aca="false">IF(C14="","",IF(OR(IF(ISNUMBER(G14),H14,F14)&gt;=$C$7,IF(ISNUMBER(G14),H14,F14)&lt;=0),"",IF(ISNUMBER(G14),H14,F14)))</f>
@@ -1310,8 +1316,8 @@
         <v>4</v>
       </c>
       <c r="B16" s="19" t="n">
-        <f aca="false">IF(C16="","",$C$5+A16-1)</f>
-        <v>46293</v>
+        <f aca="false">IF(C16="","",WORKDAY($C$5-1,A16))</f>
+        <v>46296</v>
       </c>
       <c r="C16" s="20" t="n">
         <f aca="false">IF(C15="","",IF(OR(IF(ISNUMBER(G15),H15,F15)&gt;=$C$7,IF(ISNUMBER(G15),H15,F15)&lt;=0),"",IF(ISNUMBER(G15),H15,F15)))</f>
@@ -1347,8 +1353,8 @@
         <v>5</v>
       </c>
       <c r="B17" s="19" t="n">
-        <f aca="false">IF(C17="","",$C$5+A17-1)</f>
-        <v>46294</v>
+        <f aca="false">IF(C17="","",WORKDAY($C$5-1,A17))</f>
+        <v>46297</v>
       </c>
       <c r="C17" s="20" t="n">
         <f aca="false">IF(C16="","",IF(OR(IF(ISNUMBER(G16),H16,F16)&gt;=$C$7,IF(ISNUMBER(G16),H16,F16)&lt;=0),"",IF(ISNUMBER(G16),H16,F16)))</f>
@@ -1384,8 +1390,8 @@
         <v>6</v>
       </c>
       <c r="B18" s="19" t="n">
-        <f aca="false">IF(C18="","",$C$5+A18-1)</f>
-        <v>46295</v>
+        <f aca="false">IF(C18="","",WORKDAY($C$5-1,A18))</f>
+        <v>46300</v>
       </c>
       <c r="C18" s="20" t="n">
         <f aca="false">IF(C17="","",IF(OR(IF(ISNUMBER(G17),H17,F17)&gt;=$C$7,IF(ISNUMBER(G17),H17,F17)&lt;=0),"",IF(ISNUMBER(G17),H17,F17)))</f>
@@ -1421,8 +1427,8 @@
         <v>7</v>
       </c>
       <c r="B19" s="19" t="n">
-        <f aca="false">IF(C19="","",$C$5+A19-1)</f>
-        <v>46296</v>
+        <f aca="false">IF(C19="","",WORKDAY($C$5-1,A19))</f>
+        <v>46301</v>
       </c>
       <c r="C19" s="20" t="n">
         <f aca="false">IF(C18="","",IF(OR(IF(ISNUMBER(G18),H18,F18)&gt;=$C$7,IF(ISNUMBER(G18),H18,F18)&lt;=0),"",IF(ISNUMBER(G18),H18,F18)))</f>
@@ -1458,8 +1464,8 @@
         <v>8</v>
       </c>
       <c r="B20" s="19" t="n">
-        <f aca="false">IF(C20="","",$C$5+A20-1)</f>
-        <v>46297</v>
+        <f aca="false">IF(C20="","",WORKDAY($C$5-1,A20))</f>
+        <v>46302</v>
       </c>
       <c r="C20" s="20" t="n">
         <f aca="false">IF(C19="","",IF(OR(IF(ISNUMBER(G19),H19,F19)&gt;=$C$7,IF(ISNUMBER(G19),H19,F19)&lt;=0),"",IF(ISNUMBER(G19),H19,F19)))</f>
@@ -1495,8 +1501,8 @@
         <v>9</v>
       </c>
       <c r="B21" s="19" t="n">
-        <f aca="false">IF(C21="","",$C$5+A21-1)</f>
-        <v>46298</v>
+        <f aca="false">IF(C21="","",WORKDAY($C$5-1,A21))</f>
+        <v>46303</v>
       </c>
       <c r="C21" s="20" t="n">
         <f aca="false">IF(C20="","",IF(OR(IF(ISNUMBER(G20),H20,F20)&gt;=$C$7,IF(ISNUMBER(G20),H20,F20)&lt;=0),"",IF(ISNUMBER(G20),H20,F20)))</f>
@@ -1532,8 +1538,8 @@
         <v>10</v>
       </c>
       <c r="B22" s="19" t="n">
-        <f aca="false">IF(C22="","",$C$5+A22-1)</f>
-        <v>46299</v>
+        <f aca="false">IF(C22="","",WORKDAY($C$5-1,A22))</f>
+        <v>46304</v>
       </c>
       <c r="C22" s="20" t="n">
         <f aca="false">IF(C21="","",IF(OR(IF(ISNUMBER(G21),H21,F21)&gt;=$C$7,IF(ISNUMBER(G21),H21,F21)&lt;=0),"",IF(ISNUMBER(G21),H21,F21)))</f>
@@ -1569,8 +1575,8 @@
         <v>11</v>
       </c>
       <c r="B23" s="19" t="n">
-        <f aca="false">IF(C23="","",$C$5+A23-1)</f>
-        <v>46300</v>
+        <f aca="false">IF(C23="","",WORKDAY($C$5-1,A23))</f>
+        <v>46307</v>
       </c>
       <c r="C23" s="20" t="n">
         <f aca="false">IF(C22="","",IF(OR(IF(ISNUMBER(G22),H22,F22)&gt;=$C$7,IF(ISNUMBER(G22),H22,F22)&lt;=0),"",IF(ISNUMBER(G22),H22,F22)))</f>
@@ -1606,8 +1612,8 @@
         <v>12</v>
       </c>
       <c r="B24" s="19" t="n">
-        <f aca="false">IF(C24="","",$C$5+A24-1)</f>
-        <v>46301</v>
+        <f aca="false">IF(C24="","",WORKDAY($C$5-1,A24))</f>
+        <v>46308</v>
       </c>
       <c r="C24" s="20" t="n">
         <f aca="false">IF(C23="","",IF(OR(IF(ISNUMBER(G23),H23,F23)&gt;=$C$7,IF(ISNUMBER(G23),H23,F23)&lt;=0),"",IF(ISNUMBER(G23),H23,F23)))</f>
@@ -1643,8 +1649,8 @@
         <v>13</v>
       </c>
       <c r="B25" s="19" t="n">
-        <f aca="false">IF(C25="","",$C$5+A25-1)</f>
-        <v>46302</v>
+        <f aca="false">IF(C25="","",WORKDAY($C$5-1,A25))</f>
+        <v>46309</v>
       </c>
       <c r="C25" s="20" t="n">
         <f aca="false">IF(C24="","",IF(OR(IF(ISNUMBER(G24),H24,F24)&gt;=$C$7,IF(ISNUMBER(G24),H24,F24)&lt;=0),"",IF(ISNUMBER(G24),H24,F24)))</f>
@@ -1680,8 +1686,8 @@
         <v>14</v>
       </c>
       <c r="B26" s="19" t="n">
-        <f aca="false">IF(C26="","",$C$5+A26-1)</f>
-        <v>46303</v>
+        <f aca="false">IF(C26="","",WORKDAY($C$5-1,A26))</f>
+        <v>46310</v>
       </c>
       <c r="C26" s="20" t="n">
         <f aca="false">IF(C25="","",IF(OR(IF(ISNUMBER(G25),H25,F25)&gt;=$C$7,IF(ISNUMBER(G25),H25,F25)&lt;=0),"",IF(ISNUMBER(G25),H25,F25)))</f>
@@ -1717,8 +1723,8 @@
         <v>15</v>
       </c>
       <c r="B27" s="19" t="n">
-        <f aca="false">IF(C27="","",$C$5+A27-1)</f>
-        <v>46304</v>
+        <f aca="false">IF(C27="","",WORKDAY($C$5-1,A27))</f>
+        <v>46311</v>
       </c>
       <c r="C27" s="20" t="n">
         <f aca="false">IF(C26="","",IF(OR(IF(ISNUMBER(G26),H26,F26)&gt;=$C$7,IF(ISNUMBER(G26),H26,F26)&lt;=0),"",IF(ISNUMBER(G26),H26,F26)))</f>
@@ -1754,8 +1760,8 @@
         <v>16</v>
       </c>
       <c r="B28" s="19" t="n">
-        <f aca="false">IF(C28="","",$C$5+A28-1)</f>
-        <v>46305</v>
+        <f aca="false">IF(C28="","",WORKDAY($C$5-1,A28))</f>
+        <v>46314</v>
       </c>
       <c r="C28" s="20" t="n">
         <f aca="false">IF(C27="","",IF(OR(IF(ISNUMBER(G27),H27,F27)&gt;=$C$7,IF(ISNUMBER(G27),H27,F27)&lt;=0),"",IF(ISNUMBER(G27),H27,F27)))</f>
@@ -1791,8 +1797,8 @@
         <v>17</v>
       </c>
       <c r="B29" s="19" t="n">
-        <f aca="false">IF(C29="","",$C$5+A29-1)</f>
-        <v>46306</v>
+        <f aca="false">IF(C29="","",WORKDAY($C$5-1,A29))</f>
+        <v>46315</v>
       </c>
       <c r="C29" s="20" t="n">
         <f aca="false">IF(C28="","",IF(OR(IF(ISNUMBER(G28),H28,F28)&gt;=$C$7,IF(ISNUMBER(G28),H28,F28)&lt;=0),"",IF(ISNUMBER(G28),H28,F28)))</f>
@@ -1828,8 +1834,8 @@
         <v>18</v>
       </c>
       <c r="B30" s="19" t="n">
-        <f aca="false">IF(C30="","",$C$5+A30-1)</f>
-        <v>46307</v>
+        <f aca="false">IF(C30="","",WORKDAY($C$5-1,A30))</f>
+        <v>46316</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">IF(C29="","",IF(OR(IF(ISNUMBER(G29),H29,F29)&gt;=$C$7,IF(ISNUMBER(G29),H29,F29)&lt;=0),"",IF(ISNUMBER(G29),H29,F29)))</f>
@@ -1865,8 +1871,8 @@
         <v>19</v>
       </c>
       <c r="B31" s="19" t="n">
-        <f aca="false">IF(C31="","",$C$5+A31-1)</f>
-        <v>46308</v>
+        <f aca="false">IF(C31="","",WORKDAY($C$5-1,A31))</f>
+        <v>46317</v>
       </c>
       <c r="C31" s="20" t="n">
         <f aca="false">IF(C30="","",IF(OR(IF(ISNUMBER(G30),H30,F30)&gt;=$C$7,IF(ISNUMBER(G30),H30,F30)&lt;=0),"",IF(ISNUMBER(G30),H30,F30)))</f>
@@ -1902,8 +1908,8 @@
         <v>20</v>
       </c>
       <c r="B32" s="19" t="n">
-        <f aca="false">IF(C32="","",$C$5+A32-1)</f>
-        <v>46309</v>
+        <f aca="false">IF(C32="","",WORKDAY($C$5-1,A32))</f>
+        <v>46318</v>
       </c>
       <c r="C32" s="20" t="n">
         <f aca="false">IF(C31="","",IF(OR(IF(ISNUMBER(G31),H31,F31)&gt;=$C$7,IF(ISNUMBER(G31),H31,F31)&lt;=0),"",IF(ISNUMBER(G31),H31,F31)))</f>
@@ -1939,8 +1945,8 @@
         <v>21</v>
       </c>
       <c r="B33" s="19" t="n">
-        <f aca="false">IF(C33="","",$C$5+A33-1)</f>
-        <v>46310</v>
+        <f aca="false">IF(C33="","",WORKDAY($C$5-1,A33))</f>
+        <v>46321</v>
       </c>
       <c r="C33" s="20" t="n">
         <f aca="false">IF(C32="","",IF(OR(IF(ISNUMBER(G32),H32,F32)&gt;=$C$7,IF(ISNUMBER(G32),H32,F32)&lt;=0),"",IF(ISNUMBER(G32),H32,F32)))</f>
@@ -1976,8 +1982,8 @@
         <v>22</v>
       </c>
       <c r="B34" s="19" t="n">
-        <f aca="false">IF(C34="","",$C$5+A34-1)</f>
-        <v>46311</v>
+        <f aca="false">IF(C34="","",WORKDAY($C$5-1,A34))</f>
+        <v>46322</v>
       </c>
       <c r="C34" s="20" t="n">
         <f aca="false">IF(C33="","",IF(OR(IF(ISNUMBER(G33),H33,F33)&gt;=$C$7,IF(ISNUMBER(G33),H33,F33)&lt;=0),"",IF(ISNUMBER(G33),H33,F33)))</f>
@@ -2013,8 +2019,8 @@
         <v>23</v>
       </c>
       <c r="B35" s="19" t="n">
-        <f aca="false">IF(C35="","",$C$5+A35-1)</f>
-        <v>46312</v>
+        <f aca="false">IF(C35="","",WORKDAY($C$5-1,A35))</f>
+        <v>46323</v>
       </c>
       <c r="C35" s="20" t="n">
         <f aca="false">IF(C34="","",IF(OR(IF(ISNUMBER(G34),H34,F34)&gt;=$C$7,IF(ISNUMBER(G34),H34,F34)&lt;=0),"",IF(ISNUMBER(G34),H34,F34)))</f>
@@ -2050,8 +2056,8 @@
         <v>24</v>
       </c>
       <c r="B36" s="19" t="n">
-        <f aca="false">IF(C36="","",$C$5+A36-1)</f>
-        <v>46313</v>
+        <f aca="false">IF(C36="","",WORKDAY($C$5-1,A36))</f>
+        <v>46324</v>
       </c>
       <c r="C36" s="20" t="n">
         <f aca="false">IF(C35="","",IF(OR(IF(ISNUMBER(G35),H35,F35)&gt;=$C$7,IF(ISNUMBER(G35),H35,F35)&lt;=0),"",IF(ISNUMBER(G35),H35,F35)))</f>
@@ -2087,8 +2093,8 @@
         <v>25</v>
       </c>
       <c r="B37" s="19" t="n">
-        <f aca="false">IF(C37="","",$C$5+A37-1)</f>
-        <v>46314</v>
+        <f aca="false">IF(C37="","",WORKDAY($C$5-1,A37))</f>
+        <v>46325</v>
       </c>
       <c r="C37" s="20" t="n">
         <f aca="false">IF(C36="","",IF(OR(IF(ISNUMBER(G36),H36,F36)&gt;=$C$7,IF(ISNUMBER(G36),H36,F36)&lt;=0),"",IF(ISNUMBER(G36),H36,F36)))</f>
@@ -2124,8 +2130,8 @@
         <v>26</v>
       </c>
       <c r="B38" s="19" t="n">
-        <f aca="false">IF(C38="","",$C$5+A38-1)</f>
-        <v>46315</v>
+        <f aca="false">IF(C38="","",WORKDAY($C$5-1,A38))</f>
+        <v>46328</v>
       </c>
       <c r="C38" s="20" t="n">
         <f aca="false">IF(C37="","",IF(OR(IF(ISNUMBER(G37),H37,F37)&gt;=$C$7,IF(ISNUMBER(G37),H37,F37)&lt;=0),"",IF(ISNUMBER(G37),H37,F37)))</f>
@@ -2161,8 +2167,8 @@
         <v>27</v>
       </c>
       <c r="B39" s="19" t="n">
-        <f aca="false">IF(C39="","",$C$5+A39-1)</f>
-        <v>46316</v>
+        <f aca="false">IF(C39="","",WORKDAY($C$5-1,A39))</f>
+        <v>46329</v>
       </c>
       <c r="C39" s="20" t="n">
         <f aca="false">IF(C38="","",IF(OR(IF(ISNUMBER(G38),H38,F38)&gt;=$C$7,IF(ISNUMBER(G38),H38,F38)&lt;=0),"",IF(ISNUMBER(G38),H38,F38)))</f>
@@ -2198,8 +2204,8 @@
         <v>28</v>
       </c>
       <c r="B40" s="19" t="n">
-        <f aca="false">IF(C40="","",$C$5+A40-1)</f>
-        <v>46317</v>
+        <f aca="false">IF(C40="","",WORKDAY($C$5-1,A40))</f>
+        <v>46330</v>
       </c>
       <c r="C40" s="20" t="n">
         <f aca="false">IF(C39="","",IF(OR(IF(ISNUMBER(G39),H39,F39)&gt;=$C$7,IF(ISNUMBER(G39),H39,F39)&lt;=0),"",IF(ISNUMBER(G39),H39,F39)))</f>
@@ -2235,8 +2241,8 @@
         <v>29</v>
       </c>
       <c r="B41" s="19" t="n">
-        <f aca="false">IF(C41="","",$C$5+A41-1)</f>
-        <v>46318</v>
+        <f aca="false">IF(C41="","",WORKDAY($C$5-1,A41))</f>
+        <v>46331</v>
       </c>
       <c r="C41" s="20" t="n">
         <f aca="false">IF(C40="","",IF(OR(IF(ISNUMBER(G40),H40,F40)&gt;=$C$7,IF(ISNUMBER(G40),H40,F40)&lt;=0),"",IF(ISNUMBER(G40),H40,F40)))</f>
@@ -2272,8 +2278,8 @@
         <v>30</v>
       </c>
       <c r="B42" s="19" t="n">
-        <f aca="false">IF(C42="","",$C$5+A42-1)</f>
-        <v>46319</v>
+        <f aca="false">IF(C42="","",WORKDAY($C$5-1,A42))</f>
+        <v>46332</v>
       </c>
       <c r="C42" s="20" t="n">
         <f aca="false">IF(C41="","",IF(OR(IF(ISNUMBER(G41),H41,F41)&gt;=$C$7,IF(ISNUMBER(G41),H41,F41)&lt;=0),"",IF(ISNUMBER(G41),H41,F41)))</f>
@@ -2309,8 +2315,8 @@
         <v>31</v>
       </c>
       <c r="B43" s="19" t="n">
-        <f aca="false">IF(C43="","",$C$5+A43-1)</f>
-        <v>46320</v>
+        <f aca="false">IF(C43="","",WORKDAY($C$5-1,A43))</f>
+        <v>46335</v>
       </c>
       <c r="C43" s="20" t="n">
         <f aca="false">IF(C42="","",IF(OR(IF(ISNUMBER(G42),H42,F42)&gt;=$C$7,IF(ISNUMBER(G42),H42,F42)&lt;=0),"",IF(ISNUMBER(G42),H42,F42)))</f>
@@ -2346,8 +2352,8 @@
         <v>32</v>
       </c>
       <c r="B44" s="19" t="n">
-        <f aca="false">IF(C44="","",$C$5+A44-1)</f>
-        <v>46321</v>
+        <f aca="false">IF(C44="","",WORKDAY($C$5-1,A44))</f>
+        <v>46336</v>
       </c>
       <c r="C44" s="20" t="n">
         <f aca="false">IF(C43="","",IF(OR(IF(ISNUMBER(G43),H43,F43)&gt;=$C$7,IF(ISNUMBER(G43),H43,F43)&lt;=0),"",IF(ISNUMBER(G43),H43,F43)))</f>
@@ -2383,8 +2389,8 @@
         <v>33</v>
       </c>
       <c r="B45" s="19" t="n">
-        <f aca="false">IF(C45="","",$C$5+A45-1)</f>
-        <v>46322</v>
+        <f aca="false">IF(C45="","",WORKDAY($C$5-1,A45))</f>
+        <v>46337</v>
       </c>
       <c r="C45" s="20" t="n">
         <f aca="false">IF(C44="","",IF(OR(IF(ISNUMBER(G44),H44,F44)&gt;=$C$7,IF(ISNUMBER(G44),H44,F44)&lt;=0),"",IF(ISNUMBER(G44),H44,F44)))</f>
@@ -2420,8 +2426,8 @@
         <v>34</v>
       </c>
       <c r="B46" s="19" t="n">
-        <f aca="false">IF(C46="","",$C$5+A46-1)</f>
-        <v>46323</v>
+        <f aca="false">IF(C46="","",WORKDAY($C$5-1,A46))</f>
+        <v>46338</v>
       </c>
       <c r="C46" s="20" t="n">
         <f aca="false">IF(C45="","",IF(OR(IF(ISNUMBER(G45),H45,F45)&gt;=$C$7,IF(ISNUMBER(G45),H45,F45)&lt;=0),"",IF(ISNUMBER(G45),H45,F45)))</f>
@@ -2457,8 +2463,8 @@
         <v>35</v>
       </c>
       <c r="B47" s="19" t="n">
-        <f aca="false">IF(C47="","",$C$5+A47-1)</f>
-        <v>46324</v>
+        <f aca="false">IF(C47="","",WORKDAY($C$5-1,A47))</f>
+        <v>46339</v>
       </c>
       <c r="C47" s="20" t="n">
         <f aca="false">IF(C46="","",IF(OR(IF(ISNUMBER(G46),H46,F46)&gt;=$C$7,IF(ISNUMBER(G46),H46,F46)&lt;=0),"",IF(ISNUMBER(G46),H46,F46)))</f>
@@ -2494,8 +2500,8 @@
         <v>36</v>
       </c>
       <c r="B48" s="19" t="n">
-        <f aca="false">IF(C48="","",$C$5+A48-1)</f>
-        <v>46325</v>
+        <f aca="false">IF(C48="","",WORKDAY($C$5-1,A48))</f>
+        <v>46342</v>
       </c>
       <c r="C48" s="20" t="n">
         <f aca="false">IF(C47="","",IF(OR(IF(ISNUMBER(G47),H47,F47)&gt;=$C$7,IF(ISNUMBER(G47),H47,F47)&lt;=0),"",IF(ISNUMBER(G47),H47,F47)))</f>
@@ -2531,8 +2537,8 @@
         <v>37</v>
       </c>
       <c r="B49" s="19" t="n">
-        <f aca="false">IF(C49="","",$C$5+A49-1)</f>
-        <v>46326</v>
+        <f aca="false">IF(C49="","",WORKDAY($C$5-1,A49))</f>
+        <v>46343</v>
       </c>
       <c r="C49" s="20" t="n">
         <f aca="false">IF(C48="","",IF(OR(IF(ISNUMBER(G48),H48,F48)&gt;=$C$7,IF(ISNUMBER(G48),H48,F48)&lt;=0),"",IF(ISNUMBER(G48),H48,F48)))</f>
@@ -2568,8 +2574,8 @@
         <v>38</v>
       </c>
       <c r="B50" s="19" t="n">
-        <f aca="false">IF(C50="","",$C$5+A50-1)</f>
-        <v>46327</v>
+        <f aca="false">IF(C50="","",WORKDAY($C$5-1,A50))</f>
+        <v>46344</v>
       </c>
       <c r="C50" s="20" t="n">
         <f aca="false">IF(C49="","",IF(OR(IF(ISNUMBER(G49),H49,F49)&gt;=$C$7,IF(ISNUMBER(G49),H49,F49)&lt;=0),"",IF(ISNUMBER(G49),H49,F49)))</f>
@@ -2605,8 +2611,8 @@
         <v>39</v>
       </c>
       <c r="B51" s="19" t="n">
-        <f aca="false">IF(C51="","",$C$5+A51-1)</f>
-        <v>46328</v>
+        <f aca="false">IF(C51="","",WORKDAY($C$5-1,A51))</f>
+        <v>46345</v>
       </c>
       <c r="C51" s="20" t="n">
         <f aca="false">IF(C50="","",IF(OR(IF(ISNUMBER(G50),H50,F50)&gt;=$C$7,IF(ISNUMBER(G50),H50,F50)&lt;=0),"",IF(ISNUMBER(G50),H50,F50)))</f>
@@ -2642,8 +2648,8 @@
         <v>40</v>
       </c>
       <c r="B52" s="19" t="n">
-        <f aca="false">IF(C52="","",$C$5+A52-1)</f>
-        <v>46329</v>
+        <f aca="false">IF(C52="","",WORKDAY($C$5-1,A52))</f>
+        <v>46346</v>
       </c>
       <c r="C52" s="20" t="n">
         <f aca="false">IF(C51="","",IF(OR(IF(ISNUMBER(G51),H51,F51)&gt;=$C$7,IF(ISNUMBER(G51),H51,F51)&lt;=0),"",IF(ISNUMBER(G51),H51,F51)))</f>
@@ -2679,8 +2685,8 @@
         <v>41</v>
       </c>
       <c r="B53" s="19" t="n">
-        <f aca="false">IF(C53="","",$C$5+A53-1)</f>
-        <v>46330</v>
+        <f aca="false">IF(C53="","",WORKDAY($C$5-1,A53))</f>
+        <v>46349</v>
       </c>
       <c r="C53" s="20" t="n">
         <f aca="false">IF(C52="","",IF(OR(IF(ISNUMBER(G52),H52,F52)&gt;=$C$7,IF(ISNUMBER(G52),H52,F52)&lt;=0),"",IF(ISNUMBER(G52),H52,F52)))</f>
@@ -2716,8 +2722,8 @@
         <v>42</v>
       </c>
       <c r="B54" s="19" t="n">
-        <f aca="false">IF(C54="","",$C$5+A54-1)</f>
-        <v>46331</v>
+        <f aca="false">IF(C54="","",WORKDAY($C$5-1,A54))</f>
+        <v>46350</v>
       </c>
       <c r="C54" s="20" t="n">
         <f aca="false">IF(C53="","",IF(OR(IF(ISNUMBER(G53),H53,F53)&gt;=$C$7,IF(ISNUMBER(G53),H53,F53)&lt;=0),"",IF(ISNUMBER(G53),H53,F53)))</f>
@@ -2753,8 +2759,8 @@
         <v>43</v>
       </c>
       <c r="B55" s="19" t="n">
-        <f aca="false">IF(C55="","",$C$5+A55-1)</f>
-        <v>46332</v>
+        <f aca="false">IF(C55="","",WORKDAY($C$5-1,A55))</f>
+        <v>46351</v>
       </c>
       <c r="C55" s="20" t="n">
         <f aca="false">IF(C54="","",IF(OR(IF(ISNUMBER(G54),H54,F54)&gt;=$C$7,IF(ISNUMBER(G54),H54,F54)&lt;=0),"",IF(ISNUMBER(G54),H54,F54)))</f>
@@ -2790,8 +2796,8 @@
         <v>44</v>
       </c>
       <c r="B56" s="19" t="n">
-        <f aca="false">IF(C56="","",$C$5+A56-1)</f>
-        <v>46333</v>
+        <f aca="false">IF(C56="","",WORKDAY($C$5-1,A56))</f>
+        <v>46352</v>
       </c>
       <c r="C56" s="20" t="n">
         <f aca="false">IF(C55="","",IF(OR(IF(ISNUMBER(G55),H55,F55)&gt;=$C$7,IF(ISNUMBER(G55),H55,F55)&lt;=0),"",IF(ISNUMBER(G55),H55,F55)))</f>
@@ -2827,8 +2833,8 @@
         <v>45</v>
       </c>
       <c r="B57" s="19" t="n">
-        <f aca="false">IF(C57="","",$C$5+A57-1)</f>
-        <v>46334</v>
+        <f aca="false">IF(C57="","",WORKDAY($C$5-1,A57))</f>
+        <v>46353</v>
       </c>
       <c r="C57" s="20" t="n">
         <f aca="false">IF(C56="","",IF(OR(IF(ISNUMBER(G56),H56,F56)&gt;=$C$7,IF(ISNUMBER(G56),H56,F56)&lt;=0),"",IF(ISNUMBER(G56),H56,F56)))</f>
@@ -2864,8 +2870,8 @@
         <v>46</v>
       </c>
       <c r="B58" s="19" t="n">
-        <f aca="false">IF(C58="","",$C$5+A58-1)</f>
-        <v>46335</v>
+        <f aca="false">IF(C58="","",WORKDAY($C$5-1,A58))</f>
+        <v>46356</v>
       </c>
       <c r="C58" s="20" t="n">
         <f aca="false">IF(C57="","",IF(OR(IF(ISNUMBER(G57),H57,F57)&gt;=$C$7,IF(ISNUMBER(G57),H57,F57)&lt;=0),"",IF(ISNUMBER(G57),H57,F57)))</f>
@@ -2901,8 +2907,8 @@
         <v>47</v>
       </c>
       <c r="B59" s="19" t="n">
-        <f aca="false">IF(C59="","",$C$5+A59-1)</f>
-        <v>46336</v>
+        <f aca="false">IF(C59="","",WORKDAY($C$5-1,A59))</f>
+        <v>46357</v>
       </c>
       <c r="C59" s="20" t="n">
         <f aca="false">IF(C58="","",IF(OR(IF(ISNUMBER(G58),H58,F58)&gt;=$C$7,IF(ISNUMBER(G58),H58,F58)&lt;=0),"",IF(ISNUMBER(G58),H58,F58)))</f>
@@ -2938,8 +2944,8 @@
         <v>48</v>
       </c>
       <c r="B60" s="19" t="n">
-        <f aca="false">IF(C60="","",$C$5+A60-1)</f>
-        <v>46337</v>
+        <f aca="false">IF(C60="","",WORKDAY($C$5-1,A60))</f>
+        <v>46358</v>
       </c>
       <c r="C60" s="20" t="n">
         <f aca="false">IF(C59="","",IF(OR(IF(ISNUMBER(G59),H59,F59)&gt;=$C$7,IF(ISNUMBER(G59),H59,F59)&lt;=0),"",IF(ISNUMBER(G59),H59,F59)))</f>
@@ -2975,8 +2981,8 @@
         <v>49</v>
       </c>
       <c r="B61" s="19" t="n">
-        <f aca="false">IF(C61="","",$C$5+A61-1)</f>
-        <v>46338</v>
+        <f aca="false">IF(C61="","",WORKDAY($C$5-1,A61))</f>
+        <v>46359</v>
       </c>
       <c r="C61" s="20" t="n">
         <f aca="false">IF(C60="","",IF(OR(IF(ISNUMBER(G60),H60,F60)&gt;=$C$7,IF(ISNUMBER(G60),H60,F60)&lt;=0),"",IF(ISNUMBER(G60),H60,F60)))</f>
@@ -3012,8 +3018,8 @@
         <v>50</v>
       </c>
       <c r="B62" s="19" t="n">
-        <f aca="false">IF(C62="","",$C$5+A62-1)</f>
-        <v>46339</v>
+        <f aca="false">IF(C62="","",WORKDAY($C$5-1,A62))</f>
+        <v>46360</v>
       </c>
       <c r="C62" s="20" t="n">
         <f aca="false">IF(C61="","",IF(OR(IF(ISNUMBER(G61),H61,F61)&gt;=$C$7,IF(ISNUMBER(G61),H61,F61)&lt;=0),"",IF(ISNUMBER(G61),H61,F61)))</f>
@@ -3049,8 +3055,8 @@
         <v>51</v>
       </c>
       <c r="B63" s="19" t="n">
-        <f aca="false">IF(C63="","",$C$5+A63-1)</f>
-        <v>46340</v>
+        <f aca="false">IF(C63="","",WORKDAY($C$5-1,A63))</f>
+        <v>46363</v>
       </c>
       <c r="C63" s="20" t="n">
         <f aca="false">IF(C62="","",IF(OR(IF(ISNUMBER(G62),H62,F62)&gt;=$C$7,IF(ISNUMBER(G62),H62,F62)&lt;=0),"",IF(ISNUMBER(G62),H62,F62)))</f>
@@ -3086,8 +3092,8 @@
         <v>52</v>
       </c>
       <c r="B64" s="19" t="n">
-        <f aca="false">IF(C64="","",$C$5+A64-1)</f>
-        <v>46341</v>
+        <f aca="false">IF(C64="","",WORKDAY($C$5-1,A64))</f>
+        <v>46364</v>
       </c>
       <c r="C64" s="20" t="n">
         <f aca="false">IF(C63="","",IF(OR(IF(ISNUMBER(G63),H63,F63)&gt;=$C$7,IF(ISNUMBER(G63),H63,F63)&lt;=0),"",IF(ISNUMBER(G63),H63,F63)))</f>
@@ -3123,8 +3129,8 @@
         <v>53</v>
       </c>
       <c r="B65" s="19" t="n">
-        <f aca="false">IF(C65="","",$C$5+A65-1)</f>
-        <v>46342</v>
+        <f aca="false">IF(C65="","",WORKDAY($C$5-1,A65))</f>
+        <v>46365</v>
       </c>
       <c r="C65" s="20" t="n">
         <f aca="false">IF(C64="","",IF(OR(IF(ISNUMBER(G64),H64,F64)&gt;=$C$7,IF(ISNUMBER(G64),H64,F64)&lt;=0),"",IF(ISNUMBER(G64),H64,F64)))</f>
@@ -3160,8 +3166,8 @@
         <v>54</v>
       </c>
       <c r="B66" s="19" t="n">
-        <f aca="false">IF(C66="","",$C$5+A66-1)</f>
-        <v>46343</v>
+        <f aca="false">IF(C66="","",WORKDAY($C$5-1,A66))</f>
+        <v>46366</v>
       </c>
       <c r="C66" s="20" t="n">
         <f aca="false">IF(C65="","",IF(OR(IF(ISNUMBER(G65),H65,F65)&gt;=$C$7,IF(ISNUMBER(G65),H65,F65)&lt;=0),"",IF(ISNUMBER(G65),H65,F65)))</f>
@@ -3197,8 +3203,8 @@
         <v>55</v>
       </c>
       <c r="B67" s="19" t="n">
-        <f aca="false">IF(C67="","",$C$5+A67-1)</f>
-        <v>46344</v>
+        <f aca="false">IF(C67="","",WORKDAY($C$5-1,A67))</f>
+        <v>46367</v>
       </c>
       <c r="C67" s="20" t="n">
         <f aca="false">IF(C66="","",IF(OR(IF(ISNUMBER(G66),H66,F66)&gt;=$C$7,IF(ISNUMBER(G66),H66,F66)&lt;=0),"",IF(ISNUMBER(G66),H66,F66)))</f>
@@ -3234,8 +3240,8 @@
         <v>56</v>
       </c>
       <c r="B68" s="19" t="n">
-        <f aca="false">IF(C68="","",$C$5+A68-1)</f>
-        <v>46345</v>
+        <f aca="false">IF(C68="","",WORKDAY($C$5-1,A68))</f>
+        <v>46370</v>
       </c>
       <c r="C68" s="20" t="n">
         <f aca="false">IF(C67="","",IF(OR(IF(ISNUMBER(G67),H67,F67)&gt;=$C$7,IF(ISNUMBER(G67),H67,F67)&lt;=0),"",IF(ISNUMBER(G67),H67,F67)))</f>
@@ -3271,8 +3277,8 @@
         <v>57</v>
       </c>
       <c r="B69" s="19" t="n">
-        <f aca="false">IF(C69="","",$C$5+A69-1)</f>
-        <v>46346</v>
+        <f aca="false">IF(C69="","",WORKDAY($C$5-1,A69))</f>
+        <v>46371</v>
       </c>
       <c r="C69" s="20" t="n">
         <f aca="false">IF(C68="","",IF(OR(IF(ISNUMBER(G68),H68,F68)&gt;=$C$7,IF(ISNUMBER(G68),H68,F68)&lt;=0),"",IF(ISNUMBER(G68),H68,F68)))</f>
@@ -3308,8 +3314,8 @@
         <v>58</v>
       </c>
       <c r="B70" s="19" t="n">
-        <f aca="false">IF(C70="","",$C$5+A70-1)</f>
-        <v>46347</v>
+        <f aca="false">IF(C70="","",WORKDAY($C$5-1,A70))</f>
+        <v>46372</v>
       </c>
       <c r="C70" s="20" t="n">
         <f aca="false">IF(C69="","",IF(OR(IF(ISNUMBER(G69),H69,F69)&gt;=$C$7,IF(ISNUMBER(G69),H69,F69)&lt;=0),"",IF(ISNUMBER(G69),H69,F69)))</f>
@@ -3345,8 +3351,8 @@
         <v>59</v>
       </c>
       <c r="B71" s="19" t="n">
-        <f aca="false">IF(C71="","",$C$5+A71-1)</f>
-        <v>46348</v>
+        <f aca="false">IF(C71="","",WORKDAY($C$5-1,A71))</f>
+        <v>46373</v>
       </c>
       <c r="C71" s="20" t="n">
         <f aca="false">IF(C70="","",IF(OR(IF(ISNUMBER(G70),H70,F70)&gt;=$C$7,IF(ISNUMBER(G70),H70,F70)&lt;=0),"",IF(ISNUMBER(G70),H70,F70)))</f>
@@ -3382,8 +3388,8 @@
         <v>60</v>
       </c>
       <c r="B72" s="19" t="n">
-        <f aca="false">IF(C72="","",$C$5+A72-1)</f>
-        <v>46349</v>
+        <f aca="false">IF(C72="","",WORKDAY($C$5-1,A72))</f>
+        <v>46374</v>
       </c>
       <c r="C72" s="20" t="n">
         <f aca="false">IF(C71="","",IF(OR(IF(ISNUMBER(G71),H71,F71)&gt;=$C$7,IF(ISNUMBER(G71),H71,F71)&lt;=0),"",IF(ISNUMBER(G71),H71,F71)))</f>
@@ -3419,8 +3425,8 @@
         <v>61</v>
       </c>
       <c r="B73" s="19" t="n">
-        <f aca="false">IF(C73="","",$C$5+A73-1)</f>
-        <v>46350</v>
+        <f aca="false">IF(C73="","",WORKDAY($C$5-1,A73))</f>
+        <v>46377</v>
       </c>
       <c r="C73" s="20" t="n">
         <f aca="false">IF(C72="","",IF(OR(IF(ISNUMBER(G72),H72,F72)&gt;=$C$7,IF(ISNUMBER(G72),H72,F72)&lt;=0),"",IF(ISNUMBER(G72),H72,F72)))</f>
@@ -3456,8 +3462,8 @@
         <v>62</v>
       </c>
       <c r="B74" s="19" t="n">
-        <f aca="false">IF(C74="","",$C$5+A74-1)</f>
-        <v>46351</v>
+        <f aca="false">IF(C74="","",WORKDAY($C$5-1,A74))</f>
+        <v>46378</v>
       </c>
       <c r="C74" s="20" t="n">
         <f aca="false">IF(C73="","",IF(OR(IF(ISNUMBER(G73),H73,F73)&gt;=$C$7,IF(ISNUMBER(G73),H73,F73)&lt;=0),"",IF(ISNUMBER(G73),H73,F73)))</f>
@@ -3493,8 +3499,8 @@
         <v>63</v>
       </c>
       <c r="B75" s="19" t="n">
-        <f aca="false">IF(C75="","",$C$5+A75-1)</f>
-        <v>46352</v>
+        <f aca="false">IF(C75="","",WORKDAY($C$5-1,A75))</f>
+        <v>46379</v>
       </c>
       <c r="C75" s="20" t="n">
         <f aca="false">IF(C74="","",IF(OR(IF(ISNUMBER(G74),H74,F74)&gt;=$C$7,IF(ISNUMBER(G74),H74,F74)&lt;=0),"",IF(ISNUMBER(G74),H74,F74)))</f>
@@ -3530,8 +3536,8 @@
         <v>64</v>
       </c>
       <c r="B76" s="19" t="n">
-        <f aca="false">IF(C76="","",$C$5+A76-1)</f>
-        <v>46353</v>
+        <f aca="false">IF(C76="","",WORKDAY($C$5-1,A76))</f>
+        <v>46380</v>
       </c>
       <c r="C76" s="20" t="n">
         <f aca="false">IF(C75="","",IF(OR(IF(ISNUMBER(G75),H75,F75)&gt;=$C$7,IF(ISNUMBER(G75),H75,F75)&lt;=0),"",IF(ISNUMBER(G75),H75,F75)))</f>
@@ -3567,8 +3573,8 @@
         <v>65</v>
       </c>
       <c r="B77" s="19" t="n">
-        <f aca="false">IF(C77="","",$C$5+A77-1)</f>
-        <v>46354</v>
+        <f aca="false">IF(C77="","",WORKDAY($C$5-1,A77))</f>
+        <v>46381</v>
       </c>
       <c r="C77" s="20" t="n">
         <f aca="false">IF(C76="","",IF(OR(IF(ISNUMBER(G76),H76,F76)&gt;=$C$7,IF(ISNUMBER(G76),H76,F76)&lt;=0),"",IF(ISNUMBER(G76),H76,F76)))</f>
@@ -3604,8 +3610,8 @@
         <v>66</v>
       </c>
       <c r="B78" s="19" t="n">
-        <f aca="false">IF(C78="","",$C$5+A78-1)</f>
-        <v>46355</v>
+        <f aca="false">IF(C78="","",WORKDAY($C$5-1,A78))</f>
+        <v>46384</v>
       </c>
       <c r="C78" s="20" t="n">
         <f aca="false">IF(C77="","",IF(OR(IF(ISNUMBER(G77),H77,F77)&gt;=$C$7,IF(ISNUMBER(G77),H77,F77)&lt;=0),"",IF(ISNUMBER(G77),H77,F77)))</f>
@@ -3641,8 +3647,8 @@
         <v>67</v>
       </c>
       <c r="B79" s="19" t="n">
-        <f aca="false">IF(C79="","",$C$5+A79-1)</f>
-        <v>46356</v>
+        <f aca="false">IF(C79="","",WORKDAY($C$5-1,A79))</f>
+        <v>46385</v>
       </c>
       <c r="C79" s="20" t="n">
         <f aca="false">IF(C78="","",IF(OR(IF(ISNUMBER(G78),H78,F78)&gt;=$C$7,IF(ISNUMBER(G78),H78,F78)&lt;=0),"",IF(ISNUMBER(G78),H78,F78)))</f>
@@ -3678,8 +3684,8 @@
         <v>68</v>
       </c>
       <c r="B80" s="19" t="n">
-        <f aca="false">IF(C80="","",$C$5+A80-1)</f>
-        <v>46357</v>
+        <f aca="false">IF(C80="","",WORKDAY($C$5-1,A80))</f>
+        <v>46386</v>
       </c>
       <c r="C80" s="20" t="n">
         <f aca="false">IF(C79="","",IF(OR(IF(ISNUMBER(G79),H79,F79)&gt;=$C$7,IF(ISNUMBER(G79),H79,F79)&lt;=0),"",IF(ISNUMBER(G79),H79,F79)))</f>
@@ -3715,8 +3721,8 @@
         <v>69</v>
       </c>
       <c r="B81" s="19" t="n">
-        <f aca="false">IF(C81="","",$C$5+A81-1)</f>
-        <v>46358</v>
+        <f aca="false">IF(C81="","",WORKDAY($C$5-1,A81))</f>
+        <v>46387</v>
       </c>
       <c r="C81" s="20" t="n">
         <f aca="false">IF(C80="","",IF(OR(IF(ISNUMBER(G80),H80,F80)&gt;=$C$7,IF(ISNUMBER(G80),H80,F80)&lt;=0),"",IF(ISNUMBER(G80),H80,F80)))</f>
@@ -3752,8 +3758,8 @@
         <v>70</v>
       </c>
       <c r="B82" s="19" t="n">
-        <f aca="false">IF(C82="","",$C$5+A82-1)</f>
-        <v>46359</v>
+        <f aca="false">IF(C82="","",WORKDAY($C$5-1,A82))</f>
+        <v>46388</v>
       </c>
       <c r="C82" s="20" t="n">
         <f aca="false">IF(C81="","",IF(OR(IF(ISNUMBER(G81),H81,F81)&gt;=$C$7,IF(ISNUMBER(G81),H81,F81)&lt;=0),"",IF(ISNUMBER(G81),H81,F81)))</f>
@@ -3789,8 +3795,8 @@
         <v>71</v>
       </c>
       <c r="B83" s="19" t="n">
-        <f aca="false">IF(C83="","",$C$5+A83-1)</f>
-        <v>46360</v>
+        <f aca="false">IF(C83="","",WORKDAY($C$5-1,A83))</f>
+        <v>46391</v>
       </c>
       <c r="C83" s="20" t="n">
         <f aca="false">IF(C82="","",IF(OR(IF(ISNUMBER(G82),H82,F82)&gt;=$C$7,IF(ISNUMBER(G82),H82,F82)&lt;=0),"",IF(ISNUMBER(G82),H82,F82)))</f>
@@ -3826,8 +3832,8 @@
         <v>72</v>
       </c>
       <c r="B84" s="19" t="n">
-        <f aca="false">IF(C84="","",$C$5+A84-1)</f>
-        <v>46361</v>
+        <f aca="false">IF(C84="","",WORKDAY($C$5-1,A84))</f>
+        <v>46392</v>
       </c>
       <c r="C84" s="20" t="n">
         <f aca="false">IF(C83="","",IF(OR(IF(ISNUMBER(G83),H83,F83)&gt;=$C$7,IF(ISNUMBER(G83),H83,F83)&lt;=0),"",IF(ISNUMBER(G83),H83,F83)))</f>
@@ -3863,8 +3869,8 @@
         <v>73</v>
       </c>
       <c r="B85" s="19" t="n">
-        <f aca="false">IF(C85="","",$C$5+A85-1)</f>
-        <v>46362</v>
+        <f aca="false">IF(C85="","",WORKDAY($C$5-1,A85))</f>
+        <v>46393</v>
       </c>
       <c r="C85" s="20" t="n">
         <f aca="false">IF(C84="","",IF(OR(IF(ISNUMBER(G84),H84,F84)&gt;=$C$7,IF(ISNUMBER(G84),H84,F84)&lt;=0),"",IF(ISNUMBER(G84),H84,F84)))</f>
@@ -3900,8 +3906,8 @@
         <v>74</v>
       </c>
       <c r="B86" s="19" t="n">
-        <f aca="false">IF(C86="","",$C$5+A86-1)</f>
-        <v>46363</v>
+        <f aca="false">IF(C86="","",WORKDAY($C$5-1,A86))</f>
+        <v>46394</v>
       </c>
       <c r="C86" s="20" t="n">
         <f aca="false">IF(C85="","",IF(OR(IF(ISNUMBER(G85),H85,F85)&gt;=$C$7,IF(ISNUMBER(G85),H85,F85)&lt;=0),"",IF(ISNUMBER(G85),H85,F85)))</f>
@@ -3937,8 +3943,8 @@
         <v>75</v>
       </c>
       <c r="B87" s="19" t="n">
-        <f aca="false">IF(C87="","",$C$5+A87-1)</f>
-        <v>46364</v>
+        <f aca="false">IF(C87="","",WORKDAY($C$5-1,A87))</f>
+        <v>46395</v>
       </c>
       <c r="C87" s="20" t="n">
         <f aca="false">IF(C86="","",IF(OR(IF(ISNUMBER(G86),H86,F86)&gt;=$C$7,IF(ISNUMBER(G86),H86,F86)&lt;=0),"",IF(ISNUMBER(G86),H86,F86)))</f>
@@ -3974,8 +3980,8 @@
         <v>76</v>
       </c>
       <c r="B88" s="19" t="n">
-        <f aca="false">IF(C88="","",$C$5+A88-1)</f>
-        <v>46365</v>
+        <f aca="false">IF(C88="","",WORKDAY($C$5-1,A88))</f>
+        <v>46398</v>
       </c>
       <c r="C88" s="20" t="n">
         <f aca="false">IF(C87="","",IF(OR(IF(ISNUMBER(G87),H87,F87)&gt;=$C$7,IF(ISNUMBER(G87),H87,F87)&lt;=0),"",IF(ISNUMBER(G87),H87,F87)))</f>
@@ -4011,8 +4017,8 @@
         <v>77</v>
       </c>
       <c r="B89" s="19" t="n">
-        <f aca="false">IF(C89="","",$C$5+A89-1)</f>
-        <v>46366</v>
+        <f aca="false">IF(C89="","",WORKDAY($C$5-1,A89))</f>
+        <v>46399</v>
       </c>
       <c r="C89" s="20" t="n">
         <f aca="false">IF(C88="","",IF(OR(IF(ISNUMBER(G88),H88,F88)&gt;=$C$7,IF(ISNUMBER(G88),H88,F88)&lt;=0),"",IF(ISNUMBER(G88),H88,F88)))</f>
@@ -4048,8 +4054,8 @@
         <v>78</v>
       </c>
       <c r="B90" s="19" t="n">
-        <f aca="false">IF(C90="","",$C$5+A90-1)</f>
-        <v>46367</v>
+        <f aca="false">IF(C90="","",WORKDAY($C$5-1,A90))</f>
+        <v>46400</v>
       </c>
       <c r="C90" s="20" t="n">
         <f aca="false">IF(C89="","",IF(OR(IF(ISNUMBER(G89),H89,F89)&gt;=$C$7,IF(ISNUMBER(G89),H89,F89)&lt;=0),"",IF(ISNUMBER(G89),H89,F89)))</f>
@@ -4085,8 +4091,8 @@
         <v>79</v>
       </c>
       <c r="B91" s="19" t="n">
-        <f aca="false">IF(C91="","",$C$5+A91-1)</f>
-        <v>46368</v>
+        <f aca="false">IF(C91="","",WORKDAY($C$5-1,A91))</f>
+        <v>46401</v>
       </c>
       <c r="C91" s="20" t="n">
         <f aca="false">IF(C90="","",IF(OR(IF(ISNUMBER(G90),H90,F90)&gt;=$C$7,IF(ISNUMBER(G90),H90,F90)&lt;=0),"",IF(ISNUMBER(G90),H90,F90)))</f>
@@ -4122,8 +4128,8 @@
         <v>80</v>
       </c>
       <c r="B92" s="19" t="n">
-        <f aca="false">IF(C92="","",$C$5+A92-1)</f>
-        <v>46369</v>
+        <f aca="false">IF(C92="","",WORKDAY($C$5-1,A92))</f>
+        <v>46402</v>
       </c>
       <c r="C92" s="20" t="n">
         <f aca="false">IF(C91="","",IF(OR(IF(ISNUMBER(G91),H91,F91)&gt;=$C$7,IF(ISNUMBER(G91),H91,F91)&lt;=0),"",IF(ISNUMBER(G91),H91,F91)))</f>
@@ -4159,8 +4165,8 @@
         <v>81</v>
       </c>
       <c r="B93" s="19" t="n">
-        <f aca="false">IF(C93="","",$C$5+A93-1)</f>
-        <v>46370</v>
+        <f aca="false">IF(C93="","",WORKDAY($C$5-1,A93))</f>
+        <v>46405</v>
       </c>
       <c r="C93" s="20" t="n">
         <f aca="false">IF(C92="","",IF(OR(IF(ISNUMBER(G92),H92,F92)&gt;=$C$7,IF(ISNUMBER(G92),H92,F92)&lt;=0),"",IF(ISNUMBER(G92),H92,F92)))</f>
@@ -4196,8 +4202,8 @@
         <v>82</v>
       </c>
       <c r="B94" s="19" t="n">
-        <f aca="false">IF(C94="","",$C$5+A94-1)</f>
-        <v>46371</v>
+        <f aca="false">IF(C94="","",WORKDAY($C$5-1,A94))</f>
+        <v>46406</v>
       </c>
       <c r="C94" s="20" t="n">
         <f aca="false">IF(C93="","",IF(OR(IF(ISNUMBER(G93),H93,F93)&gt;=$C$7,IF(ISNUMBER(G93),H93,F93)&lt;=0),"",IF(ISNUMBER(G93),H93,F93)))</f>
@@ -4233,8 +4239,8 @@
         <v>83</v>
       </c>
       <c r="B95" s="19" t="n">
-        <f aca="false">IF(C95="","",$C$5+A95-1)</f>
-        <v>46372</v>
+        <f aca="false">IF(C95="","",WORKDAY($C$5-1,A95))</f>
+        <v>46407</v>
       </c>
       <c r="C95" s="20" t="n">
         <f aca="false">IF(C94="","",IF(OR(IF(ISNUMBER(G94),H94,F94)&gt;=$C$7,IF(ISNUMBER(G94),H94,F94)&lt;=0),"",IF(ISNUMBER(G94),H94,F94)))</f>
@@ -4270,8 +4276,8 @@
         <v>84</v>
       </c>
       <c r="B96" s="19" t="n">
-        <f aca="false">IF(C96="","",$C$5+A96-1)</f>
-        <v>46373</v>
+        <f aca="false">IF(C96="","",WORKDAY($C$5-1,A96))</f>
+        <v>46408</v>
       </c>
       <c r="C96" s="20" t="n">
         <f aca="false">IF(C95="","",IF(OR(IF(ISNUMBER(G95),H95,F95)&gt;=$C$7,IF(ISNUMBER(G95),H95,F95)&lt;=0),"",IF(ISNUMBER(G95),H95,F95)))</f>
@@ -4307,8 +4313,8 @@
         <v>85</v>
       </c>
       <c r="B97" s="19" t="n">
-        <f aca="false">IF(C97="","",$C$5+A97-1)</f>
-        <v>46374</v>
+        <f aca="false">IF(C97="","",WORKDAY($C$5-1,A97))</f>
+        <v>46409</v>
       </c>
       <c r="C97" s="20" t="n">
         <f aca="false">IF(C96="","",IF(OR(IF(ISNUMBER(G96),H96,F96)&gt;=$C$7,IF(ISNUMBER(G96),H96,F96)&lt;=0),"",IF(ISNUMBER(G96),H96,F96)))</f>
@@ -4344,8 +4350,8 @@
         <v>86</v>
       </c>
       <c r="B98" s="19" t="n">
-        <f aca="false">IF(C98="","",$C$5+A98-1)</f>
-        <v>46375</v>
+        <f aca="false">IF(C98="","",WORKDAY($C$5-1,A98))</f>
+        <v>46412</v>
       </c>
       <c r="C98" s="20" t="n">
         <f aca="false">IF(C97="","",IF(OR(IF(ISNUMBER(G97),H97,F97)&gt;=$C$7,IF(ISNUMBER(G97),H97,F97)&lt;=0),"",IF(ISNUMBER(G97),H97,F97)))</f>
@@ -4381,8 +4387,8 @@
         <v>87</v>
       </c>
       <c r="B99" s="19" t="n">
-        <f aca="false">IF(C99="","",$C$5+A99-1)</f>
-        <v>46376</v>
+        <f aca="false">IF(C99="","",WORKDAY($C$5-1,A99))</f>
+        <v>46413</v>
       </c>
       <c r="C99" s="20" t="n">
         <f aca="false">IF(C98="","",IF(OR(IF(ISNUMBER(G98),H98,F98)&gt;=$C$7,IF(ISNUMBER(G98),H98,F98)&lt;=0),"",IF(ISNUMBER(G98),H98,F98)))</f>
@@ -4418,8 +4424,8 @@
         <v>88</v>
       </c>
       <c r="B100" s="19" t="n">
-        <f aca="false">IF(C100="","",$C$5+A100-1)</f>
-        <v>46377</v>
+        <f aca="false">IF(C100="","",WORKDAY($C$5-1,A100))</f>
+        <v>46414</v>
       </c>
       <c r="C100" s="20" t="n">
         <f aca="false">IF(C99="","",IF(OR(IF(ISNUMBER(G99),H99,F99)&gt;=$C$7,IF(ISNUMBER(G99),H99,F99)&lt;=0),"",IF(ISNUMBER(G99),H99,F99)))</f>
@@ -4455,8 +4461,8 @@
         <v>89</v>
       </c>
       <c r="B101" s="19" t="n">
-        <f aca="false">IF(C101="","",$C$5+A101-1)</f>
-        <v>46378</v>
+        <f aca="false">IF(C101="","",WORKDAY($C$5-1,A101))</f>
+        <v>46415</v>
       </c>
       <c r="C101" s="20" t="n">
         <f aca="false">IF(C100="","",IF(OR(IF(ISNUMBER(G100),H100,F100)&gt;=$C$7,IF(ISNUMBER(G100),H100,F100)&lt;=0),"",IF(ISNUMBER(G100),H100,F100)))</f>
@@ -4492,8 +4498,8 @@
         <v>90</v>
       </c>
       <c r="B102" s="19" t="n">
-        <f aca="false">IF(C102="","",$C$5+A102-1)</f>
-        <v>46379</v>
+        <f aca="false">IF(C102="","",WORKDAY($C$5-1,A102))</f>
+        <v>46416</v>
       </c>
       <c r="C102" s="20" t="n">
         <f aca="false">IF(C101="","",IF(OR(IF(ISNUMBER(G101),H101,F101)&gt;=$C$7,IF(ISNUMBER(G101),H101,F101)&lt;=0),"",IF(ISNUMBER(G101),H101,F101)))</f>
@@ -4529,8 +4535,8 @@
         <v>91</v>
       </c>
       <c r="B103" s="19" t="n">
-        <f aca="false">IF(C103="","",$C$5+A103-1)</f>
-        <v>46380</v>
+        <f aca="false">IF(C103="","",WORKDAY($C$5-1,A103))</f>
+        <v>46419</v>
       </c>
       <c r="C103" s="20" t="n">
         <f aca="false">IF(C102="","",IF(OR(IF(ISNUMBER(G102),H102,F102)&gt;=$C$7,IF(ISNUMBER(G102),H102,F102)&lt;=0),"",IF(ISNUMBER(G102),H102,F102)))</f>
@@ -4566,8 +4572,8 @@
         <v>92</v>
       </c>
       <c r="B104" s="19" t="n">
-        <f aca="false">IF(C104="","",$C$5+A104-1)</f>
-        <v>46381</v>
+        <f aca="false">IF(C104="","",WORKDAY($C$5-1,A104))</f>
+        <v>46420</v>
       </c>
       <c r="C104" s="20" t="n">
         <f aca="false">IF(C103="","",IF(OR(IF(ISNUMBER(G103),H103,F103)&gt;=$C$7,IF(ISNUMBER(G103),H103,F103)&lt;=0),"",IF(ISNUMBER(G103),H103,F103)))</f>
@@ -4603,8 +4609,8 @@
         <v>93</v>
       </c>
       <c r="B105" s="19" t="n">
-        <f aca="false">IF(C105="","",$C$5+A105-1)</f>
-        <v>46382</v>
+        <f aca="false">IF(C105="","",WORKDAY($C$5-1,A105))</f>
+        <v>46421</v>
       </c>
       <c r="C105" s="20" t="n">
         <f aca="false">IF(C104="","",IF(OR(IF(ISNUMBER(G104),H104,F104)&gt;=$C$7,IF(ISNUMBER(G104),H104,F104)&lt;=0),"",IF(ISNUMBER(G104),H104,F104)))</f>
@@ -4640,8 +4646,8 @@
         <v>94</v>
       </c>
       <c r="B106" s="19" t="n">
-        <f aca="false">IF(C106="","",$C$5+A106-1)</f>
-        <v>46383</v>
+        <f aca="false">IF(C106="","",WORKDAY($C$5-1,A106))</f>
+        <v>46422</v>
       </c>
       <c r="C106" s="20" t="n">
         <f aca="false">IF(C105="","",IF(OR(IF(ISNUMBER(G105),H105,F105)&gt;=$C$7,IF(ISNUMBER(G105),H105,F105)&lt;=0),"",IF(ISNUMBER(G105),H105,F105)))</f>
@@ -4677,8 +4683,8 @@
         <v>95</v>
       </c>
       <c r="B107" s="19" t="n">
-        <f aca="false">IF(C107="","",$C$5+A107-1)</f>
-        <v>46384</v>
+        <f aca="false">IF(C107="","",WORKDAY($C$5-1,A107))</f>
+        <v>46423</v>
       </c>
       <c r="C107" s="20" t="n">
         <f aca="false">IF(C106="","",IF(OR(IF(ISNUMBER(G106),H106,F106)&gt;=$C$7,IF(ISNUMBER(G106),H106,F106)&lt;=0),"",IF(ISNUMBER(G106),H106,F106)))</f>
@@ -4714,8 +4720,8 @@
         <v>96</v>
       </c>
       <c r="B108" s="19" t="n">
-        <f aca="false">IF(C108="","",$C$5+A108-1)</f>
-        <v>46385</v>
+        <f aca="false">IF(C108="","",WORKDAY($C$5-1,A108))</f>
+        <v>46426</v>
       </c>
       <c r="C108" s="20" t="n">
         <f aca="false">IF(C107="","",IF(OR(IF(ISNUMBER(G107),H107,F107)&gt;=$C$7,IF(ISNUMBER(G107),H107,F107)&lt;=0),"",IF(ISNUMBER(G107),H107,F107)))</f>
@@ -4751,8 +4757,8 @@
         <v>97</v>
       </c>
       <c r="B109" s="19" t="n">
-        <f aca="false">IF(C109="","",$C$5+A109-1)</f>
-        <v>46386</v>
+        <f aca="false">IF(C109="","",WORKDAY($C$5-1,A109))</f>
+        <v>46427</v>
       </c>
       <c r="C109" s="20" t="n">
         <f aca="false">IF(C108="","",IF(OR(IF(ISNUMBER(G108),H108,F108)&gt;=$C$7,IF(ISNUMBER(G108),H108,F108)&lt;=0),"",IF(ISNUMBER(G108),H108,F108)))</f>
@@ -4788,8 +4794,8 @@
         <v>98</v>
       </c>
       <c r="B110" s="19" t="n">
-        <f aca="false">IF(C110="","",$C$5+A110-1)</f>
-        <v>46387</v>
+        <f aca="false">IF(C110="","",WORKDAY($C$5-1,A110))</f>
+        <v>46428</v>
       </c>
       <c r="C110" s="20" t="n">
         <f aca="false">IF(C109="","",IF(OR(IF(ISNUMBER(G109),H109,F109)&gt;=$C$7,IF(ISNUMBER(G109),H109,F109)&lt;=0),"",IF(ISNUMBER(G109),H109,F109)))</f>
@@ -4825,8 +4831,8 @@
         <v>99</v>
       </c>
       <c r="B111" s="19" t="n">
-        <f aca="false">IF(C111="","",$C$5+A111-1)</f>
-        <v>46388</v>
+        <f aca="false">IF(C111="","",WORKDAY($C$5-1,A111))</f>
+        <v>46429</v>
       </c>
       <c r="C111" s="20" t="n">
         <f aca="false">IF(C110="","",IF(OR(IF(ISNUMBER(G110),H110,F110)&gt;=$C$7,IF(ISNUMBER(G110),H110,F110)&lt;=0),"",IF(ISNUMBER(G110),H110,F110)))</f>
@@ -4862,8 +4868,8 @@
         <v>100</v>
       </c>
       <c r="B112" s="19" t="n">
-        <f aca="false">IF(C112="","",$C$5+A112-1)</f>
-        <v>46389</v>
+        <f aca="false">IF(C112="","",WORKDAY($C$5-1,A112))</f>
+        <v>46430</v>
       </c>
       <c r="C112" s="20" t="n">
         <f aca="false">IF(C111="","",IF(OR(IF(ISNUMBER(G111),H111,F111)&gt;=$C$7,IF(ISNUMBER(G111),H111,F111)&lt;=0),"",IF(ISNUMBER(G111),H111,F111)))</f>
@@ -4899,8 +4905,8 @@
         <v>101</v>
       </c>
       <c r="B113" s="19" t="n">
-        <f aca="false">IF(C113="","",$C$5+A113-1)</f>
-        <v>46390</v>
+        <f aca="false">IF(C113="","",WORKDAY($C$5-1,A113))</f>
+        <v>46433</v>
       </c>
       <c r="C113" s="20" t="n">
         <f aca="false">IF(C112="","",IF(OR(IF(ISNUMBER(G112),H112,F112)&gt;=$C$7,IF(ISNUMBER(G112),H112,F112)&lt;=0),"",IF(ISNUMBER(G112),H112,F112)))</f>
@@ -4936,8 +4942,8 @@
         <v>102</v>
       </c>
       <c r="B114" s="19" t="n">
-        <f aca="false">IF(C114="","",$C$5+A114-1)</f>
-        <v>46391</v>
+        <f aca="false">IF(C114="","",WORKDAY($C$5-1,A114))</f>
+        <v>46434</v>
       </c>
       <c r="C114" s="20" t="n">
         <f aca="false">IF(C113="","",IF(OR(IF(ISNUMBER(G113),H113,F113)&gt;=$C$7,IF(ISNUMBER(G113),H113,F113)&lt;=0),"",IF(ISNUMBER(G113),H113,F113)))</f>
@@ -4973,8 +4979,8 @@
         <v>103</v>
       </c>
       <c r="B115" s="19" t="n">
-        <f aca="false">IF(C115="","",$C$5+A115-1)</f>
-        <v>46392</v>
+        <f aca="false">IF(C115="","",WORKDAY($C$5-1,A115))</f>
+        <v>46435</v>
       </c>
       <c r="C115" s="20" t="n">
         <f aca="false">IF(C114="","",IF(OR(IF(ISNUMBER(G114),H114,F114)&gt;=$C$7,IF(ISNUMBER(G114),H114,F114)&lt;=0),"",IF(ISNUMBER(G114),H114,F114)))</f>
@@ -5010,8 +5016,8 @@
         <v>104</v>
       </c>
       <c r="B116" s="19" t="n">
-        <f aca="false">IF(C116="","",$C$5+A116-1)</f>
-        <v>46393</v>
+        <f aca="false">IF(C116="","",WORKDAY($C$5-1,A116))</f>
+        <v>46436</v>
       </c>
       <c r="C116" s="20" t="n">
         <f aca="false">IF(C115="","",IF(OR(IF(ISNUMBER(G115),H115,F115)&gt;=$C$7,IF(ISNUMBER(G115),H115,F115)&lt;=0),"",IF(ISNUMBER(G115),H115,F115)))</f>
@@ -5047,8 +5053,8 @@
         <v>105</v>
       </c>
       <c r="B117" s="19" t="n">
-        <f aca="false">IF(C117="","",$C$5+A117-1)</f>
-        <v>46394</v>
+        <f aca="false">IF(C117="","",WORKDAY($C$5-1,A117))</f>
+        <v>46437</v>
       </c>
       <c r="C117" s="20" t="n">
         <f aca="false">IF(C116="","",IF(OR(IF(ISNUMBER(G116),H116,F116)&gt;=$C$7,IF(ISNUMBER(G116),H116,F116)&lt;=0),"",IF(ISNUMBER(G116),H116,F116)))</f>
@@ -5084,8 +5090,8 @@
         <v>106</v>
       </c>
       <c r="B118" s="19" t="n">
-        <f aca="false">IF(C118="","",$C$5+A118-1)</f>
-        <v>46395</v>
+        <f aca="false">IF(C118="","",WORKDAY($C$5-1,A118))</f>
+        <v>46440</v>
       </c>
       <c r="C118" s="20" t="n">
         <f aca="false">IF(C117="","",IF(OR(IF(ISNUMBER(G117),H117,F117)&gt;=$C$7,IF(ISNUMBER(G117),H117,F117)&lt;=0),"",IF(ISNUMBER(G117),H117,F117)))</f>
@@ -5121,8 +5127,8 @@
         <v>107</v>
       </c>
       <c r="B119" s="19" t="n">
-        <f aca="false">IF(C119="","",$C$5+A119-1)</f>
-        <v>46396</v>
+        <f aca="false">IF(C119="","",WORKDAY($C$5-1,A119))</f>
+        <v>46441</v>
       </c>
       <c r="C119" s="20" t="n">
         <f aca="false">IF(C118="","",IF(OR(IF(ISNUMBER(G118),H118,F118)&gt;=$C$7,IF(ISNUMBER(G118),H118,F118)&lt;=0),"",IF(ISNUMBER(G118),H118,F118)))</f>
@@ -5158,8 +5164,8 @@
         <v>108</v>
       </c>
       <c r="B120" s="19" t="n">
-        <f aca="false">IF(C120="","",$C$5+A120-1)</f>
-        <v>46397</v>
+        <f aca="false">IF(C120="","",WORKDAY($C$5-1,A120))</f>
+        <v>46442</v>
       </c>
       <c r="C120" s="20" t="n">
         <f aca="false">IF(C119="","",IF(OR(IF(ISNUMBER(G119),H119,F119)&gt;=$C$7,IF(ISNUMBER(G119),H119,F119)&lt;=0),"",IF(ISNUMBER(G119),H119,F119)))</f>
@@ -5195,7 +5201,7 @@
         <v/>
       </c>
       <c r="B121" s="19" t="str">
-        <f aca="false">IF(C121="","",$C$5+A121-1)</f>
+        <f aca="false">IF(C121="","",WORKDAY($C$5-1,A121))</f>
         <v/>
       </c>
       <c r="C121" s="20" t="str">
@@ -5232,7 +5238,7 @@
         <v/>
       </c>
       <c r="B122" s="19" t="str">
-        <f aca="false">IF(C122="","",$C$5+A122-1)</f>
+        <f aca="false">IF(C122="","",WORKDAY($C$5-1,A122))</f>
         <v/>
       </c>
       <c r="C122" s="20" t="str">
@@ -5269,7 +5275,7 @@
         <v/>
       </c>
       <c r="B123" s="19" t="str">
-        <f aca="false">IF(C123="","",$C$5+A123-1)</f>
+        <f aca="false">IF(C123="","",WORKDAY($C$5-1,A123))</f>
         <v/>
       </c>
       <c r="C123" s="20" t="str">
@@ -5306,7 +5312,7 @@
         <v/>
       </c>
       <c r="B124" s="19" t="str">
-        <f aca="false">IF(C124="","",$C$5+A124-1)</f>
+        <f aca="false">IF(C124="","",WORKDAY($C$5-1,A124))</f>
         <v/>
       </c>
       <c r="C124" s="20" t="str">
@@ -5343,7 +5349,7 @@
         <v/>
       </c>
       <c r="B125" s="19" t="str">
-        <f aca="false">IF(C125="","",$C$5+A125-1)</f>
+        <f aca="false">IF(C125="","",WORKDAY($C$5-1,A125))</f>
         <v/>
       </c>
       <c r="C125" s="20" t="str">
@@ -5380,7 +5386,7 @@
         <v/>
       </c>
       <c r="B126" s="19" t="str">
-        <f aca="false">IF(C126="","",$C$5+A126-1)</f>
+        <f aca="false">IF(C126="","",WORKDAY($C$5-1,A126))</f>
         <v/>
       </c>
       <c r="C126" s="20" t="str">
@@ -5417,7 +5423,7 @@
         <v/>
       </c>
       <c r="B127" s="19" t="str">
-        <f aca="false">IF(C127="","",$C$5+A127-1)</f>
+        <f aca="false">IF(C127="","",WORKDAY($C$5-1,A127))</f>
         <v/>
       </c>
       <c r="C127" s="20" t="str">
@@ -5454,7 +5460,7 @@
         <v/>
       </c>
       <c r="B128" s="19" t="str">
-        <f aca="false">IF(C128="","",$C$5+A128-1)</f>
+        <f aca="false">IF(C128="","",WORKDAY($C$5-1,A128))</f>
         <v/>
       </c>
       <c r="C128" s="20" t="str">
@@ -5491,7 +5497,7 @@
         <v/>
       </c>
       <c r="B129" s="19" t="str">
-        <f aca="false">IF(C129="","",$C$5+A129-1)</f>
+        <f aca="false">IF(C129="","",WORKDAY($C$5-1,A129))</f>
         <v/>
       </c>
       <c r="C129" s="20" t="str">
@@ -5528,7 +5534,7 @@
         <v/>
       </c>
       <c r="B130" s="19" t="str">
-        <f aca="false">IF(C130="","",$C$5+A130-1)</f>
+        <f aca="false">IF(C130="","",WORKDAY($C$5-1,A130))</f>
         <v/>
       </c>
       <c r="C130" s="20" t="str">
@@ -5565,7 +5571,7 @@
         <v/>
       </c>
       <c r="B131" s="19" t="str">
-        <f aca="false">IF(C131="","",$C$5+A131-1)</f>
+        <f aca="false">IF(C131="","",WORKDAY($C$5-1,A131))</f>
         <v/>
       </c>
       <c r="C131" s="20" t="str">
@@ -5602,7 +5608,7 @@
         <v/>
       </c>
       <c r="B132" s="19" t="str">
-        <f aca="false">IF(C132="","",$C$5+A132-1)</f>
+        <f aca="false">IF(C132="","",WORKDAY($C$5-1,A132))</f>
         <v/>
       </c>
       <c r="C132" s="20" t="str">
@@ -5639,7 +5645,7 @@
         <v/>
       </c>
       <c r="B133" s="19" t="str">
-        <f aca="false">IF(C133="","",$C$5+A133-1)</f>
+        <f aca="false">IF(C133="","",WORKDAY($C$5-1,A133))</f>
         <v/>
       </c>
       <c r="C133" s="20" t="str">
@@ -5676,7 +5682,7 @@
         <v/>
       </c>
       <c r="B134" s="19" t="str">
-        <f aca="false">IF(C134="","",$C$5+A134-1)</f>
+        <f aca="false">IF(C134="","",WORKDAY($C$5-1,A134))</f>
         <v/>
       </c>
       <c r="C134" s="20" t="str">
@@ -5713,7 +5719,7 @@
         <v/>
       </c>
       <c r="B135" s="19" t="str">
-        <f aca="false">IF(C135="","",$C$5+A135-1)</f>
+        <f aca="false">IF(C135="","",WORKDAY($C$5-1,A135))</f>
         <v/>
       </c>
       <c r="C135" s="20" t="str">
@@ -5750,7 +5756,7 @@
         <v/>
       </c>
       <c r="B136" s="19" t="str">
-        <f aca="false">IF(C136="","",$C$5+A136-1)</f>
+        <f aca="false">IF(C136="","",WORKDAY($C$5-1,A136))</f>
         <v/>
       </c>
       <c r="C136" s="20" t="str">
@@ -5787,7 +5793,7 @@
         <v/>
       </c>
       <c r="B137" s="19" t="str">
-        <f aca="false">IF(C137="","",$C$5+A137-1)</f>
+        <f aca="false">IF(C137="","",WORKDAY($C$5-1,A137))</f>
         <v/>
       </c>
       <c r="C137" s="20" t="str">
@@ -5824,7 +5830,7 @@
         <v/>
       </c>
       <c r="B138" s="19" t="str">
-        <f aca="false">IF(C138="","",$C$5+A138-1)</f>
+        <f aca="false">IF(C138="","",WORKDAY($C$5-1,A138))</f>
         <v/>
       </c>
       <c r="C138" s="20" t="str">
@@ -5861,7 +5867,7 @@
         <v/>
       </c>
       <c r="B139" s="19" t="str">
-        <f aca="false">IF(C139="","",$C$5+A139-1)</f>
+        <f aca="false">IF(C139="","",WORKDAY($C$5-1,A139))</f>
         <v/>
       </c>
       <c r="C139" s="20" t="str">
@@ -5898,7 +5904,7 @@
         <v/>
       </c>
       <c r="B140" s="19" t="str">
-        <f aca="false">IF(C140="","",$C$5+A140-1)</f>
+        <f aca="false">IF(C140="","",WORKDAY($C$5-1,A140))</f>
         <v/>
       </c>
       <c r="C140" s="20" t="str">
@@ -5935,7 +5941,7 @@
         <v/>
       </c>
       <c r="B141" s="19" t="str">
-        <f aca="false">IF(C141="","",$C$5+A141-1)</f>
+        <f aca="false">IF(C141="","",WORKDAY($C$5-1,A141))</f>
         <v/>
       </c>
       <c r="C141" s="20" t="str">
@@ -5972,7 +5978,7 @@
         <v/>
       </c>
       <c r="B142" s="19" t="str">
-        <f aca="false">IF(C142="","",$C$5+A142-1)</f>
+        <f aca="false">IF(C142="","",WORKDAY($C$5-1,A142))</f>
         <v/>
       </c>
       <c r="C142" s="20" t="str">
@@ -6009,7 +6015,7 @@
         <v/>
       </c>
       <c r="B143" s="19" t="str">
-        <f aca="false">IF(C143="","",$C$5+A143-1)</f>
+        <f aca="false">IF(C143="","",WORKDAY($C$5-1,A143))</f>
         <v/>
       </c>
       <c r="C143" s="20" t="str">
@@ -6046,7 +6052,7 @@
         <v/>
       </c>
       <c r="B144" s="19" t="str">
-        <f aca="false">IF(C144="","",$C$5+A144-1)</f>
+        <f aca="false">IF(C144="","",WORKDAY($C$5-1,A144))</f>
         <v/>
       </c>
       <c r="C144" s="20" t="str">
@@ -6083,7 +6089,7 @@
         <v/>
       </c>
       <c r="B145" s="19" t="str">
-        <f aca="false">IF(C145="","",$C$5+A145-1)</f>
+        <f aca="false">IF(C145="","",WORKDAY($C$5-1,A145))</f>
         <v/>
       </c>
       <c r="C145" s="20" t="str">
@@ -6120,7 +6126,7 @@
         <v/>
       </c>
       <c r="B146" s="19" t="str">
-        <f aca="false">IF(C146="","",$C$5+A146-1)</f>
+        <f aca="false">IF(C146="","",WORKDAY($C$5-1,A146))</f>
         <v/>
       </c>
       <c r="C146" s="20" t="str">
@@ -6157,7 +6163,7 @@
         <v/>
       </c>
       <c r="B147" s="19" t="str">
-        <f aca="false">IF(C147="","",$C$5+A147-1)</f>
+        <f aca="false">IF(C147="","",WORKDAY($C$5-1,A147))</f>
         <v/>
       </c>
       <c r="C147" s="20" t="str">
@@ -6194,7 +6200,7 @@
         <v/>
       </c>
       <c r="B148" s="19" t="str">
-        <f aca="false">IF(C148="","",$C$5+A148-1)</f>
+        <f aca="false">IF(C148="","",WORKDAY($C$5-1,A148))</f>
         <v/>
       </c>
       <c r="C148" s="20" t="str">
@@ -6231,7 +6237,7 @@
         <v/>
       </c>
       <c r="B149" s="19" t="str">
-        <f aca="false">IF(C149="","",$C$5+A149-1)</f>
+        <f aca="false">IF(C149="","",WORKDAY($C$5-1,A149))</f>
         <v/>
       </c>
       <c r="C149" s="20" t="str">
@@ -6268,7 +6274,7 @@
         <v/>
       </c>
       <c r="B150" s="19" t="str">
-        <f aca="false">IF(C150="","",$C$5+A150-1)</f>
+        <f aca="false">IF(C150="","",WORKDAY($C$5-1,A150))</f>
         <v/>
       </c>
       <c r="C150" s="20" t="str">
@@ -6305,7 +6311,7 @@
         <v/>
       </c>
       <c r="B151" s="19" t="str">
-        <f aca="false">IF(C151="","",$C$5+A151-1)</f>
+        <f aca="false">IF(C151="","",WORKDAY($C$5-1,A151))</f>
         <v/>
       </c>
       <c r="C151" s="20" t="str">
@@ -6342,7 +6348,7 @@
         <v/>
       </c>
       <c r="B152" s="19" t="str">
-        <f aca="false">IF(C152="","",$C$5+A152-1)</f>
+        <f aca="false">IF(C152="","",WORKDAY($C$5-1,A152))</f>
         <v/>
       </c>
       <c r="C152" s="20" t="str">
@@ -6379,7 +6385,7 @@
         <v/>
       </c>
       <c r="B153" s="19" t="str">
-        <f aca="false">IF(C153="","",$C$5+A153-1)</f>
+        <f aca="false">IF(C153="","",WORKDAY($C$5-1,A153))</f>
         <v/>
       </c>
       <c r="C153" s="20" t="str">
@@ -6416,7 +6422,7 @@
         <v/>
       </c>
       <c r="B154" s="19" t="str">
-        <f aca="false">IF(C154="","",$C$5+A154-1)</f>
+        <f aca="false">IF(C154="","",WORKDAY($C$5-1,A154))</f>
         <v/>
       </c>
       <c r="C154" s="20" t="str">
@@ -6453,7 +6459,7 @@
         <v/>
       </c>
       <c r="B155" s="19" t="str">
-        <f aca="false">IF(C155="","",$C$5+A155-1)</f>
+        <f aca="false">IF(C155="","",WORKDAY($C$5-1,A155))</f>
         <v/>
       </c>
       <c r="C155" s="20" t="str">
@@ -6490,7 +6496,7 @@
         <v/>
       </c>
       <c r="B156" s="19" t="str">
-        <f aca="false">IF(C156="","",$C$5+A156-1)</f>
+        <f aca="false">IF(C156="","",WORKDAY($C$5-1,A156))</f>
         <v/>
       </c>
       <c r="C156" s="20" t="str">
@@ -6527,7 +6533,7 @@
         <v/>
       </c>
       <c r="B157" s="19" t="str">
-        <f aca="false">IF(C157="","",$C$5+A157-1)</f>
+        <f aca="false">IF(C157="","",WORKDAY($C$5-1,A157))</f>
         <v/>
       </c>
       <c r="C157" s="20" t="str">
@@ -6564,7 +6570,7 @@
         <v/>
       </c>
       <c r="B158" s="19" t="str">
-        <f aca="false">IF(C158="","",$C$5+A158-1)</f>
+        <f aca="false">IF(C158="","",WORKDAY($C$5-1,A158))</f>
         <v/>
       </c>
       <c r="C158" s="20" t="str">
@@ -6601,7 +6607,7 @@
         <v/>
       </c>
       <c r="B159" s="19" t="str">
-        <f aca="false">IF(C159="","",$C$5+A159-1)</f>
+        <f aca="false">IF(C159="","",WORKDAY($C$5-1,A159))</f>
         <v/>
       </c>
       <c r="C159" s="20" t="str">
@@ -6638,7 +6644,7 @@
         <v/>
       </c>
       <c r="B160" s="19" t="str">
-        <f aca="false">IF(C160="","",$C$5+A160-1)</f>
+        <f aca="false">IF(C160="","",WORKDAY($C$5-1,A160))</f>
         <v/>
       </c>
       <c r="C160" s="20" t="str">
@@ -6675,7 +6681,7 @@
         <v/>
       </c>
       <c r="B161" s="19" t="str">
-        <f aca="false">IF(C161="","",$C$5+A161-1)</f>
+        <f aca="false">IF(C161="","",WORKDAY($C$5-1,A161))</f>
         <v/>
       </c>
       <c r="C161" s="20" t="str">
@@ -6712,7 +6718,7 @@
         <v/>
       </c>
       <c r="B162" s="19" t="str">
-        <f aca="false">IF(C162="","",$C$5+A162-1)</f>
+        <f aca="false">IF(C162="","",WORKDAY($C$5-1,A162))</f>
         <v/>
       </c>
       <c r="C162" s="20" t="str">
@@ -6749,7 +6755,7 @@
         <v/>
       </c>
       <c r="B163" s="19" t="str">
-        <f aca="false">IF(C163="","",$C$5+A163-1)</f>
+        <f aca="false">IF(C163="","",WORKDAY($C$5-1,A163))</f>
         <v/>
       </c>
       <c r="C163" s="20" t="str">
@@ -6786,7 +6792,7 @@
         <v/>
       </c>
       <c r="B164" s="19" t="str">
-        <f aca="false">IF(C164="","",$C$5+A164-1)</f>
+        <f aca="false">IF(C164="","",WORKDAY($C$5-1,A164))</f>
         <v/>
       </c>
       <c r="C164" s="20" t="str">
@@ -6823,7 +6829,7 @@
         <v/>
       </c>
       <c r="B165" s="19" t="str">
-        <f aca="false">IF(C165="","",$C$5+A165-1)</f>
+        <f aca="false">IF(C165="","",WORKDAY($C$5-1,A165))</f>
         <v/>
       </c>
       <c r="C165" s="20" t="str">
@@ -6860,7 +6866,7 @@
         <v/>
       </c>
       <c r="B166" s="19" t="str">
-        <f aca="false">IF(C166="","",$C$5+A166-1)</f>
+        <f aca="false">IF(C166="","",WORKDAY($C$5-1,A166))</f>
         <v/>
       </c>
       <c r="C166" s="20" t="str">
@@ -6897,7 +6903,7 @@
         <v/>
       </c>
       <c r="B167" s="19" t="str">
-        <f aca="false">IF(C167="","",$C$5+A167-1)</f>
+        <f aca="false">IF(C167="","",WORKDAY($C$5-1,A167))</f>
         <v/>
       </c>
       <c r="C167" s="20" t="str">
@@ -6934,7 +6940,7 @@
         <v/>
       </c>
       <c r="B168" s="19" t="str">
-        <f aca="false">IF(C168="","",$C$5+A168-1)</f>
+        <f aca="false">IF(C168="","",WORKDAY($C$5-1,A168))</f>
         <v/>
       </c>
       <c r="C168" s="20" t="str">
@@ -6971,7 +6977,7 @@
         <v/>
       </c>
       <c r="B169" s="19" t="str">
-        <f aca="false">IF(C169="","",$C$5+A169-1)</f>
+        <f aca="false">IF(C169="","",WORKDAY($C$5-1,A169))</f>
         <v/>
       </c>
       <c r="C169" s="20" t="str">
@@ -7008,7 +7014,7 @@
         <v/>
       </c>
       <c r="B170" s="19" t="str">
-        <f aca="false">IF(C170="","",$C$5+A170-1)</f>
+        <f aca="false">IF(C170="","",WORKDAY($C$5-1,A170))</f>
         <v/>
       </c>
       <c r="C170" s="20" t="str">
@@ -7045,7 +7051,7 @@
         <v/>
       </c>
       <c r="B171" s="19" t="str">
-        <f aca="false">IF(C171="","",$C$5+A171-1)</f>
+        <f aca="false">IF(C171="","",WORKDAY($C$5-1,A171))</f>
         <v/>
       </c>
       <c r="C171" s="20" t="str">
@@ -7082,7 +7088,7 @@
         <v/>
       </c>
       <c r="B172" s="19" t="str">
-        <f aca="false">IF(C172="","",$C$5+A172-1)</f>
+        <f aca="false">IF(C172="","",WORKDAY($C$5-1,A172))</f>
         <v/>
       </c>
       <c r="C172" s="20" t="str">
@@ -7119,7 +7125,7 @@
         <v/>
       </c>
       <c r="B173" s="19" t="str">
-        <f aca="false">IF(C173="","",$C$5+A173-1)</f>
+        <f aca="false">IF(C173="","",WORKDAY($C$5-1,A173))</f>
         <v/>
       </c>
       <c r="C173" s="20" t="str">
@@ -7156,7 +7162,7 @@
         <v/>
       </c>
       <c r="B174" s="19" t="str">
-        <f aca="false">IF(C174="","",$C$5+A174-1)</f>
+        <f aca="false">IF(C174="","",WORKDAY($C$5-1,A174))</f>
         <v/>
       </c>
       <c r="C174" s="20" t="str">
@@ -7193,7 +7199,7 @@
         <v/>
       </c>
       <c r="B175" s="19" t="str">
-        <f aca="false">IF(C175="","",$C$5+A175-1)</f>
+        <f aca="false">IF(C175="","",WORKDAY($C$5-1,A175))</f>
         <v/>
       </c>
       <c r="C175" s="20" t="str">
@@ -7230,7 +7236,7 @@
         <v/>
       </c>
       <c r="B176" s="19" t="str">
-        <f aca="false">IF(C176="","",$C$5+A176-1)</f>
+        <f aca="false">IF(C176="","",WORKDAY($C$5-1,A176))</f>
         <v/>
       </c>
       <c r="C176" s="20" t="str">
@@ -7267,7 +7273,7 @@
         <v/>
       </c>
       <c r="B177" s="19" t="str">
-        <f aca="false">IF(C177="","",$C$5+A177-1)</f>
+        <f aca="false">IF(C177="","",WORKDAY($C$5-1,A177))</f>
         <v/>
       </c>
       <c r="C177" s="20" t="str">
@@ -7304,7 +7310,7 @@
         <v/>
       </c>
       <c r="B178" s="19" t="str">
-        <f aca="false">IF(C178="","",$C$5+A178-1)</f>
+        <f aca="false">IF(C178="","",WORKDAY($C$5-1,A178))</f>
         <v/>
       </c>
       <c r="C178" s="20" t="str">
@@ -7341,7 +7347,7 @@
         <v/>
       </c>
       <c r="B179" s="19" t="str">
-        <f aca="false">IF(C179="","",$C$5+A179-1)</f>
+        <f aca="false">IF(C179="","",WORKDAY($C$5-1,A179))</f>
         <v/>
       </c>
       <c r="C179" s="20" t="str">
@@ -7378,7 +7384,7 @@
         <v/>
       </c>
       <c r="B180" s="19" t="str">
-        <f aca="false">IF(C180="","",$C$5+A180-1)</f>
+        <f aca="false">IF(C180="","",WORKDAY($C$5-1,A180))</f>
         <v/>
       </c>
       <c r="C180" s="20" t="str">
@@ -7415,7 +7421,7 @@
         <v/>
       </c>
       <c r="B181" s="19" t="str">
-        <f aca="false">IF(C181="","",$C$5+A181-1)</f>
+        <f aca="false">IF(C181="","",WORKDAY($C$5-1,A181))</f>
         <v/>
       </c>
       <c r="C181" s="20" t="str">
@@ -7452,7 +7458,7 @@
         <v/>
       </c>
       <c r="B182" s="19" t="str">
-        <f aca="false">IF(C182="","",$C$5+A182-1)</f>
+        <f aca="false">IF(C182="","",WORKDAY($C$5-1,A182))</f>
         <v/>
       </c>
       <c r="C182" s="20" t="str">
@@ -7489,7 +7495,7 @@
         <v/>
       </c>
       <c r="B183" s="19" t="str">
-        <f aca="false">IF(C183="","",$C$5+A183-1)</f>
+        <f aca="false">IF(C183="","",WORKDAY($C$5-1,A183))</f>
         <v/>
       </c>
       <c r="C183" s="20" t="str">
@@ -7526,7 +7532,7 @@
         <v/>
       </c>
       <c r="B184" s="19" t="str">
-        <f aca="false">IF(C184="","",$C$5+A184-1)</f>
+        <f aca="false">IF(C184="","",WORKDAY($C$5-1,A184))</f>
         <v/>
       </c>
       <c r="C184" s="20" t="str">
@@ -7563,7 +7569,7 @@
         <v/>
       </c>
       <c r="B185" s="19" t="str">
-        <f aca="false">IF(C185="","",$C$5+A185-1)</f>
+        <f aca="false">IF(C185="","",WORKDAY($C$5-1,A185))</f>
         <v/>
       </c>
       <c r="C185" s="20" t="str">
@@ -7600,7 +7606,7 @@
         <v/>
       </c>
       <c r="B186" s="19" t="str">
-        <f aca="false">IF(C186="","",$C$5+A186-1)</f>
+        <f aca="false">IF(C186="","",WORKDAY($C$5-1,A186))</f>
         <v/>
       </c>
       <c r="C186" s="20" t="str">
@@ -7637,7 +7643,7 @@
         <v/>
       </c>
       <c r="B187" s="19" t="str">
-        <f aca="false">IF(C187="","",$C$5+A187-1)</f>
+        <f aca="false">IF(C187="","",WORKDAY($C$5-1,A187))</f>
         <v/>
       </c>
       <c r="C187" s="20" t="str">
@@ -7674,7 +7680,7 @@
         <v/>
       </c>
       <c r="B188" s="19" t="str">
-        <f aca="false">IF(C188="","",$C$5+A188-1)</f>
+        <f aca="false">IF(C188="","",WORKDAY($C$5-1,A188))</f>
         <v/>
       </c>
       <c r="C188" s="20" t="str">
@@ -7711,7 +7717,7 @@
         <v/>
       </c>
       <c r="B189" s="19" t="str">
-        <f aca="false">IF(C189="","",$C$5+A189-1)</f>
+        <f aca="false">IF(C189="","",WORKDAY($C$5-1,A189))</f>
         <v/>
       </c>
       <c r="C189" s="20" t="str">
@@ -7748,7 +7754,7 @@
         <v/>
       </c>
       <c r="B190" s="19" t="str">
-        <f aca="false">IF(C190="","",$C$5+A190-1)</f>
+        <f aca="false">IF(C190="","",WORKDAY($C$5-1,A190))</f>
         <v/>
       </c>
       <c r="C190" s="20" t="str">
@@ -7785,7 +7791,7 @@
         <v/>
       </c>
       <c r="B191" s="19" t="str">
-        <f aca="false">IF(C191="","",$C$5+A191-1)</f>
+        <f aca="false">IF(C191="","",WORKDAY($C$5-1,A191))</f>
         <v/>
       </c>
       <c r="C191" s="20" t="str">
@@ -7822,7 +7828,7 @@
         <v/>
       </c>
       <c r="B192" s="19" t="str">
-        <f aca="false">IF(C192="","",$C$5+A192-1)</f>
+        <f aca="false">IF(C192="","",WORKDAY($C$5-1,A192))</f>
         <v/>
       </c>
       <c r="C192" s="20" t="str">
@@ -7859,7 +7865,7 @@
         <v/>
       </c>
       <c r="B193" s="19" t="str">
-        <f aca="false">IF(C193="","",$C$5+A193-1)</f>
+        <f aca="false">IF(C193="","",WORKDAY($C$5-1,A193))</f>
         <v/>
       </c>
       <c r="C193" s="20" t="str">
@@ -7896,7 +7902,7 @@
         <v/>
       </c>
       <c r="B194" s="19" t="str">
-        <f aca="false">IF(C194="","",$C$5+A194-1)</f>
+        <f aca="false">IF(C194="","",WORKDAY($C$5-1,A194))</f>
         <v/>
       </c>
       <c r="C194" s="20" t="str">
@@ -7933,7 +7939,7 @@
         <v/>
       </c>
       <c r="B195" s="19" t="str">
-        <f aca="false">IF(C195="","",$C$5+A195-1)</f>
+        <f aca="false">IF(C195="","",WORKDAY($C$5-1,A195))</f>
         <v/>
       </c>
       <c r="C195" s="20" t="str">
@@ -7970,7 +7976,7 @@
         <v/>
       </c>
       <c r="B196" s="19" t="str">
-        <f aca="false">IF(C196="","",$C$5+A196-1)</f>
+        <f aca="false">IF(C196="","",WORKDAY($C$5-1,A196))</f>
         <v/>
       </c>
       <c r="C196" s="20" t="str">
@@ -8007,7 +8013,7 @@
         <v/>
       </c>
       <c r="B197" s="19" t="str">
-        <f aca="false">IF(C197="","",$C$5+A197-1)</f>
+        <f aca="false">IF(C197="","",WORKDAY($C$5-1,A197))</f>
         <v/>
       </c>
       <c r="C197" s="20" t="str">
@@ -8044,7 +8050,7 @@
         <v/>
       </c>
       <c r="B198" s="19" t="str">
-        <f aca="false">IF(C198="","",$C$5+A198-1)</f>
+        <f aca="false">IF(C198="","",WORKDAY($C$5-1,A198))</f>
         <v/>
       </c>
       <c r="C198" s="20" t="str">
@@ -8081,7 +8087,7 @@
         <v/>
       </c>
       <c r="B199" s="19" t="str">
-        <f aca="false">IF(C199="","",$C$5+A199-1)</f>
+        <f aca="false">IF(C199="","",WORKDAY($C$5-1,A199))</f>
         <v/>
       </c>
       <c r="C199" s="20" t="str">
@@ -8118,7 +8124,7 @@
         <v/>
       </c>
       <c r="B200" s="19" t="str">
-        <f aca="false">IF(C200="","",$C$5+A200-1)</f>
+        <f aca="false">IF(C200="","",WORKDAY($C$5-1,A200))</f>
         <v/>
       </c>
       <c r="C200" s="20" t="str">
@@ -8155,7 +8161,7 @@
         <v/>
       </c>
       <c r="B201" s="19" t="str">
-        <f aca="false">IF(C201="","",$C$5+A201-1)</f>
+        <f aca="false">IF(C201="","",WORKDAY($C$5-1,A201))</f>
         <v/>
       </c>
       <c r="C201" s="20" t="str">
@@ -8192,7 +8198,7 @@
         <v/>
       </c>
       <c r="B202" s="19" t="str">
-        <f aca="false">IF(C202="","",$C$5+A202-1)</f>
+        <f aca="false">IF(C202="","",WORKDAY($C$5-1,A202))</f>
         <v/>
       </c>
       <c r="C202" s="20" t="str">
@@ -8229,7 +8235,7 @@
         <v/>
       </c>
       <c r="B203" s="19" t="str">
-        <f aca="false">IF(C203="","",$C$5+A203-1)</f>
+        <f aca="false">IF(C203="","",WORKDAY($C$5-1,A203))</f>
         <v/>
       </c>
       <c r="C203" s="20" t="str">
@@ -8266,7 +8272,7 @@
         <v/>
       </c>
       <c r="B204" s="19" t="str">
-        <f aca="false">IF(C204="","",$C$5+A204-1)</f>
+        <f aca="false">IF(C204="","",WORKDAY($C$5-1,A204))</f>
         <v/>
       </c>
       <c r="C204" s="20" t="str">
@@ -8303,7 +8309,7 @@
         <v/>
       </c>
       <c r="B205" s="19" t="str">
-        <f aca="false">IF(C205="","",$C$5+A205-1)</f>
+        <f aca="false">IF(C205="","",WORKDAY($C$5-1,A205))</f>
         <v/>
       </c>
       <c r="C205" s="20" t="str">
@@ -8340,7 +8346,7 @@
         <v/>
       </c>
       <c r="B206" s="19" t="str">
-        <f aca="false">IF(C206="","",$C$5+A206-1)</f>
+        <f aca="false">IF(C206="","",WORKDAY($C$5-1,A206))</f>
         <v/>
       </c>
       <c r="C206" s="20" t="str">
@@ -8377,7 +8383,7 @@
         <v/>
       </c>
       <c r="B207" s="19" t="str">
-        <f aca="false">IF(C207="","",$C$5+A207-1)</f>
+        <f aca="false">IF(C207="","",WORKDAY($C$5-1,A207))</f>
         <v/>
       </c>
       <c r="C207" s="20" t="str">
@@ -8414,7 +8420,7 @@
         <v/>
       </c>
       <c r="B208" s="19" t="str">
-        <f aca="false">IF(C208="","",$C$5+A208-1)</f>
+        <f aca="false">IF(C208="","",WORKDAY($C$5-1,A208))</f>
         <v/>
       </c>
       <c r="C208" s="20" t="str">
@@ -8451,7 +8457,7 @@
         <v/>
       </c>
       <c r="B209" s="19" t="str">
-        <f aca="false">IF(C209="","",$C$5+A209-1)</f>
+        <f aca="false">IF(C209="","",WORKDAY($C$5-1,A209))</f>
         <v/>
       </c>
       <c r="C209" s="20" t="str">
@@ -8488,7 +8494,7 @@
         <v/>
       </c>
       <c r="B210" s="19" t="str">
-        <f aca="false">IF(C210="","",$C$5+A210-1)</f>
+        <f aca="false">IF(C210="","",WORKDAY($C$5-1,A210))</f>
         <v/>
       </c>
       <c r="C210" s="20" t="str">
@@ -8525,7 +8531,7 @@
         <v/>
       </c>
       <c r="B211" s="19" t="str">
-        <f aca="false">IF(C211="","",$C$5+A211-1)</f>
+        <f aca="false">IF(C211="","",WORKDAY($C$5-1,A211))</f>
         <v/>
       </c>
       <c r="C211" s="20" t="str">
@@ -8562,7 +8568,7 @@
         <v/>
       </c>
       <c r="B212" s="19" t="str">
-        <f aca="false">IF(C212="","",$C$5+A212-1)</f>
+        <f aca="false">IF(C212="","",WORKDAY($C$5-1,A212))</f>
         <v/>
       </c>
       <c r="C212" s="20" t="str">
@@ -8599,7 +8605,7 @@
         <v/>
       </c>
       <c r="B213" s="19" t="str">
-        <f aca="false">IF(C213="","",$C$5+A213-1)</f>
+        <f aca="false">IF(C213="","",WORKDAY($C$5-1,A213))</f>
         <v/>
       </c>
       <c r="C213" s="20" t="str">
@@ -8636,7 +8642,7 @@
         <v/>
       </c>
       <c r="B214" s="19" t="str">
-        <f aca="false">IF(C214="","",$C$5+A214-1)</f>
+        <f aca="false">IF(C214="","",WORKDAY($C$5-1,A214))</f>
         <v/>
       </c>
       <c r="C214" s="20" t="str">
@@ -8673,7 +8679,7 @@
         <v/>
       </c>
       <c r="B215" s="19" t="str">
-        <f aca="false">IF(C215="","",$C$5+A215-1)</f>
+        <f aca="false">IF(C215="","",WORKDAY($C$5-1,A215))</f>
         <v/>
       </c>
       <c r="C215" s="20" t="str">
@@ -8710,7 +8716,7 @@
         <v/>
       </c>
       <c r="B216" s="19" t="str">
-        <f aca="false">IF(C216="","",$C$5+A216-1)</f>
+        <f aca="false">IF(C216="","",WORKDAY($C$5-1,A216))</f>
         <v/>
       </c>
       <c r="C216" s="20" t="str">
@@ -8747,7 +8753,7 @@
         <v/>
       </c>
       <c r="B217" s="19" t="str">
-        <f aca="false">IF(C217="","",$C$5+A217-1)</f>
+        <f aca="false">IF(C217="","",WORKDAY($C$5-1,A217))</f>
         <v/>
       </c>
       <c r="C217" s="20" t="str">
@@ -8784,7 +8790,7 @@
         <v/>
       </c>
       <c r="B218" s="19" t="str">
-        <f aca="false">IF(C218="","",$C$5+A218-1)</f>
+        <f aca="false">IF(C218="","",WORKDAY($C$5-1,A218))</f>
         <v/>
       </c>
       <c r="C218" s="20" t="str">
@@ -8821,7 +8827,7 @@
         <v/>
       </c>
       <c r="B219" s="19" t="str">
-        <f aca="false">IF(C219="","",$C$5+A219-1)</f>
+        <f aca="false">IF(C219="","",WORKDAY($C$5-1,A219))</f>
         <v/>
       </c>
       <c r="C219" s="20" t="str">
@@ -8858,7 +8864,7 @@
         <v/>
       </c>
       <c r="B220" s="19" t="str">
-        <f aca="false">IF(C220="","",$C$5+A220-1)</f>
+        <f aca="false">IF(C220="","",WORKDAY($C$5-1,A220))</f>
         <v/>
       </c>
       <c r="C220" s="20" t="str">
@@ -8895,7 +8901,7 @@
         <v/>
       </c>
       <c r="B221" s="19" t="str">
-        <f aca="false">IF(C221="","",$C$5+A221-1)</f>
+        <f aca="false">IF(C221="","",WORKDAY($C$5-1,A221))</f>
         <v/>
       </c>
       <c r="C221" s="20" t="str">
@@ -8932,7 +8938,7 @@
         <v/>
       </c>
       <c r="B222" s="19" t="str">
-        <f aca="false">IF(C222="","",$C$5+A222-1)</f>
+        <f aca="false">IF(C222="","",WORKDAY($C$5-1,A222))</f>
         <v/>
       </c>
       <c r="C222" s="20" t="str">
@@ -8969,7 +8975,7 @@
         <v/>
       </c>
       <c r="B223" s="19" t="str">
-        <f aca="false">IF(C223="","",$C$5+A223-1)</f>
+        <f aca="false">IF(C223="","",WORKDAY($C$5-1,A223))</f>
         <v/>
       </c>
       <c r="C223" s="20" t="str">
@@ -9006,7 +9012,7 @@
         <v/>
       </c>
       <c r="B224" s="19" t="str">
-        <f aca="false">IF(C224="","",$C$5+A224-1)</f>
+        <f aca="false">IF(C224="","",WORKDAY($C$5-1,A224))</f>
         <v/>
       </c>
       <c r="C224" s="20" t="str">
@@ -9043,7 +9049,7 @@
         <v/>
       </c>
       <c r="B225" s="19" t="str">
-        <f aca="false">IF(C225="","",$C$5+A225-1)</f>
+        <f aca="false">IF(C225="","",WORKDAY($C$5-1,A225))</f>
         <v/>
       </c>
       <c r="C225" s="20" t="str">
@@ -9080,7 +9086,7 @@
         <v/>
       </c>
       <c r="B226" s="19" t="str">
-        <f aca="false">IF(C226="","",$C$5+A226-1)</f>
+        <f aca="false">IF(C226="","",WORKDAY($C$5-1,A226))</f>
         <v/>
       </c>
       <c r="C226" s="20" t="str">
@@ -9117,7 +9123,7 @@
         <v/>
       </c>
       <c r="B227" s="19" t="str">
-        <f aca="false">IF(C227="","",$C$5+A227-1)</f>
+        <f aca="false">IF(C227="","",WORKDAY($C$5-1,A227))</f>
         <v/>
       </c>
       <c r="C227" s="20" t="str">
@@ -9154,7 +9160,7 @@
         <v/>
       </c>
       <c r="B228" s="19" t="str">
-        <f aca="false">IF(C228="","",$C$5+A228-1)</f>
+        <f aca="false">IF(C228="","",WORKDAY($C$5-1,A228))</f>
         <v/>
       </c>
       <c r="C228" s="20" t="str">
@@ -9191,7 +9197,7 @@
         <v/>
       </c>
       <c r="B229" s="19" t="str">
-        <f aca="false">IF(C229="","",$C$5+A229-1)</f>
+        <f aca="false">IF(C229="","",WORKDAY($C$5-1,A229))</f>
         <v/>
       </c>
       <c r="C229" s="20" t="str">
@@ -9228,7 +9234,7 @@
         <v/>
       </c>
       <c r="B230" s="19" t="str">
-        <f aca="false">IF(C230="","",$C$5+A230-1)</f>
+        <f aca="false">IF(C230="","",WORKDAY($C$5-1,A230))</f>
         <v/>
       </c>
       <c r="C230" s="20" t="str">
@@ -9265,7 +9271,7 @@
         <v/>
       </c>
       <c r="B231" s="19" t="str">
-        <f aca="false">IF(C231="","",$C$5+A231-1)</f>
+        <f aca="false">IF(C231="","",WORKDAY($C$5-1,A231))</f>
         <v/>
       </c>
       <c r="C231" s="20" t="str">
@@ -9302,7 +9308,7 @@
         <v/>
       </c>
       <c r="B232" s="19" t="str">
-        <f aca="false">IF(C232="","",$C$5+A232-1)</f>
+        <f aca="false">IF(C232="","",WORKDAY($C$5-1,A232))</f>
         <v/>
       </c>
       <c r="C232" s="20" t="str">
@@ -9339,7 +9345,7 @@
         <v/>
       </c>
       <c r="B233" s="19" t="str">
-        <f aca="false">IF(C233="","",$C$5+A233-1)</f>
+        <f aca="false">IF(C233="","",WORKDAY($C$5-1,A233))</f>
         <v/>
       </c>
       <c r="C233" s="20" t="str">
@@ -9376,7 +9382,7 @@
         <v/>
       </c>
       <c r="B234" s="19" t="str">
-        <f aca="false">IF(C234="","",$C$5+A234-1)</f>
+        <f aca="false">IF(C234="","",WORKDAY($C$5-1,A234))</f>
         <v/>
       </c>
       <c r="C234" s="20" t="str">
@@ -9413,7 +9419,7 @@
         <v/>
       </c>
       <c r="B235" s="19" t="str">
-        <f aca="false">IF(C235="","",$C$5+A235-1)</f>
+        <f aca="false">IF(C235="","",WORKDAY($C$5-1,A235))</f>
         <v/>
       </c>
       <c r="C235" s="20" t="str">
@@ -9450,7 +9456,7 @@
         <v/>
       </c>
       <c r="B236" s="19" t="str">
-        <f aca="false">IF(C236="","",$C$5+A236-1)</f>
+        <f aca="false">IF(C236="","",WORKDAY($C$5-1,A236))</f>
         <v/>
       </c>
       <c r="C236" s="20" t="str">
@@ -9487,7 +9493,7 @@
         <v/>
       </c>
       <c r="B237" s="19" t="str">
-        <f aca="false">IF(C237="","",$C$5+A237-1)</f>
+        <f aca="false">IF(C237="","",WORKDAY($C$5-1,A237))</f>
         <v/>
       </c>
       <c r="C237" s="20" t="str">
@@ -9524,7 +9530,7 @@
         <v/>
       </c>
       <c r="B238" s="19" t="str">
-        <f aca="false">IF(C238="","",$C$5+A238-1)</f>
+        <f aca="false">IF(C238="","",WORKDAY($C$5-1,A238))</f>
         <v/>
       </c>
       <c r="C238" s="20" t="str">
@@ -9561,7 +9567,7 @@
         <v/>
       </c>
       <c r="B239" s="19" t="str">
-        <f aca="false">IF(C239="","",$C$5+A239-1)</f>
+        <f aca="false">IF(C239="","",WORKDAY($C$5-1,A239))</f>
         <v/>
       </c>
       <c r="C239" s="20" t="str">
@@ -9598,7 +9604,7 @@
         <v/>
       </c>
       <c r="B240" s="19" t="str">
-        <f aca="false">IF(C240="","",$C$5+A240-1)</f>
+        <f aca="false">IF(C240="","",WORKDAY($C$5-1,A240))</f>
         <v/>
       </c>
       <c r="C240" s="20" t="str">
@@ -9635,7 +9641,7 @@
         <v/>
       </c>
       <c r="B241" s="19" t="str">
-        <f aca="false">IF(C241="","",$C$5+A241-1)</f>
+        <f aca="false">IF(C241="","",WORKDAY($C$5-1,A241))</f>
         <v/>
       </c>
       <c r="C241" s="20" t="str">
@@ -9672,7 +9678,7 @@
         <v/>
       </c>
       <c r="B242" s="19" t="str">
-        <f aca="false">IF(C242="","",$C$5+A242-1)</f>
+        <f aca="false">IF(C242="","",WORKDAY($C$5-1,A242))</f>
         <v/>
       </c>
       <c r="C242" s="20" t="str">
@@ -9709,7 +9715,7 @@
         <v/>
       </c>
       <c r="B243" s="19" t="str">
-        <f aca="false">IF(C243="","",$C$5+A243-1)</f>
+        <f aca="false">IF(C243="","",WORKDAY($C$5-1,A243))</f>
         <v/>
       </c>
       <c r="C243" s="20" t="str">
@@ -9746,7 +9752,7 @@
         <v/>
       </c>
       <c r="B244" s="19" t="str">
-        <f aca="false">IF(C244="","",$C$5+A244-1)</f>
+        <f aca="false">IF(C244="","",WORKDAY($C$5-1,A244))</f>
         <v/>
       </c>
       <c r="C244" s="20" t="str">
@@ -9783,7 +9789,7 @@
         <v/>
       </c>
       <c r="B245" s="19" t="str">
-        <f aca="false">IF(C245="","",$C$5+A245-1)</f>
+        <f aca="false">IF(C245="","",WORKDAY($C$5-1,A245))</f>
         <v/>
       </c>
       <c r="C245" s="20" t="str">
@@ -9820,7 +9826,7 @@
         <v/>
       </c>
       <c r="B246" s="19" t="str">
-        <f aca="false">IF(C246="","",$C$5+A246-1)</f>
+        <f aca="false">IF(C246="","",WORKDAY($C$5-1,A246))</f>
         <v/>
       </c>
       <c r="C246" s="20" t="str">
@@ -9857,7 +9863,7 @@
         <v/>
       </c>
       <c r="B247" s="19" t="str">
-        <f aca="false">IF(C247="","",$C$5+A247-1)</f>
+        <f aca="false">IF(C247="","",WORKDAY($C$5-1,A247))</f>
         <v/>
       </c>
       <c r="C247" s="20" t="str">
@@ -9894,7 +9900,7 @@
         <v/>
       </c>
       <c r="B248" s="19" t="str">
-        <f aca="false">IF(C248="","",$C$5+A248-1)</f>
+        <f aca="false">IF(C248="","",WORKDAY($C$5-1,A248))</f>
         <v/>
       </c>
       <c r="C248" s="20" t="str">
@@ -9931,7 +9937,7 @@
         <v/>
       </c>
       <c r="B249" s="19" t="str">
-        <f aca="false">IF(C249="","",$C$5+A249-1)</f>
+        <f aca="false">IF(C249="","",WORKDAY($C$5-1,A249))</f>
         <v/>
       </c>
       <c r="C249" s="20" t="str">
@@ -9968,7 +9974,7 @@
         <v/>
       </c>
       <c r="B250" s="19" t="str">
-        <f aca="false">IF(C250="","",$C$5+A250-1)</f>
+        <f aca="false">IF(C250="","",WORKDAY($C$5-1,A250))</f>
         <v/>
       </c>
       <c r="C250" s="20" t="str">
@@ -10005,7 +10011,7 @@
         <v/>
       </c>
       <c r="B251" s="19" t="str">
-        <f aca="false">IF(C251="","",$C$5+A251-1)</f>
+        <f aca="false">IF(C251="","",WORKDAY($C$5-1,A251))</f>
         <v/>
       </c>
       <c r="C251" s="20" t="str">
@@ -10042,7 +10048,7 @@
         <v/>
       </c>
       <c r="B252" s="19" t="str">
-        <f aca="false">IF(C252="","",$C$5+A252-1)</f>
+        <f aca="false">IF(C252="","",WORKDAY($C$5-1,A252))</f>
         <v/>
       </c>
       <c r="C252" s="20" t="str">
@@ -10079,7 +10085,7 @@
         <v/>
       </c>
       <c r="B253" s="19" t="str">
-        <f aca="false">IF(C253="","",$C$5+A253-1)</f>
+        <f aca="false">IF(C253="","",WORKDAY($C$5-1,A253))</f>
         <v/>
       </c>
       <c r="C253" s="20" t="str">
@@ -10116,7 +10122,7 @@
         <v/>
       </c>
       <c r="B254" s="19" t="str">
-        <f aca="false">IF(C254="","",$C$5+A254-1)</f>
+        <f aca="false">IF(C254="","",WORKDAY($C$5-1,A254))</f>
         <v/>
       </c>
       <c r="C254" s="20" t="str">
@@ -10153,7 +10159,7 @@
         <v/>
       </c>
       <c r="B255" s="19" t="str">
-        <f aca="false">IF(C255="","",$C$5+A255-1)</f>
+        <f aca="false">IF(C255="","",WORKDAY($C$5-1,A255))</f>
         <v/>
       </c>
       <c r="C255" s="20" t="str">
@@ -10190,7 +10196,7 @@
         <v/>
       </c>
       <c r="B256" s="19" t="str">
-        <f aca="false">IF(C256="","",$C$5+A256-1)</f>
+        <f aca="false">IF(C256="","",WORKDAY($C$5-1,A256))</f>
         <v/>
       </c>
       <c r="C256" s="20" t="str">
@@ -10227,7 +10233,7 @@
         <v/>
       </c>
       <c r="B257" s="19" t="str">
-        <f aca="false">IF(C257="","",$C$5+A257-1)</f>
+        <f aca="false">IF(C257="","",WORKDAY($C$5-1,A257))</f>
         <v/>
       </c>
       <c r="C257" s="20" t="str">
@@ -10264,7 +10270,7 @@
         <v/>
       </c>
       <c r="B258" s="19" t="str">
-        <f aca="false">IF(C258="","",$C$5+A258-1)</f>
+        <f aca="false">IF(C258="","",WORKDAY($C$5-1,A258))</f>
         <v/>
       </c>
       <c r="C258" s="20" t="str">
@@ -10301,7 +10307,7 @@
         <v/>
       </c>
       <c r="B259" s="19" t="str">
-        <f aca="false">IF(C259="","",$C$5+A259-1)</f>
+        <f aca="false">IF(C259="","",WORKDAY($C$5-1,A259))</f>
         <v/>
       </c>
       <c r="C259" s="20" t="str">
@@ -10338,7 +10344,7 @@
         <v/>
       </c>
       <c r="B260" s="19" t="str">
-        <f aca="false">IF(C260="","",$C$5+A260-1)</f>
+        <f aca="false">IF(C260="","",WORKDAY($C$5-1,A260))</f>
         <v/>
       </c>
       <c r="C260" s="20" t="str">
@@ -10375,7 +10381,7 @@
         <v/>
       </c>
       <c r="B261" s="19" t="str">
-        <f aca="false">IF(C261="","",$C$5+A261-1)</f>
+        <f aca="false">IF(C261="","",WORKDAY($C$5-1,A261))</f>
         <v/>
       </c>
       <c r="C261" s="20" t="str">
@@ -10412,7 +10418,7 @@
         <v/>
       </c>
       <c r="B262" s="19" t="str">
-        <f aca="false">IF(C262="","",$C$5+A262-1)</f>
+        <f aca="false">IF(C262="","",WORKDAY($C$5-1,A262))</f>
         <v/>
       </c>
       <c r="C262" s="20" t="str">
@@ -10449,7 +10455,7 @@
         <v/>
       </c>
       <c r="B263" s="19" t="str">
-        <f aca="false">IF(C263="","",$C$5+A263-1)</f>
+        <f aca="false">IF(C263="","",WORKDAY($C$5-1,A263))</f>
         <v/>
       </c>
       <c r="C263" s="20" t="str">
@@ -10486,7 +10492,7 @@
         <v/>
       </c>
       <c r="B264" s="19" t="str">
-        <f aca="false">IF(C264="","",$C$5+A264-1)</f>
+        <f aca="false">IF(C264="","",WORKDAY($C$5-1,A264))</f>
         <v/>
       </c>
       <c r="C264" s="20" t="str">
@@ -10523,7 +10529,7 @@
         <v/>
       </c>
       <c r="B265" s="19" t="str">
-        <f aca="false">IF(C265="","",$C$5+A265-1)</f>
+        <f aca="false">IF(C265="","",WORKDAY($C$5-1,A265))</f>
         <v/>
       </c>
       <c r="C265" s="20" t="str">
@@ -10560,7 +10566,7 @@
         <v/>
       </c>
       <c r="B266" s="19" t="str">
-        <f aca="false">IF(C266="","",$C$5+A266-1)</f>
+        <f aca="false">IF(C266="","",WORKDAY($C$5-1,A266))</f>
         <v/>
       </c>
       <c r="C266" s="20" t="str">
@@ -10597,7 +10603,7 @@
         <v/>
       </c>
       <c r="B267" s="19" t="str">
-        <f aca="false">IF(C267="","",$C$5+A267-1)</f>
+        <f aca="false">IF(C267="","",WORKDAY($C$5-1,A267))</f>
         <v/>
       </c>
       <c r="C267" s="20" t="str">
@@ -10634,7 +10640,7 @@
         <v/>
       </c>
       <c r="B268" s="19" t="str">
-        <f aca="false">IF(C268="","",$C$5+A268-1)</f>
+        <f aca="false">IF(C268="","",WORKDAY($C$5-1,A268))</f>
         <v/>
       </c>
       <c r="C268" s="20" t="str">
@@ -10671,7 +10677,7 @@
         <v/>
       </c>
       <c r="B269" s="19" t="str">
-        <f aca="false">IF(C269="","",$C$5+A269-1)</f>
+        <f aca="false">IF(C269="","",WORKDAY($C$5-1,A269))</f>
         <v/>
       </c>
       <c r="C269" s="20" t="str">
@@ -10708,7 +10714,7 @@
         <v/>
       </c>
       <c r="B270" s="19" t="str">
-        <f aca="false">IF(C270="","",$C$5+A270-1)</f>
+        <f aca="false">IF(C270="","",WORKDAY($C$5-1,A270))</f>
         <v/>
       </c>
       <c r="C270" s="20" t="str">
@@ -10745,7 +10751,7 @@
         <v/>
       </c>
       <c r="B271" s="19" t="str">
-        <f aca="false">IF(C271="","",$C$5+A271-1)</f>
+        <f aca="false">IF(C271="","",WORKDAY($C$5-1,A271))</f>
         <v/>
       </c>
       <c r="C271" s="20" t="str">
@@ -10782,7 +10788,7 @@
         <v/>
       </c>
       <c r="B272" s="19" t="str">
-        <f aca="false">IF(C272="","",$C$5+A272-1)</f>
+        <f aca="false">IF(C272="","",WORKDAY($C$5-1,A272))</f>
         <v/>
       </c>
       <c r="C272" s="20" t="str">
@@ -10819,7 +10825,7 @@
         <v/>
       </c>
       <c r="B273" s="19" t="str">
-        <f aca="false">IF(C273="","",$C$5+A273-1)</f>
+        <f aca="false">IF(C273="","",WORKDAY($C$5-1,A273))</f>
         <v/>
       </c>
       <c r="C273" s="20" t="str">
@@ -10856,7 +10862,7 @@
         <v/>
       </c>
       <c r="B274" s="19" t="str">
-        <f aca="false">IF(C274="","",$C$5+A274-1)</f>
+        <f aca="false">IF(C274="","",WORKDAY($C$5-1,A274))</f>
         <v/>
       </c>
       <c r="C274" s="20" t="str">
@@ -10893,7 +10899,7 @@
         <v/>
       </c>
       <c r="B275" s="19" t="str">
-        <f aca="false">IF(C275="","",$C$5+A275-1)</f>
+        <f aca="false">IF(C275="","",WORKDAY($C$5-1,A275))</f>
         <v/>
       </c>
       <c r="C275" s="20" t="str">
@@ -10930,7 +10936,7 @@
         <v/>
       </c>
       <c r="B276" s="19" t="str">
-        <f aca="false">IF(C276="","",$C$5+A276-1)</f>
+        <f aca="false">IF(C276="","",WORKDAY($C$5-1,A276))</f>
         <v/>
       </c>
       <c r="C276" s="20" t="str">
@@ -10967,7 +10973,7 @@
         <v/>
       </c>
       <c r="B277" s="19" t="str">
-        <f aca="false">IF(C277="","",$C$5+A277-1)</f>
+        <f aca="false">IF(C277="","",WORKDAY($C$5-1,A277))</f>
         <v/>
       </c>
       <c r="C277" s="20" t="str">
@@ -11004,7 +11010,7 @@
         <v/>
       </c>
       <c r="B278" s="19" t="str">
-        <f aca="false">IF(C278="","",$C$5+A278-1)</f>
+        <f aca="false">IF(C278="","",WORKDAY($C$5-1,A278))</f>
         <v/>
       </c>
       <c r="C278" s="20" t="str">
@@ -11041,7 +11047,7 @@
         <v/>
       </c>
       <c r="B279" s="19" t="str">
-        <f aca="false">IF(C279="","",$C$5+A279-1)</f>
+        <f aca="false">IF(C279="","",WORKDAY($C$5-1,A279))</f>
         <v/>
       </c>
       <c r="C279" s="20" t="str">
@@ -11078,7 +11084,7 @@
         <v/>
       </c>
       <c r="B280" s="19" t="str">
-        <f aca="false">IF(C280="","",$C$5+A280-1)</f>
+        <f aca="false">IF(C280="","",WORKDAY($C$5-1,A280))</f>
         <v/>
       </c>
       <c r="C280" s="20" t="str">
@@ -11115,7 +11121,7 @@
         <v/>
       </c>
       <c r="B281" s="19" t="str">
-        <f aca="false">IF(C281="","",$C$5+A281-1)</f>
+        <f aca="false">IF(C281="","",WORKDAY($C$5-1,A281))</f>
         <v/>
       </c>
       <c r="C281" s="20" t="str">
@@ -11152,7 +11158,7 @@
         <v/>
       </c>
       <c r="B282" s="19" t="str">
-        <f aca="false">IF(C282="","",$C$5+A282-1)</f>
+        <f aca="false">IF(C282="","",WORKDAY($C$5-1,A282))</f>
         <v/>
       </c>
       <c r="C282" s="20" t="str">
@@ -11189,7 +11195,7 @@
         <v/>
       </c>
       <c r="B283" s="19" t="str">
-        <f aca="false">IF(C283="","",$C$5+A283-1)</f>
+        <f aca="false">IF(C283="","",WORKDAY($C$5-1,A283))</f>
         <v/>
       </c>
       <c r="C283" s="20" t="str">
@@ -11226,7 +11232,7 @@
         <v/>
       </c>
       <c r="B284" s="19" t="str">
-        <f aca="false">IF(C284="","",$C$5+A284-1)</f>
+        <f aca="false">IF(C284="","",WORKDAY($C$5-1,A284))</f>
         <v/>
       </c>
       <c r="C284" s="20" t="str">
@@ -11263,7 +11269,7 @@
         <v/>
       </c>
       <c r="B285" s="19" t="str">
-        <f aca="false">IF(C285="","",$C$5+A285-1)</f>
+        <f aca="false">IF(C285="","",WORKDAY($C$5-1,A285))</f>
         <v/>
       </c>
       <c r="C285" s="20" t="str">
@@ -11300,7 +11306,7 @@
         <v/>
       </c>
       <c r="B286" s="19" t="str">
-        <f aca="false">IF(C286="","",$C$5+A286-1)</f>
+        <f aca="false">IF(C286="","",WORKDAY($C$5-1,A286))</f>
         <v/>
       </c>
       <c r="C286" s="20" t="str">
@@ -11337,7 +11343,7 @@
         <v/>
       </c>
       <c r="B287" s="19" t="str">
-        <f aca="false">IF(C287="","",$C$5+A287-1)</f>
+        <f aca="false">IF(C287="","",WORKDAY($C$5-1,A287))</f>
         <v/>
       </c>
       <c r="C287" s="20" t="str">
@@ -11374,7 +11380,7 @@
         <v/>
       </c>
       <c r="B288" s="19" t="str">
-        <f aca="false">IF(C288="","",$C$5+A288-1)</f>
+        <f aca="false">IF(C288="","",WORKDAY($C$5-1,A288))</f>
         <v/>
       </c>
       <c r="C288" s="20" t="str">
@@ -11411,7 +11417,7 @@
         <v/>
       </c>
       <c r="B289" s="19" t="str">
-        <f aca="false">IF(C289="","",$C$5+A289-1)</f>
+        <f aca="false">IF(C289="","",WORKDAY($C$5-1,A289))</f>
         <v/>
       </c>
       <c r="C289" s="20" t="str">
@@ -11448,7 +11454,7 @@
         <v/>
       </c>
       <c r="B290" s="19" t="str">
-        <f aca="false">IF(C290="","",$C$5+A290-1)</f>
+        <f aca="false">IF(C290="","",WORKDAY($C$5-1,A290))</f>
         <v/>
       </c>
       <c r="C290" s="20" t="str">
@@ -11485,7 +11491,7 @@
         <v/>
       </c>
       <c r="B291" s="19" t="str">
-        <f aca="false">IF(C291="","",$C$5+A291-1)</f>
+        <f aca="false">IF(C291="","",WORKDAY($C$5-1,A291))</f>
         <v/>
       </c>
       <c r="C291" s="20" t="str">
@@ -11522,7 +11528,7 @@
         <v/>
       </c>
       <c r="B292" s="19" t="str">
-        <f aca="false">IF(C292="","",$C$5+A292-1)</f>
+        <f aca="false">IF(C292="","",WORKDAY($C$5-1,A292))</f>
         <v/>
       </c>
       <c r="C292" s="20" t="str">
@@ -11559,7 +11565,7 @@
         <v/>
       </c>
       <c r="B293" s="19" t="str">
-        <f aca="false">IF(C293="","",$C$5+A293-1)</f>
+        <f aca="false">IF(C293="","",WORKDAY($C$5-1,A293))</f>
         <v/>
       </c>
       <c r="C293" s="20" t="str">
@@ -11596,7 +11602,7 @@
         <v/>
       </c>
       <c r="B294" s="19" t="str">
-        <f aca="false">IF(C294="","",$C$5+A294-1)</f>
+        <f aca="false">IF(C294="","",WORKDAY($C$5-1,A294))</f>
         <v/>
       </c>
       <c r="C294" s="20" t="str">
@@ -11633,7 +11639,7 @@
         <v/>
       </c>
       <c r="B295" s="19" t="str">
-        <f aca="false">IF(C295="","",$C$5+A295-1)</f>
+        <f aca="false">IF(C295="","",WORKDAY($C$5-1,A295))</f>
         <v/>
       </c>
       <c r="C295" s="20" t="str">
@@ -11670,7 +11676,7 @@
         <v/>
       </c>
       <c r="B296" s="19" t="str">
-        <f aca="false">IF(C296="","",$C$5+A296-1)</f>
+        <f aca="false">IF(C296="","",WORKDAY($C$5-1,A296))</f>
         <v/>
       </c>
       <c r="C296" s="20" t="str">
@@ -11707,7 +11713,7 @@
         <v/>
       </c>
       <c r="B297" s="19" t="str">
-        <f aca="false">IF(C297="","",$C$5+A297-1)</f>
+        <f aca="false">IF(C297="","",WORKDAY($C$5-1,A297))</f>
         <v/>
       </c>
       <c r="C297" s="20" t="str">
@@ -11744,7 +11750,7 @@
         <v/>
       </c>
       <c r="B298" s="19" t="str">
-        <f aca="false">IF(C298="","",$C$5+A298-1)</f>
+        <f aca="false">IF(C298="","",WORKDAY($C$5-1,A298))</f>
         <v/>
       </c>
       <c r="C298" s="20" t="str">
@@ -11781,7 +11787,7 @@
         <v/>
       </c>
       <c r="B299" s="19" t="str">
-        <f aca="false">IF(C299="","",$C$5+A299-1)</f>
+        <f aca="false">IF(C299="","",WORKDAY($C$5-1,A299))</f>
         <v/>
       </c>
       <c r="C299" s="20" t="str">
@@ -11818,7 +11824,7 @@
         <v/>
       </c>
       <c r="B300" s="19" t="str">
-        <f aca="false">IF(C300="","",$C$5+A300-1)</f>
+        <f aca="false">IF(C300="","",WORKDAY($C$5-1,A300))</f>
         <v/>
       </c>
       <c r="C300" s="20" t="str">
@@ -11855,7 +11861,7 @@
         <v/>
       </c>
       <c r="B301" s="19" t="str">
-        <f aca="false">IF(C301="","",$C$5+A301-1)</f>
+        <f aca="false">IF(C301="","",WORKDAY($C$5-1,A301))</f>
         <v/>
       </c>
       <c r="C301" s="20" t="str">
@@ -11892,7 +11898,7 @@
         <v/>
       </c>
       <c r="B302" s="19" t="str">
-        <f aca="false">IF(C302="","",$C$5+A302-1)</f>
+        <f aca="false">IF(C302="","",WORKDAY($C$5-1,A302))</f>
         <v/>
       </c>
       <c r="C302" s="20" t="str">
@@ -11929,7 +11935,7 @@
         <v/>
       </c>
       <c r="B303" s="19" t="str">
-        <f aca="false">IF(C303="","",$C$5+A303-1)</f>
+        <f aca="false">IF(C303="","",WORKDAY($C$5-1,A303))</f>
         <v/>
       </c>
       <c r="C303" s="20" t="str">
@@ -11966,7 +11972,7 @@
         <v/>
       </c>
       <c r="B304" s="19" t="str">
-        <f aca="false">IF(C304="","",$C$5+A304-1)</f>
+        <f aca="false">IF(C304="","",WORKDAY($C$5-1,A304))</f>
         <v/>
       </c>
       <c r="C304" s="20" t="str">
@@ -12003,7 +12009,7 @@
         <v/>
       </c>
       <c r="B305" s="19" t="str">
-        <f aca="false">IF(C305="","",$C$5+A305-1)</f>
+        <f aca="false">IF(C305="","",WORKDAY($C$5-1,A305))</f>
         <v/>
       </c>
       <c r="C305" s="20" t="str">
@@ -12040,7 +12046,7 @@
         <v/>
       </c>
       <c r="B306" s="19" t="str">
-        <f aca="false">IF(C306="","",$C$5+A306-1)</f>
+        <f aca="false">IF(C306="","",WORKDAY($C$5-1,A306))</f>
         <v/>
       </c>
       <c r="C306" s="20" t="str">
@@ -12077,7 +12083,7 @@
         <v/>
       </c>
       <c r="B307" s="19" t="str">
-        <f aca="false">IF(C307="","",$C$5+A307-1)</f>
+        <f aca="false">IF(C307="","",WORKDAY($C$5-1,A307))</f>
         <v/>
       </c>
       <c r="C307" s="20" t="str">
@@ -12114,7 +12120,7 @@
         <v/>
       </c>
       <c r="B308" s="19" t="str">
-        <f aca="false">IF(C308="","",$C$5+A308-1)</f>
+        <f aca="false">IF(C308="","",WORKDAY($C$5-1,A308))</f>
         <v/>
       </c>
       <c r="C308" s="20" t="str">
@@ -12151,7 +12157,7 @@
         <v/>
       </c>
       <c r="B309" s="19" t="str">
-        <f aca="false">IF(C309="","",$C$5+A309-1)</f>
+        <f aca="false">IF(C309="","",WORKDAY($C$5-1,A309))</f>
         <v/>
       </c>
       <c r="C309" s="20" t="str">
@@ -12188,7 +12194,7 @@
         <v/>
       </c>
       <c r="B310" s="19" t="str">
-        <f aca="false">IF(C310="","",$C$5+A310-1)</f>
+        <f aca="false">IF(C310="","",WORKDAY($C$5-1,A310))</f>
         <v/>
       </c>
       <c r="C310" s="20" t="str">
@@ -12225,7 +12231,7 @@
         <v/>
       </c>
       <c r="B311" s="19" t="str">
-        <f aca="false">IF(C311="","",$C$5+A311-1)</f>
+        <f aca="false">IF(C311="","",WORKDAY($C$5-1,A311))</f>
         <v/>
       </c>
       <c r="C311" s="20" t="str">
@@ -12262,7 +12268,7 @@
         <v/>
       </c>
       <c r="B312" s="19" t="str">
-        <f aca="false">IF(C312="","",$C$5+A312-1)</f>
+        <f aca="false">IF(C312="","",WORKDAY($C$5-1,A312))</f>
         <v/>
       </c>
       <c r="C312" s="20" t="str">
@@ -12299,7 +12305,7 @@
         <v/>
       </c>
       <c r="B313" s="19" t="str">
-        <f aca="false">IF(C313="","",$C$5+A313-1)</f>
+        <f aca="false">IF(C313="","",WORKDAY($C$5-1,A313))</f>
         <v/>
       </c>
       <c r="C313" s="20" t="str">
@@ -12336,7 +12342,7 @@
         <v/>
       </c>
       <c r="B314" s="19" t="str">
-        <f aca="false">IF(C314="","",$C$5+A314-1)</f>
+        <f aca="false">IF(C314="","",WORKDAY($C$5-1,A314))</f>
         <v/>
       </c>
       <c r="C314" s="20" t="str">
@@ -12373,7 +12379,7 @@
         <v/>
       </c>
       <c r="B315" s="19" t="str">
-        <f aca="false">IF(C315="","",$C$5+A315-1)</f>
+        <f aca="false">IF(C315="","",WORKDAY($C$5-1,A315))</f>
         <v/>
       </c>
       <c r="C315" s="20" t="str">
@@ -12410,7 +12416,7 @@
         <v/>
       </c>
       <c r="B316" s="19" t="str">
-        <f aca="false">IF(C316="","",$C$5+A316-1)</f>
+        <f aca="false">IF(C316="","",WORKDAY($C$5-1,A316))</f>
         <v/>
       </c>
       <c r="C316" s="20" t="str">
@@ -12447,7 +12453,7 @@
         <v/>
       </c>
       <c r="B317" s="19" t="str">
-        <f aca="false">IF(C317="","",$C$5+A317-1)</f>
+        <f aca="false">IF(C317="","",WORKDAY($C$5-1,A317))</f>
         <v/>
       </c>
       <c r="C317" s="20" t="str">
@@ -12484,7 +12490,7 @@
         <v/>
       </c>
       <c r="B318" s="19" t="str">
-        <f aca="false">IF(C318="","",$C$5+A318-1)</f>
+        <f aca="false">IF(C318="","",WORKDAY($C$5-1,A318))</f>
         <v/>
       </c>
       <c r="C318" s="20" t="str">
@@ -12521,7 +12527,7 @@
         <v/>
       </c>
       <c r="B319" s="19" t="str">
-        <f aca="false">IF(C319="","",$C$5+A319-1)</f>
+        <f aca="false">IF(C319="","",WORKDAY($C$5-1,A319))</f>
         <v/>
       </c>
       <c r="C319" s="20" t="str">
@@ -12558,7 +12564,7 @@
         <v/>
       </c>
       <c r="B320" s="19" t="str">
-        <f aca="false">IF(C320="","",$C$5+A320-1)</f>
+        <f aca="false">IF(C320="","",WORKDAY($C$5-1,A320))</f>
         <v/>
       </c>
       <c r="C320" s="20" t="str">
@@ -12595,7 +12601,7 @@
         <v/>
       </c>
       <c r="B321" s="19" t="str">
-        <f aca="false">IF(C321="","",$C$5+A321-1)</f>
+        <f aca="false">IF(C321="","",WORKDAY($C$5-1,A321))</f>
         <v/>
       </c>
       <c r="C321" s="20" t="str">
@@ -12632,7 +12638,7 @@
         <v/>
       </c>
       <c r="B322" s="19" t="str">
-        <f aca="false">IF(C322="","",$C$5+A322-1)</f>
+        <f aca="false">IF(C322="","",WORKDAY($C$5-1,A322))</f>
         <v/>
       </c>
       <c r="C322" s="20" t="str">
@@ -12669,7 +12675,7 @@
         <v/>
       </c>
       <c r="B323" s="19" t="str">
-        <f aca="false">IF(C323="","",$C$5+A323-1)</f>
+        <f aca="false">IF(C323="","",WORKDAY($C$5-1,A323))</f>
         <v/>
       </c>
       <c r="C323" s="20" t="str">
@@ -12706,7 +12712,7 @@
         <v/>
       </c>
       <c r="B324" s="19" t="str">
-        <f aca="false">IF(C324="","",$C$5+A324-1)</f>
+        <f aca="false">IF(C324="","",WORKDAY($C$5-1,A324))</f>
         <v/>
       </c>
       <c r="C324" s="20" t="str">
@@ -12743,7 +12749,7 @@
         <v/>
       </c>
       <c r="B325" s="19" t="str">
-        <f aca="false">IF(C325="","",$C$5+A325-1)</f>
+        <f aca="false">IF(C325="","",WORKDAY($C$5-1,A325))</f>
         <v/>
       </c>
       <c r="C325" s="20" t="str">
@@ -12780,7 +12786,7 @@
         <v/>
       </c>
       <c r="B326" s="19" t="str">
-        <f aca="false">IF(C326="","",$C$5+A326-1)</f>
+        <f aca="false">IF(C326="","",WORKDAY($C$5-1,A326))</f>
         <v/>
       </c>
       <c r="C326" s="20" t="str">
@@ -12817,7 +12823,7 @@
         <v/>
       </c>
       <c r="B327" s="19" t="str">
-        <f aca="false">IF(C327="","",$C$5+A327-1)</f>
+        <f aca="false">IF(C327="","",WORKDAY($C$5-1,A327))</f>
         <v/>
       </c>
       <c r="C327" s="20" t="str">
@@ -12854,7 +12860,7 @@
         <v/>
       </c>
       <c r="B328" s="19" t="str">
-        <f aca="false">IF(C328="","",$C$5+A328-1)</f>
+        <f aca="false">IF(C328="","",WORKDAY($C$5-1,A328))</f>
         <v/>
       </c>
       <c r="C328" s="20" t="str">
@@ -12891,7 +12897,7 @@
         <v/>
       </c>
       <c r="B329" s="19" t="str">
-        <f aca="false">IF(C329="","",$C$5+A329-1)</f>
+        <f aca="false">IF(C329="","",WORKDAY($C$5-1,A329))</f>
         <v/>
       </c>
       <c r="C329" s="20" t="str">
@@ -12928,7 +12934,7 @@
         <v/>
       </c>
       <c r="B330" s="19" t="str">
-        <f aca="false">IF(C330="","",$C$5+A330-1)</f>
+        <f aca="false">IF(C330="","",WORKDAY($C$5-1,A330))</f>
         <v/>
       </c>
       <c r="C330" s="20" t="str">
@@ -12965,7 +12971,7 @@
         <v/>
       </c>
       <c r="B331" s="19" t="str">
-        <f aca="false">IF(C331="","",$C$5+A331-1)</f>
+        <f aca="false">IF(C331="","",WORKDAY($C$5-1,A331))</f>
         <v/>
       </c>
       <c r="C331" s="20" t="str">
@@ -13002,7 +13008,7 @@
         <v/>
       </c>
       <c r="B332" s="19" t="str">
-        <f aca="false">IF(C332="","",$C$5+A332-1)</f>
+        <f aca="false">IF(C332="","",WORKDAY($C$5-1,A332))</f>
         <v/>
       </c>
       <c r="C332" s="20" t="str">
@@ -13039,7 +13045,7 @@
         <v/>
       </c>
       <c r="B333" s="19" t="str">
-        <f aca="false">IF(C333="","",$C$5+A333-1)</f>
+        <f aca="false">IF(C333="","",WORKDAY($C$5-1,A333))</f>
         <v/>
       </c>
       <c r="C333" s="20" t="str">
@@ -13076,7 +13082,7 @@
         <v/>
       </c>
       <c r="B334" s="19" t="str">
-        <f aca="false">IF(C334="","",$C$5+A334-1)</f>
+        <f aca="false">IF(C334="","",WORKDAY($C$5-1,A334))</f>
         <v/>
       </c>
       <c r="C334" s="20" t="str">
@@ -13113,7 +13119,7 @@
         <v/>
       </c>
       <c r="B335" s="19" t="str">
-        <f aca="false">IF(C335="","",$C$5+A335-1)</f>
+        <f aca="false">IF(C335="","",WORKDAY($C$5-1,A335))</f>
         <v/>
       </c>
       <c r="C335" s="20" t="str">
@@ -13150,7 +13156,7 @@
         <v/>
       </c>
       <c r="B336" s="19" t="str">
-        <f aca="false">IF(C336="","",$C$5+A336-1)</f>
+        <f aca="false">IF(C336="","",WORKDAY($C$5-1,A336))</f>
         <v/>
       </c>
       <c r="C336" s="20" t="str">
@@ -13187,7 +13193,7 @@
         <v/>
       </c>
       <c r="B337" s="19" t="str">
-        <f aca="false">IF(C337="","",$C$5+A337-1)</f>
+        <f aca="false">IF(C337="","",WORKDAY($C$5-1,A337))</f>
         <v/>
       </c>
       <c r="C337" s="20" t="str">
@@ -13224,7 +13230,7 @@
         <v/>
       </c>
       <c r="B338" s="19" t="str">
-        <f aca="false">IF(C338="","",$C$5+A338-1)</f>
+        <f aca="false">IF(C338="","",WORKDAY($C$5-1,A338))</f>
         <v/>
       </c>
       <c r="C338" s="20" t="str">
@@ -13261,7 +13267,7 @@
         <v/>
       </c>
       <c r="B339" s="19" t="str">
-        <f aca="false">IF(C339="","",$C$5+A339-1)</f>
+        <f aca="false">IF(C339="","",WORKDAY($C$5-1,A339))</f>
         <v/>
       </c>
       <c r="C339" s="20" t="str">
@@ -13298,7 +13304,7 @@
         <v/>
       </c>
       <c r="B340" s="19" t="str">
-        <f aca="false">IF(C340="","",$C$5+A340-1)</f>
+        <f aca="false">IF(C340="","",WORKDAY($C$5-1,A340))</f>
         <v/>
       </c>
       <c r="C340" s="20" t="str">
@@ -13335,7 +13341,7 @@
         <v/>
       </c>
       <c r="B341" s="19" t="str">
-        <f aca="false">IF(C341="","",$C$5+A341-1)</f>
+        <f aca="false">IF(C341="","",WORKDAY($C$5-1,A341))</f>
         <v/>
       </c>
       <c r="C341" s="20" t="str">
@@ -13372,7 +13378,7 @@
         <v/>
       </c>
       <c r="B342" s="19" t="str">
-        <f aca="false">IF(C342="","",$C$5+A342-1)</f>
+        <f aca="false">IF(C342="","",WORKDAY($C$5-1,A342))</f>
         <v/>
       </c>
       <c r="C342" s="20" t="str">
@@ -13409,7 +13415,7 @@
         <v/>
       </c>
       <c r="B343" s="19" t="str">
-        <f aca="false">IF(C343="","",$C$5+A343-1)</f>
+        <f aca="false">IF(C343="","",WORKDAY($C$5-1,A343))</f>
         <v/>
       </c>
       <c r="C343" s="20" t="str">
@@ -13446,7 +13452,7 @@
         <v/>
       </c>
       <c r="B344" s="19" t="str">
-        <f aca="false">IF(C344="","",$C$5+A344-1)</f>
+        <f aca="false">IF(C344="","",WORKDAY($C$5-1,A344))</f>
         <v/>
       </c>
       <c r="C344" s="20" t="str">
@@ -13483,7 +13489,7 @@
         <v/>
       </c>
       <c r="B345" s="19" t="str">
-        <f aca="false">IF(C345="","",$C$5+A345-1)</f>
+        <f aca="false">IF(C345="","",WORKDAY($C$5-1,A345))</f>
         <v/>
       </c>
       <c r="C345" s="20" t="str">
@@ -13520,7 +13526,7 @@
         <v/>
       </c>
       <c r="B346" s="19" t="str">
-        <f aca="false">IF(C346="","",$C$5+A346-1)</f>
+        <f aca="false">IF(C346="","",WORKDAY($C$5-1,A346))</f>
         <v/>
       </c>
       <c r="C346" s="20" t="str">
@@ -13557,7 +13563,7 @@
         <v/>
       </c>
       <c r="B347" s="19" t="str">
-        <f aca="false">IF(C347="","",$C$5+A347-1)</f>
+        <f aca="false">IF(C347="","",WORKDAY($C$5-1,A347))</f>
         <v/>
       </c>
       <c r="C347" s="20" t="str">
@@ -13594,7 +13600,7 @@
         <v/>
       </c>
       <c r="B348" s="19" t="str">
-        <f aca="false">IF(C348="","",$C$5+A348-1)</f>
+        <f aca="false">IF(C348="","",WORKDAY($C$5-1,A348))</f>
         <v/>
       </c>
       <c r="C348" s="20" t="str">
@@ -13631,7 +13637,7 @@
         <v/>
       </c>
       <c r="B349" s="19" t="str">
-        <f aca="false">IF(C349="","",$C$5+A349-1)</f>
+        <f aca="false">IF(C349="","",WORKDAY($C$5-1,A349))</f>
         <v/>
       </c>
       <c r="C349" s="20" t="str">
@@ -13668,7 +13674,7 @@
         <v/>
       </c>
       <c r="B350" s="19" t="str">
-        <f aca="false">IF(C350="","",$C$5+A350-1)</f>
+        <f aca="false">IF(C350="","",WORKDAY($C$5-1,A350))</f>
         <v/>
       </c>
       <c r="C350" s="20" t="str">
@@ -13705,7 +13711,7 @@
         <v/>
       </c>
       <c r="B351" s="19" t="str">
-        <f aca="false">IF(C351="","",$C$5+A351-1)</f>
+        <f aca="false">IF(C351="","",WORKDAY($C$5-1,A351))</f>
         <v/>
       </c>
       <c r="C351" s="20" t="str">
@@ -13742,7 +13748,7 @@
         <v/>
       </c>
       <c r="B352" s="19" t="str">
-        <f aca="false">IF(C352="","",$C$5+A352-1)</f>
+        <f aca="false">IF(C352="","",WORKDAY($C$5-1,A352))</f>
         <v/>
       </c>
       <c r="C352" s="20" t="str">
@@ -13779,7 +13785,7 @@
         <v/>
       </c>
       <c r="B353" s="19" t="str">
-        <f aca="false">IF(C353="","",$C$5+A353-1)</f>
+        <f aca="false">IF(C353="","",WORKDAY($C$5-1,A353))</f>
         <v/>
       </c>
       <c r="C353" s="20" t="str">
@@ -13816,7 +13822,7 @@
         <v/>
       </c>
       <c r="B354" s="19" t="str">
-        <f aca="false">IF(C354="","",$C$5+A354-1)</f>
+        <f aca="false">IF(C354="","",WORKDAY($C$5-1,A354))</f>
         <v/>
       </c>
       <c r="C354" s="20" t="str">
@@ -13853,7 +13859,7 @@
         <v/>
       </c>
       <c r="B355" s="19" t="str">
-        <f aca="false">IF(C355="","",$C$5+A355-1)</f>
+        <f aca="false">IF(C355="","",WORKDAY($C$5-1,A355))</f>
         <v/>
       </c>
       <c r="C355" s="20" t="str">
@@ -13890,7 +13896,7 @@
         <v/>
       </c>
       <c r="B356" s="19" t="str">
-        <f aca="false">IF(C356="","",$C$5+A356-1)</f>
+        <f aca="false">IF(C356="","",WORKDAY($C$5-1,A356))</f>
         <v/>
       </c>
       <c r="C356" s="20" t="str">
@@ -13927,7 +13933,7 @@
         <v/>
       </c>
       <c r="B357" s="19" t="str">
-        <f aca="false">IF(C357="","",$C$5+A357-1)</f>
+        <f aca="false">IF(C357="","",WORKDAY($C$5-1,A357))</f>
         <v/>
       </c>
       <c r="C357" s="20" t="str">
@@ -13964,7 +13970,7 @@
         <v/>
       </c>
       <c r="B358" s="19" t="str">
-        <f aca="false">IF(C358="","",$C$5+A358-1)</f>
+        <f aca="false">IF(C358="","",WORKDAY($C$5-1,A358))</f>
         <v/>
       </c>
       <c r="C358" s="20" t="str">
@@ -14001,7 +14007,7 @@
         <v/>
       </c>
       <c r="B359" s="19" t="str">
-        <f aca="false">IF(C359="","",$C$5+A359-1)</f>
+        <f aca="false">IF(C359="","",WORKDAY($C$5-1,A359))</f>
         <v/>
       </c>
       <c r="C359" s="20" t="str">
@@ -14038,7 +14044,7 @@
         <v/>
       </c>
       <c r="B360" s="19" t="str">
-        <f aca="false">IF(C360="","",$C$5+A360-1)</f>
+        <f aca="false">IF(C360="","",WORKDAY($C$5-1,A360))</f>
         <v/>
       </c>
       <c r="C360" s="20" t="str">
@@ -14075,7 +14081,7 @@
         <v/>
       </c>
       <c r="B361" s="19" t="str">
-        <f aca="false">IF(C361="","",$C$5+A361-1)</f>
+        <f aca="false">IF(C361="","",WORKDAY($C$5-1,A361))</f>
         <v/>
       </c>
       <c r="C361" s="20" t="str">
@@ -14112,7 +14118,7 @@
         <v/>
       </c>
       <c r="B362" s="19" t="str">
-        <f aca="false">IF(C362="","",$C$5+A362-1)</f>
+        <f aca="false">IF(C362="","",WORKDAY($C$5-1,A362))</f>
         <v/>
       </c>
       <c r="C362" s="20" t="str">
@@ -14149,7 +14155,7 @@
         <v/>
       </c>
       <c r="B363" s="19" t="str">
-        <f aca="false">IF(C363="","",$C$5+A363-1)</f>
+        <f aca="false">IF(C363="","",WORKDAY($C$5-1,A363))</f>
         <v/>
       </c>
       <c r="C363" s="20" t="str">
@@ -14186,7 +14192,7 @@
         <v/>
       </c>
       <c r="B364" s="19" t="str">
-        <f aca="false">IF(C364="","",$C$5+A364-1)</f>
+        <f aca="false">IF(C364="","",WORKDAY($C$5-1,A364))</f>
         <v/>
       </c>
       <c r="C364" s="20" t="str">
@@ -14223,7 +14229,7 @@
         <v/>
       </c>
       <c r="B365" s="19" t="str">
-        <f aca="false">IF(C365="","",$C$5+A365-1)</f>
+        <f aca="false">IF(C365="","",WORKDAY($C$5-1,A365))</f>
         <v/>
       </c>
       <c r="C365" s="20" t="str">
@@ -14260,7 +14266,7 @@
         <v/>
       </c>
       <c r="B366" s="19" t="str">
-        <f aca="false">IF(C366="","",$C$5+A366-1)</f>
+        <f aca="false">IF(C366="","",WORKDAY($C$5-1,A366))</f>
         <v/>
       </c>
       <c r="C366" s="20" t="str">
@@ -14297,7 +14303,7 @@
         <v/>
       </c>
       <c r="B367" s="19" t="str">
-        <f aca="false">IF(C367="","",$C$5+A367-1)</f>
+        <f aca="false">IF(C367="","",WORKDAY($C$5-1,A367))</f>
         <v/>
       </c>
       <c r="C367" s="20" t="str">
@@ -14334,7 +14340,7 @@
         <v/>
       </c>
       <c r="B368" s="19" t="str">
-        <f aca="false">IF(C368="","",$C$5+A368-1)</f>
+        <f aca="false">IF(C368="","",WORKDAY($C$5-1,A368))</f>
         <v/>
       </c>
       <c r="C368" s="20" t="str">
@@ -14371,7 +14377,7 @@
         <v/>
       </c>
       <c r="B369" s="19" t="str">
-        <f aca="false">IF(C369="","",$C$5+A369-1)</f>
+        <f aca="false">IF(C369="","",WORKDAY($C$5-1,A369))</f>
         <v/>
       </c>
       <c r="C369" s="20" t="str">
@@ -14408,7 +14414,7 @@
         <v/>
       </c>
       <c r="B370" s="19" t="str">
-        <f aca="false">IF(C370="","",$C$5+A370-1)</f>
+        <f aca="false">IF(C370="","",WORKDAY($C$5-1,A370))</f>
         <v/>
       </c>
       <c r="C370" s="20" t="str">
@@ -14445,7 +14451,7 @@
         <v/>
       </c>
       <c r="B371" s="19" t="str">
-        <f aca="false">IF(C371="","",$C$5+A371-1)</f>
+        <f aca="false">IF(C371="","",WORKDAY($C$5-1,A371))</f>
         <v/>
       </c>
       <c r="C371" s="20" t="str">
@@ -14482,7 +14488,7 @@
         <v/>
       </c>
       <c r="B372" s="19" t="str">
-        <f aca="false">IF(C372="","",$C$5+A372-1)</f>
+        <f aca="false">IF(C372="","",WORKDAY($C$5-1,A372))</f>
         <v/>
       </c>
       <c r="C372" s="20" t="str">
@@ -14519,7 +14525,7 @@
         <v/>
       </c>
       <c r="B373" s="19" t="str">
-        <f aca="false">IF(C373="","",$C$5+A373-1)</f>
+        <f aca="false">IF(C373="","",WORKDAY($C$5-1,A373))</f>
         <v/>
       </c>
       <c r="C373" s="20" t="str">
@@ -14556,7 +14562,7 @@
         <v/>
       </c>
       <c r="B374" s="19" t="str">
-        <f aca="false">IF(C374="","",$C$5+A374-1)</f>
+        <f aca="false">IF(C374="","",WORKDAY($C$5-1,A374))</f>
         <v/>
       </c>
       <c r="C374" s="20" t="str">
@@ -14593,7 +14599,7 @@
         <v/>
       </c>
       <c r="B375" s="19" t="str">
-        <f aca="false">IF(C375="","",$C$5+A375-1)</f>
+        <f aca="false">IF(C375="","",WORKDAY($C$5-1,A375))</f>
         <v/>
       </c>
       <c r="C375" s="20" t="str">
@@ -14630,7 +14636,7 @@
         <v/>
       </c>
       <c r="B376" s="19" t="str">
-        <f aca="false">IF(C376="","",$C$5+A376-1)</f>
+        <f aca="false">IF(C376="","",WORKDAY($C$5-1,A376))</f>
         <v/>
       </c>
       <c r="C376" s="20" t="str">
@@ -14667,7 +14673,7 @@
         <v/>
       </c>
       <c r="B377" s="19" t="str">
-        <f aca="false">IF(C377="","",$C$5+A377-1)</f>
+        <f aca="false">IF(C377="","",WORKDAY($C$5-1,A377))</f>
         <v/>
       </c>
       <c r="C377" s="20" t="str">
@@ -14704,7 +14710,7 @@
         <v/>
       </c>
       <c r="B378" s="19" t="str">
-        <f aca="false">IF(C378="","",$C$5+A378-1)</f>
+        <f aca="false">IF(C378="","",WORKDAY($C$5-1,A378))</f>
         <v/>
       </c>
       <c r="C378" s="20" t="str">
@@ -14741,7 +14747,7 @@
         <v/>
       </c>
       <c r="B379" s="19" t="str">
-        <f aca="false">IF(C379="","",$C$5+A379-1)</f>
+        <f aca="false">IF(C379="","",WORKDAY($C$5-1,A379))</f>
         <v/>
       </c>
       <c r="C379" s="20" t="str">
@@ -14778,7 +14784,7 @@
         <v/>
       </c>
       <c r="B380" s="19" t="str">
-        <f aca="false">IF(C380="","",$C$5+A380-1)</f>
+        <f aca="false">IF(C380="","",WORKDAY($C$5-1,A380))</f>
         <v/>
       </c>
       <c r="C380" s="20" t="str">
@@ -14815,7 +14821,7 @@
         <v/>
       </c>
       <c r="B381" s="19" t="str">
-        <f aca="false">IF(C381="","",$C$5+A381-1)</f>
+        <f aca="false">IF(C381="","",WORKDAY($C$5-1,A381))</f>
         <v/>
       </c>
       <c r="C381" s="20" t="str">
@@ -14852,7 +14858,7 @@
         <v/>
       </c>
       <c r="B382" s="19" t="str">
-        <f aca="false">IF(C382="","",$C$5+A382-1)</f>
+        <f aca="false">IF(C382="","",WORKDAY($C$5-1,A382))</f>
         <v/>
       </c>
       <c r="C382" s="20" t="str">
@@ -14889,7 +14895,7 @@
         <v/>
       </c>
       <c r="B383" s="19" t="str">
-        <f aca="false">IF(C383="","",$C$5+A383-1)</f>
+        <f aca="false">IF(C383="","",WORKDAY($C$5-1,A383))</f>
         <v/>
       </c>
       <c r="C383" s="20" t="str">
@@ -14926,7 +14932,7 @@
         <v/>
       </c>
       <c r="B384" s="19" t="str">
-        <f aca="false">IF(C384="","",$C$5+A384-1)</f>
+        <f aca="false">IF(C384="","",WORKDAY($C$5-1,A384))</f>
         <v/>
       </c>
       <c r="C384" s="20" t="str">
@@ -14963,7 +14969,7 @@
         <v/>
       </c>
       <c r="B385" s="19" t="str">
-        <f aca="false">IF(C385="","",$C$5+A385-1)</f>
+        <f aca="false">IF(C385="","",WORKDAY($C$5-1,A385))</f>
         <v/>
       </c>
       <c r="C385" s="20" t="str">
@@ -15000,7 +15006,7 @@
         <v/>
       </c>
       <c r="B386" s="19" t="str">
-        <f aca="false">IF(C386="","",$C$5+A386-1)</f>
+        <f aca="false">IF(C386="","",WORKDAY($C$5-1,A386))</f>
         <v/>
       </c>
       <c r="C386" s="20" t="str">
@@ -15037,7 +15043,7 @@
         <v/>
       </c>
       <c r="B387" s="19" t="str">
-        <f aca="false">IF(C387="","",$C$5+A387-1)</f>
+        <f aca="false">IF(C387="","",WORKDAY($C$5-1,A387))</f>
         <v/>
       </c>
       <c r="C387" s="20" t="str">
@@ -15074,7 +15080,7 @@
         <v/>
       </c>
       <c r="B388" s="19" t="str">
-        <f aca="false">IF(C388="","",$C$5+A388-1)</f>
+        <f aca="false">IF(C388="","",WORKDAY($C$5-1,A388))</f>
         <v/>
       </c>
       <c r="C388" s="20" t="str">
@@ -15111,7 +15117,7 @@
         <v/>
       </c>
       <c r="B389" s="19" t="str">
-        <f aca="false">IF(C389="","",$C$5+A389-1)</f>
+        <f aca="false">IF(C389="","",WORKDAY($C$5-1,A389))</f>
         <v/>
       </c>
       <c r="C389" s="20" t="str">
@@ -15148,7 +15154,7 @@
         <v/>
       </c>
       <c r="B390" s="19" t="str">
-        <f aca="false">IF(C390="","",$C$5+A390-1)</f>
+        <f aca="false">IF(C390="","",WORKDAY($C$5-1,A390))</f>
         <v/>
       </c>
       <c r="C390" s="20" t="str">
@@ -15185,7 +15191,7 @@
         <v/>
       </c>
       <c r="B391" s="19" t="str">
-        <f aca="false">IF(C391="","",$C$5+A391-1)</f>
+        <f aca="false">IF(C391="","",WORKDAY($C$5-1,A391))</f>
         <v/>
       </c>
       <c r="C391" s="20" t="str">
@@ -15222,7 +15228,7 @@
         <v/>
       </c>
       <c r="B392" s="19" t="str">
-        <f aca="false">IF(C392="","",$C$5+A392-1)</f>
+        <f aca="false">IF(C392="","",WORKDAY($C$5-1,A392))</f>
         <v/>
       </c>
       <c r="C392" s="20" t="str">
@@ -15259,7 +15265,7 @@
         <v/>
       </c>
       <c r="B393" s="19" t="str">
-        <f aca="false">IF(C393="","",$C$5+A393-1)</f>
+        <f aca="false">IF(C393="","",WORKDAY($C$5-1,A393))</f>
         <v/>
       </c>
       <c r="C393" s="20" t="str">
@@ -15296,7 +15302,7 @@
         <v/>
       </c>
       <c r="B394" s="19" t="str">
-        <f aca="false">IF(C394="","",$C$5+A394-1)</f>
+        <f aca="false">IF(C394="","",WORKDAY($C$5-1,A394))</f>
         <v/>
       </c>
       <c r="C394" s="20" t="str">
@@ -15333,7 +15339,7 @@
         <v/>
       </c>
       <c r="B395" s="19" t="str">
-        <f aca="false">IF(C395="","",$C$5+A395-1)</f>
+        <f aca="false">IF(C395="","",WORKDAY($C$5-1,A395))</f>
         <v/>
       </c>
       <c r="C395" s="20" t="str">
@@ -15370,7 +15376,7 @@
         <v/>
       </c>
       <c r="B396" s="19" t="str">
-        <f aca="false">IF(C396="","",$C$5+A396-1)</f>
+        <f aca="false">IF(C396="","",WORKDAY($C$5-1,A396))</f>
         <v/>
       </c>
       <c r="C396" s="20" t="str">
@@ -15407,7 +15413,7 @@
         <v/>
       </c>
       <c r="B397" s="19" t="str">
-        <f aca="false">IF(C397="","",$C$5+A397-1)</f>
+        <f aca="false">IF(C397="","",WORKDAY($C$5-1,A397))</f>
         <v/>
       </c>
       <c r="C397" s="20" t="str">
@@ -15444,7 +15450,7 @@
         <v/>
       </c>
       <c r="B398" s="19" t="str">
-        <f aca="false">IF(C398="","",$C$5+A398-1)</f>
+        <f aca="false">IF(C398="","",WORKDAY($C$5-1,A398))</f>
         <v/>
       </c>
       <c r="C398" s="20" t="str">
@@ -15481,7 +15487,7 @@
         <v/>
       </c>
       <c r="B399" s="19" t="str">
-        <f aca="false">IF(C399="","",$C$5+A399-1)</f>
+        <f aca="false">IF(C399="","",WORKDAY($C$5-1,A399))</f>
         <v/>
       </c>
       <c r="C399" s="20" t="str">
@@ -15518,7 +15524,7 @@
         <v/>
       </c>
       <c r="B400" s="19" t="str">
-        <f aca="false">IF(C400="","",$C$5+A400-1)</f>
+        <f aca="false">IF(C400="","",WORKDAY($C$5-1,A400))</f>
         <v/>
       </c>
       <c r="C400" s="20" t="str">
@@ -15555,7 +15561,7 @@
         <v/>
       </c>
       <c r="B401" s="19" t="str">
-        <f aca="false">IF(C401="","",$C$5+A401-1)</f>
+        <f aca="false">IF(C401="","",WORKDAY($C$5-1,A401))</f>
         <v/>
       </c>
       <c r="C401" s="20" t="str">
@@ -15592,7 +15598,7 @@
         <v/>
       </c>
       <c r="B402" s="19" t="str">
-        <f aca="false">IF(C402="","",$C$5+A402-1)</f>
+        <f aca="false">IF(C402="","",WORKDAY($C$5-1,A402))</f>
         <v/>
       </c>
       <c r="C402" s="20" t="str">
@@ -15629,7 +15635,7 @@
         <v/>
       </c>
       <c r="B403" s="19" t="str">
-        <f aca="false">IF(C403="","",$C$5+A403-1)</f>
+        <f aca="false">IF(C403="","",WORKDAY($C$5-1,A403))</f>
         <v/>
       </c>
       <c r="C403" s="20" t="str">
@@ -15666,7 +15672,7 @@
         <v/>
       </c>
       <c r="B404" s="19" t="str">
-        <f aca="false">IF(C404="","",$C$5+A404-1)</f>
+        <f aca="false">IF(C404="","",WORKDAY($C$5-1,A404))</f>
         <v/>
       </c>
       <c r="C404" s="20" t="str">
@@ -15703,7 +15709,7 @@
         <v/>
       </c>
       <c r="B405" s="19" t="str">
-        <f aca="false">IF(C405="","",$C$5+A405-1)</f>
+        <f aca="false">IF(C405="","",WORKDAY($C$5-1,A405))</f>
         <v/>
       </c>
       <c r="C405" s="20" t="str">
@@ -15740,7 +15746,7 @@
         <v/>
       </c>
       <c r="B406" s="19" t="str">
-        <f aca="false">IF(C406="","",$C$5+A406-1)</f>
+        <f aca="false">IF(C406="","",WORKDAY($C$5-1,A406))</f>
         <v/>
       </c>
       <c r="C406" s="20" t="str">
@@ -15777,7 +15783,7 @@
         <v/>
       </c>
       <c r="B407" s="19" t="str">
-        <f aca="false">IF(C407="","",$C$5+A407-1)</f>
+        <f aca="false">IF(C407="","",WORKDAY($C$5-1,A407))</f>
         <v/>
       </c>
       <c r="C407" s="20" t="str">
@@ -15814,7 +15820,7 @@
         <v/>
       </c>
       <c r="B408" s="19" t="str">
-        <f aca="false">IF(C408="","",$C$5+A408-1)</f>
+        <f aca="false">IF(C408="","",WORKDAY($C$5-1,A408))</f>
         <v/>
       </c>
       <c r="C408" s="20" t="str">
@@ -15851,7 +15857,7 @@
         <v/>
       </c>
       <c r="B409" s="19" t="str">
-        <f aca="false">IF(C409="","",$C$5+A409-1)</f>
+        <f aca="false">IF(C409="","",WORKDAY($C$5-1,A409))</f>
         <v/>
       </c>
       <c r="C409" s="20" t="str">
@@ -15888,7 +15894,7 @@
         <v/>
       </c>
       <c r="B410" s="19" t="str">
-        <f aca="false">IF(C410="","",$C$5+A410-1)</f>
+        <f aca="false">IF(C410="","",WORKDAY($C$5-1,A410))</f>
         <v/>
       </c>
       <c r="C410" s="20" t="str">
@@ -15925,7 +15931,7 @@
         <v/>
       </c>
       <c r="B411" s="19" t="str">
-        <f aca="false">IF(C411="","",$C$5+A411-1)</f>
+        <f aca="false">IF(C411="","",WORKDAY($C$5-1,A411))</f>
         <v/>
       </c>
       <c r="C411" s="20" t="str">
@@ -15962,7 +15968,7 @@
         <v/>
       </c>
       <c r="B412" s="19" t="str">
-        <f aca="false">IF(C412="","",$C$5+A412-1)</f>
+        <f aca="false">IF(C412="","",WORKDAY($C$5-1,A412))</f>
         <v/>
       </c>
       <c r="C412" s="20" t="str">
@@ -15999,7 +16005,7 @@
         <v/>
       </c>
       <c r="B413" s="19" t="str">
-        <f aca="false">IF(C413="","",$C$5+A413-1)</f>
+        <f aca="false">IF(C413="","",WORKDAY($C$5-1,A413))</f>
         <v/>
       </c>
       <c r="C413" s="20" t="str">
@@ -16036,7 +16042,7 @@
         <v/>
       </c>
       <c r="B414" s="19" t="str">
-        <f aca="false">IF(C414="","",$C$5+A414-1)</f>
+        <f aca="false">IF(C414="","",WORKDAY($C$5-1,A414))</f>
         <v/>
       </c>
       <c r="C414" s="20" t="str">
@@ -16073,7 +16079,7 @@
         <v/>
       </c>
       <c r="B415" s="19" t="str">
-        <f aca="false">IF(C415="","",$C$5+A415-1)</f>
+        <f aca="false">IF(C415="","",WORKDAY($C$5-1,A415))</f>
         <v/>
       </c>
       <c r="C415" s="20" t="str">
@@ -16110,7 +16116,7 @@
         <v/>
       </c>
       <c r="B416" s="19" t="str">
-        <f aca="false">IF(C416="","",$C$5+A416-1)</f>
+        <f aca="false">IF(C416="","",WORKDAY($C$5-1,A416))</f>
         <v/>
       </c>
       <c r="C416" s="20" t="str">
@@ -16147,7 +16153,7 @@
         <v/>
       </c>
       <c r="B417" s="19" t="str">
-        <f aca="false">IF(C417="","",$C$5+A417-1)</f>
+        <f aca="false">IF(C417="","",WORKDAY($C$5-1,A417))</f>
         <v/>
       </c>
       <c r="C417" s="20" t="str">
@@ -16184,7 +16190,7 @@
         <v/>
       </c>
       <c r="B418" s="19" t="str">
-        <f aca="false">IF(C418="","",$C$5+A418-1)</f>
+        <f aca="false">IF(C418="","",WORKDAY($C$5-1,A418))</f>
         <v/>
       </c>
       <c r="C418" s="20" t="str">
@@ -16221,7 +16227,7 @@
         <v/>
       </c>
       <c r="B419" s="19" t="str">
-        <f aca="false">IF(C419="","",$C$5+A419-1)</f>
+        <f aca="false">IF(C419="","",WORKDAY($C$5-1,A419))</f>
         <v/>
       </c>
       <c r="C419" s="20" t="str">
@@ -16258,7 +16264,7 @@
         <v/>
       </c>
       <c r="B420" s="19" t="str">
-        <f aca="false">IF(C420="","",$C$5+A420-1)</f>
+        <f aca="false">IF(C420="","",WORKDAY($C$5-1,A420))</f>
         <v/>
       </c>
       <c r="C420" s="20" t="str">
@@ -16295,7 +16301,7 @@
         <v/>
       </c>
       <c r="B421" s="19" t="str">
-        <f aca="false">IF(C421="","",$C$5+A421-1)</f>
+        <f aca="false">IF(C421="","",WORKDAY($C$5-1,A421))</f>
         <v/>
       </c>
       <c r="C421" s="20" t="str">
@@ -16332,7 +16338,7 @@
         <v/>
       </c>
       <c r="B422" s="19" t="str">
-        <f aca="false">IF(C422="","",$C$5+A422-1)</f>
+        <f aca="false">IF(C422="","",WORKDAY($C$5-1,A422))</f>
         <v/>
       </c>
       <c r="C422" s="20" t="str">
@@ -16369,7 +16375,7 @@
         <v/>
       </c>
       <c r="B423" s="19" t="str">
-        <f aca="false">IF(C423="","",$C$5+A423-1)</f>
+        <f aca="false">IF(C423="","",WORKDAY($C$5-1,A423))</f>
         <v/>
       </c>
       <c r="C423" s="20" t="str">
@@ -16406,7 +16412,7 @@
         <v/>
       </c>
       <c r="B424" s="19" t="str">
-        <f aca="false">IF(C424="","",$C$5+A424-1)</f>
+        <f aca="false">IF(C424="","",WORKDAY($C$5-1,A424))</f>
         <v/>
       </c>
       <c r="C424" s="20" t="str">
@@ -16443,7 +16449,7 @@
         <v/>
       </c>
       <c r="B425" s="19" t="str">
-        <f aca="false">IF(C425="","",$C$5+A425-1)</f>
+        <f aca="false">IF(C425="","",WORKDAY($C$5-1,A425))</f>
         <v/>
       </c>
       <c r="C425" s="20" t="str">
@@ -16480,7 +16486,7 @@
         <v/>
       </c>
       <c r="B426" s="19" t="str">
-        <f aca="false">IF(C426="","",$C$5+A426-1)</f>
+        <f aca="false">IF(C426="","",WORKDAY($C$5-1,A426))</f>
         <v/>
       </c>
       <c r="C426" s="20" t="str">
@@ -16517,7 +16523,7 @@
         <v/>
       </c>
       <c r="B427" s="19" t="str">
-        <f aca="false">IF(C427="","",$C$5+A427-1)</f>
+        <f aca="false">IF(C427="","",WORKDAY($C$5-1,A427))</f>
         <v/>
       </c>
       <c r="C427" s="20" t="str">
@@ -16554,7 +16560,7 @@
         <v/>
       </c>
       <c r="B428" s="19" t="str">
-        <f aca="false">IF(C428="","",$C$5+A428-1)</f>
+        <f aca="false">IF(C428="","",WORKDAY($C$5-1,A428))</f>
         <v/>
       </c>
       <c r="C428" s="20" t="str">
@@ -16591,7 +16597,7 @@
         <v/>
       </c>
       <c r="B429" s="19" t="str">
-        <f aca="false">IF(C429="","",$C$5+A429-1)</f>
+        <f aca="false">IF(C429="","",WORKDAY($C$5-1,A429))</f>
         <v/>
       </c>
       <c r="C429" s="20" t="str">
@@ -16628,7 +16634,7 @@
         <v/>
       </c>
       <c r="B430" s="19" t="str">
-        <f aca="false">IF(C430="","",$C$5+A430-1)</f>
+        <f aca="false">IF(C430="","",WORKDAY($C$5-1,A430))</f>
         <v/>
       </c>
       <c r="C430" s="20" t="str">
@@ -16665,7 +16671,7 @@
         <v/>
       </c>
       <c r="B431" s="19" t="str">
-        <f aca="false">IF(C431="","",$C$5+A431-1)</f>
+        <f aca="false">IF(C431="","",WORKDAY($C$5-1,A431))</f>
         <v/>
       </c>
       <c r="C431" s="20" t="str">
@@ -16702,7 +16708,7 @@
         <v/>
       </c>
       <c r="B432" s="19" t="str">
-        <f aca="false">IF(C432="","",$C$5+A432-1)</f>
+        <f aca="false">IF(C432="","",WORKDAY($C$5-1,A432))</f>
         <v/>
       </c>
       <c r="C432" s="20" t="str">
@@ -16739,7 +16745,7 @@
         <v/>
       </c>
       <c r="B433" s="19" t="str">
-        <f aca="false">IF(C433="","",$C$5+A433-1)</f>
+        <f aca="false">IF(C433="","",WORKDAY($C$5-1,A433))</f>
         <v/>
       </c>
       <c r="C433" s="20" t="str">
@@ -16776,7 +16782,7 @@
         <v/>
       </c>
       <c r="B434" s="19" t="str">
-        <f aca="false">IF(C434="","",$C$5+A434-1)</f>
+        <f aca="false">IF(C434="","",WORKDAY($C$5-1,A434))</f>
         <v/>
       </c>
       <c r="C434" s="20" t="str">
@@ -16813,7 +16819,7 @@
         <v/>
       </c>
       <c r="B435" s="19" t="str">
-        <f aca="false">IF(C435="","",$C$5+A435-1)</f>
+        <f aca="false">IF(C435="","",WORKDAY($C$5-1,A435))</f>
         <v/>
       </c>
       <c r="C435" s="20" t="str">
@@ -16850,7 +16856,7 @@
         <v/>
       </c>
       <c r="B436" s="19" t="str">
-        <f aca="false">IF(C436="","",$C$5+A436-1)</f>
+        <f aca="false">IF(C436="","",WORKDAY($C$5-1,A436))</f>
         <v/>
       </c>
       <c r="C436" s="20" t="str">
@@ -16887,7 +16893,7 @@
         <v/>
       </c>
       <c r="B437" s="19" t="str">
-        <f aca="false">IF(C437="","",$C$5+A437-1)</f>
+        <f aca="false">IF(C437="","",WORKDAY($C$5-1,A437))</f>
         <v/>
       </c>
       <c r="C437" s="20" t="str">
@@ -16924,7 +16930,7 @@
         <v/>
       </c>
       <c r="B438" s="19" t="str">
-        <f aca="false">IF(C438="","",$C$5+A438-1)</f>
+        <f aca="false">IF(C438="","",WORKDAY($C$5-1,A438))</f>
         <v/>
       </c>
       <c r="C438" s="20" t="str">
@@ -16961,7 +16967,7 @@
         <v/>
       </c>
       <c r="B439" s="19" t="str">
-        <f aca="false">IF(C439="","",$C$5+A439-1)</f>
+        <f aca="false">IF(C439="","",WORKDAY($C$5-1,A439))</f>
         <v/>
       </c>
       <c r="C439" s="20" t="str">
@@ -16998,7 +17004,7 @@
         <v/>
       </c>
       <c r="B440" s="19" t="str">
-        <f aca="false">IF(C440="","",$C$5+A440-1)</f>
+        <f aca="false">IF(C440="","",WORKDAY($C$5-1,A440))</f>
         <v/>
       </c>
       <c r="C440" s="20" t="str">
@@ -17035,7 +17041,7 @@
         <v/>
       </c>
       <c r="B441" s="19" t="str">
-        <f aca="false">IF(C441="","",$C$5+A441-1)</f>
+        <f aca="false">IF(C441="","",WORKDAY($C$5-1,A441))</f>
         <v/>
       </c>
       <c r="C441" s="20" t="str">
@@ -17072,7 +17078,7 @@
         <v/>
       </c>
       <c r="B442" s="19" t="str">
-        <f aca="false">IF(C442="","",$C$5+A442-1)</f>
+        <f aca="false">IF(C442="","",WORKDAY($C$5-1,A442))</f>
         <v/>
       </c>
       <c r="C442" s="20" t="str">
@@ -17109,7 +17115,7 @@
         <v/>
       </c>
       <c r="B443" s="19" t="str">
-        <f aca="false">IF(C443="","",$C$5+A443-1)</f>
+        <f aca="false">IF(C443="","",WORKDAY($C$5-1,A443))</f>
         <v/>
       </c>
       <c r="C443" s="20" t="str">
@@ -17146,7 +17152,7 @@
         <v/>
       </c>
       <c r="B444" s="19" t="str">
-        <f aca="false">IF(C444="","",$C$5+A444-1)</f>
+        <f aca="false">IF(C444="","",WORKDAY($C$5-1,A444))</f>
         <v/>
       </c>
       <c r="C444" s="20" t="str">
@@ -17183,7 +17189,7 @@
         <v/>
       </c>
       <c r="B445" s="19" t="str">
-        <f aca="false">IF(C445="","",$C$5+A445-1)</f>
+        <f aca="false">IF(C445="","",WORKDAY($C$5-1,A445))</f>
         <v/>
       </c>
       <c r="C445" s="20" t="str">
@@ -17220,7 +17226,7 @@
         <v/>
       </c>
       <c r="B446" s="19" t="str">
-        <f aca="false">IF(C446="","",$C$5+A446-1)</f>
+        <f aca="false">IF(C446="","",WORKDAY($C$5-1,A446))</f>
         <v/>
       </c>
       <c r="C446" s="20" t="str">
@@ -17257,7 +17263,7 @@
         <v/>
       </c>
       <c r="B447" s="19" t="str">
-        <f aca="false">IF(C447="","",$C$5+A447-1)</f>
+        <f aca="false">IF(C447="","",WORKDAY($C$5-1,A447))</f>
         <v/>
       </c>
       <c r="C447" s="20" t="str">
@@ -17294,7 +17300,7 @@
         <v/>
       </c>
       <c r="B448" s="19" t="str">
-        <f aca="false">IF(C448="","",$C$5+A448-1)</f>
+        <f aca="false">IF(C448="","",WORKDAY($C$5-1,A448))</f>
         <v/>
       </c>
       <c r="C448" s="20" t="str">
@@ -17331,7 +17337,7 @@
         <v/>
       </c>
       <c r="B449" s="19" t="str">
-        <f aca="false">IF(C449="","",$C$5+A449-1)</f>
+        <f aca="false">IF(C449="","",WORKDAY($C$5-1,A449))</f>
         <v/>
       </c>
       <c r="C449" s="20" t="str">
@@ -17368,7 +17374,7 @@
         <v/>
       </c>
       <c r="B450" s="19" t="str">
-        <f aca="false">IF(C450="","",$C$5+A450-1)</f>
+        <f aca="false">IF(C450="","",WORKDAY($C$5-1,A450))</f>
         <v/>
       </c>
       <c r="C450" s="20" t="str">
@@ -17405,7 +17411,7 @@
         <v/>
       </c>
       <c r="B451" s="19" t="str">
-        <f aca="false">IF(C451="","",$C$5+A451-1)</f>
+        <f aca="false">IF(C451="","",WORKDAY($C$5-1,A451))</f>
         <v/>
       </c>
       <c r="C451" s="20" t="str">
@@ -17442,7 +17448,7 @@
         <v/>
       </c>
       <c r="B452" s="19" t="str">
-        <f aca="false">IF(C452="","",$C$5+A452-1)</f>
+        <f aca="false">IF(C452="","",WORKDAY($C$5-1,A452))</f>
         <v/>
       </c>
       <c r="C452" s="20" t="str">
@@ -17479,7 +17485,7 @@
         <v/>
       </c>
       <c r="B453" s="19" t="str">
-        <f aca="false">IF(C453="","",$C$5+A453-1)</f>
+        <f aca="false">IF(C453="","",WORKDAY($C$5-1,A453))</f>
         <v/>
       </c>
       <c r="C453" s="20" t="str">
@@ -17516,7 +17522,7 @@
         <v/>
       </c>
       <c r="B454" s="19" t="str">
-        <f aca="false">IF(C454="","",$C$5+A454-1)</f>
+        <f aca="false">IF(C454="","",WORKDAY($C$5-1,A454))</f>
         <v/>
       </c>
       <c r="C454" s="20" t="str">
@@ -17553,7 +17559,7 @@
         <v/>
       </c>
       <c r="B455" s="19" t="str">
-        <f aca="false">IF(C455="","",$C$5+A455-1)</f>
+        <f aca="false">IF(C455="","",WORKDAY($C$5-1,A455))</f>
         <v/>
       </c>
       <c r="C455" s="20" t="str">
@@ -17590,7 +17596,7 @@
         <v/>
       </c>
       <c r="B456" s="19" t="str">
-        <f aca="false">IF(C456="","",$C$5+A456-1)</f>
+        <f aca="false">IF(C456="","",WORKDAY($C$5-1,A456))</f>
         <v/>
       </c>
       <c r="C456" s="20" t="str">
@@ -17627,7 +17633,7 @@
         <v/>
       </c>
       <c r="B457" s="19" t="str">
-        <f aca="false">IF(C457="","",$C$5+A457-1)</f>
+        <f aca="false">IF(C457="","",WORKDAY($C$5-1,A457))</f>
         <v/>
       </c>
       <c r="C457" s="20" t="str">
@@ -17664,7 +17670,7 @@
         <v/>
       </c>
       <c r="B458" s="19" t="str">
-        <f aca="false">IF(C458="","",$C$5+A458-1)</f>
+        <f aca="false">IF(C458="","",WORKDAY($C$5-1,A458))</f>
         <v/>
       </c>
       <c r="C458" s="20" t="str">
@@ -17701,7 +17707,7 @@
         <v/>
       </c>
       <c r="B459" s="19" t="str">
-        <f aca="false">IF(C459="","",$C$5+A459-1)</f>
+        <f aca="false">IF(C459="","",WORKDAY($C$5-1,A459))</f>
         <v/>
       </c>
       <c r="C459" s="20" t="str">
@@ -17738,7 +17744,7 @@
         <v/>
       </c>
       <c r="B460" s="19" t="str">
-        <f aca="false">IF(C460="","",$C$5+A460-1)</f>
+        <f aca="false">IF(C460="","",WORKDAY($C$5-1,A460))</f>
         <v/>
       </c>
       <c r="C460" s="20" t="str">
@@ -17775,7 +17781,7 @@
         <v/>
       </c>
       <c r="B461" s="19" t="str">
-        <f aca="false">IF(C461="","",$C$5+A461-1)</f>
+        <f aca="false">IF(C461="","",WORKDAY($C$5-1,A461))</f>
         <v/>
       </c>
       <c r="C461" s="20" t="str">
@@ -17812,7 +17818,7 @@
         <v/>
       </c>
       <c r="B462" s="19" t="str">
-        <f aca="false">IF(C462="","",$C$5+A462-1)</f>
+        <f aca="false">IF(C462="","",WORKDAY($C$5-1,A462))</f>
         <v/>
       </c>
       <c r="C462" s="20" t="str">
@@ -17849,7 +17855,7 @@
         <v/>
       </c>
       <c r="B463" s="19" t="str">
-        <f aca="false">IF(C463="","",$C$5+A463-1)</f>
+        <f aca="false">IF(C463="","",WORKDAY($C$5-1,A463))</f>
         <v/>
       </c>
       <c r="C463" s="20" t="str">
@@ -17886,7 +17892,7 @@
         <v/>
       </c>
       <c r="B464" s="19" t="str">
-        <f aca="false">IF(C464="","",$C$5+A464-1)</f>
+        <f aca="false">IF(C464="","",WORKDAY($C$5-1,A464))</f>
         <v/>
       </c>
       <c r="C464" s="20" t="str">
@@ -17923,7 +17929,7 @@
         <v/>
       </c>
       <c r="B465" s="19" t="str">
-        <f aca="false">IF(C465="","",$C$5+A465-1)</f>
+        <f aca="false">IF(C465="","",WORKDAY($C$5-1,A465))</f>
         <v/>
       </c>
       <c r="C465" s="20" t="str">
@@ -17960,7 +17966,7 @@
         <v/>
       </c>
       <c r="B466" s="19" t="str">
-        <f aca="false">IF(C466="","",$C$5+A466-1)</f>
+        <f aca="false">IF(C466="","",WORKDAY($C$5-1,A466))</f>
         <v/>
       </c>
       <c r="C466" s="20" t="str">
@@ -17997,7 +18003,7 @@
         <v/>
       </c>
       <c r="B467" s="19" t="str">
-        <f aca="false">IF(C467="","",$C$5+A467-1)</f>
+        <f aca="false">IF(C467="","",WORKDAY($C$5-1,A467))</f>
         <v/>
       </c>
       <c r="C467" s="20" t="str">
@@ -18034,7 +18040,7 @@
         <v/>
       </c>
       <c r="B468" s="19" t="str">
-        <f aca="false">IF(C468="","",$C$5+A468-1)</f>
+        <f aca="false">IF(C468="","",WORKDAY($C$5-1,A468))</f>
         <v/>
       </c>
       <c r="C468" s="20" t="str">
@@ -18071,7 +18077,7 @@
         <v/>
       </c>
       <c r="B469" s="19" t="str">
-        <f aca="false">IF(C469="","",$C$5+A469-1)</f>
+        <f aca="false">IF(C469="","",WORKDAY($C$5-1,A469))</f>
         <v/>
       </c>
       <c r="C469" s="20" t="str">
@@ -18108,7 +18114,7 @@
         <v/>
       </c>
       <c r="B470" s="19" t="str">
-        <f aca="false">IF(C470="","",$C$5+A470-1)</f>
+        <f aca="false">IF(C470="","",WORKDAY($C$5-1,A470))</f>
         <v/>
       </c>
       <c r="C470" s="20" t="str">
@@ -18145,7 +18151,7 @@
         <v/>
       </c>
       <c r="B471" s="19" t="str">
-        <f aca="false">IF(C471="","",$C$5+A471-1)</f>
+        <f aca="false">IF(C471="","",WORKDAY($C$5-1,A471))</f>
         <v/>
       </c>
       <c r="C471" s="20" t="str">
@@ -18182,7 +18188,7 @@
         <v/>
       </c>
       <c r="B472" s="19" t="str">
-        <f aca="false">IF(C472="","",$C$5+A472-1)</f>
+        <f aca="false">IF(C472="","",WORKDAY($C$5-1,A472))</f>
         <v/>
       </c>
       <c r="C472" s="20" t="str">
@@ -18219,7 +18225,7 @@
         <v/>
       </c>
       <c r="B473" s="19" t="str">
-        <f aca="false">IF(C473="","",$C$5+A473-1)</f>
+        <f aca="false">IF(C473="","",WORKDAY($C$5-1,A473))</f>
         <v/>
       </c>
       <c r="C473" s="20" t="str">
@@ -18256,7 +18262,7 @@
         <v/>
       </c>
       <c r="B474" s="19" t="str">
-        <f aca="false">IF(C474="","",$C$5+A474-1)</f>
+        <f aca="false">IF(C474="","",WORKDAY($C$5-1,A474))</f>
         <v/>
       </c>
       <c r="C474" s="20" t="str">
@@ -18293,7 +18299,7 @@
         <v/>
       </c>
       <c r="B475" s="19" t="str">
-        <f aca="false">IF(C475="","",$C$5+A475-1)</f>
+        <f aca="false">IF(C475="","",WORKDAY($C$5-1,A475))</f>
         <v/>
       </c>
       <c r="C475" s="20" t="str">
@@ -18330,7 +18336,7 @@
         <v/>
       </c>
       <c r="B476" s="19" t="str">
-        <f aca="false">IF(C476="","",$C$5+A476-1)</f>
+        <f aca="false">IF(C476="","",WORKDAY($C$5-1,A476))</f>
         <v/>
       </c>
       <c r="C476" s="20" t="str">
@@ -18367,7 +18373,7 @@
         <v/>
       </c>
       <c r="B477" s="19" t="str">
-        <f aca="false">IF(C477="","",$C$5+A477-1)</f>
+        <f aca="false">IF(C477="","",WORKDAY($C$5-1,A477))</f>
         <v/>
       </c>
       <c r="C477" s="20" t="str">
@@ -18404,7 +18410,7 @@
         <v/>
       </c>
       <c r="B478" s="19" t="str">
-        <f aca="false">IF(C478="","",$C$5+A478-1)</f>
+        <f aca="false">IF(C478="","",WORKDAY($C$5-1,A478))</f>
         <v/>
       </c>
       <c r="C478" s="20" t="str">
@@ -18441,7 +18447,7 @@
         <v/>
       </c>
       <c r="B479" s="19" t="str">
-        <f aca="false">IF(C479="","",$C$5+A479-1)</f>
+        <f aca="false">IF(C479="","",WORKDAY($C$5-1,A479))</f>
         <v/>
       </c>
       <c r="C479" s="20" t="str">
@@ -18478,7 +18484,7 @@
         <v/>
       </c>
       <c r="B480" s="19" t="str">
-        <f aca="false">IF(C480="","",$C$5+A480-1)</f>
+        <f aca="false">IF(C480="","",WORKDAY($C$5-1,A480))</f>
         <v/>
       </c>
       <c r="C480" s="20" t="str">
@@ -18515,7 +18521,7 @@
         <v/>
       </c>
       <c r="B481" s="19" t="str">
-        <f aca="false">IF(C481="","",$C$5+A481-1)</f>
+        <f aca="false">IF(C481="","",WORKDAY($C$5-1,A481))</f>
         <v/>
       </c>
       <c r="C481" s="20" t="str">
@@ -18552,7 +18558,7 @@
         <v/>
       </c>
       <c r="B482" s="19" t="str">
-        <f aca="false">IF(C482="","",$C$5+A482-1)</f>
+        <f aca="false">IF(C482="","",WORKDAY($C$5-1,A482))</f>
         <v/>
       </c>
       <c r="C482" s="20" t="str">
@@ -18589,7 +18595,7 @@
         <v/>
       </c>
       <c r="B483" s="19" t="str">
-        <f aca="false">IF(C483="","",$C$5+A483-1)</f>
+        <f aca="false">IF(C483="","",WORKDAY($C$5-1,A483))</f>
         <v/>
       </c>
       <c r="C483" s="20" t="str">
@@ -18626,7 +18632,7 @@
         <v/>
       </c>
       <c r="B484" s="19" t="str">
-        <f aca="false">IF(C484="","",$C$5+A484-1)</f>
+        <f aca="false">IF(C484="","",WORKDAY($C$5-1,A484))</f>
         <v/>
       </c>
       <c r="C484" s="20" t="str">
@@ -18663,7 +18669,7 @@
         <v/>
       </c>
       <c r="B485" s="19" t="str">
-        <f aca="false">IF(C485="","",$C$5+A485-1)</f>
+        <f aca="false">IF(C485="","",WORKDAY($C$5-1,A485))</f>
         <v/>
       </c>
       <c r="C485" s="20" t="str">
@@ -18700,7 +18706,7 @@
         <v/>
       </c>
       <c r="B486" s="19" t="str">
-        <f aca="false">IF(C486="","",$C$5+A486-1)</f>
+        <f aca="false">IF(C486="","",WORKDAY($C$5-1,A486))</f>
         <v/>
       </c>
       <c r="C486" s="20" t="str">
@@ -18737,7 +18743,7 @@
         <v/>
       </c>
       <c r="B487" s="19" t="str">
-        <f aca="false">IF(C487="","",$C$5+A487-1)</f>
+        <f aca="false">IF(C487="","",WORKDAY($C$5-1,A487))</f>
         <v/>
       </c>
       <c r="C487" s="20" t="str">
@@ -18774,7 +18780,7 @@
         <v/>
       </c>
       <c r="B488" s="19" t="str">
-        <f aca="false">IF(C488="","",$C$5+A488-1)</f>
+        <f aca="false">IF(C488="","",WORKDAY($C$5-1,A488))</f>
         <v/>
       </c>
       <c r="C488" s="20" t="str">
@@ -18811,7 +18817,7 @@
         <v/>
       </c>
       <c r="B489" s="19" t="str">
-        <f aca="false">IF(C489="","",$C$5+A489-1)</f>
+        <f aca="false">IF(C489="","",WORKDAY($C$5-1,A489))</f>
         <v/>
       </c>
       <c r="C489" s="20" t="str">
@@ -18848,7 +18854,7 @@
         <v/>
       </c>
       <c r="B490" s="19" t="str">
-        <f aca="false">IF(C490="","",$C$5+A490-1)</f>
+        <f aca="false">IF(C490="","",WORKDAY($C$5-1,A490))</f>
         <v/>
       </c>
       <c r="C490" s="20" t="str">
@@ -18885,7 +18891,7 @@
         <v/>
       </c>
       <c r="B491" s="19" t="str">
-        <f aca="false">IF(C491="","",$C$5+A491-1)</f>
+        <f aca="false">IF(C491="","",WORKDAY($C$5-1,A491))</f>
         <v/>
       </c>
       <c r="C491" s="20" t="str">
@@ -18922,7 +18928,7 @@
         <v/>
       </c>
       <c r="B492" s="19" t="str">
-        <f aca="false">IF(C492="","",$C$5+A492-1)</f>
+        <f aca="false">IF(C492="","",WORKDAY($C$5-1,A492))</f>
         <v/>
       </c>
       <c r="C492" s="20" t="str">
@@ -18959,7 +18965,7 @@
         <v/>
       </c>
       <c r="B493" s="19" t="str">
-        <f aca="false">IF(C493="","",$C$5+A493-1)</f>
+        <f aca="false">IF(C493="","",WORKDAY($C$5-1,A493))</f>
         <v/>
       </c>
       <c r="C493" s="20" t="str">
@@ -18996,7 +19002,7 @@
         <v/>
       </c>
       <c r="B494" s="19" t="str">
-        <f aca="false">IF(C494="","",$C$5+A494-1)</f>
+        <f aca="false">IF(C494="","",WORKDAY($C$5-1,A494))</f>
         <v/>
       </c>
       <c r="C494" s="20" t="str">
@@ -19033,7 +19039,7 @@
         <v/>
       </c>
       <c r="B495" s="19" t="str">
-        <f aca="false">IF(C495="","",$C$5+A495-1)</f>
+        <f aca="false">IF(C495="","",WORKDAY($C$5-1,A495))</f>
         <v/>
       </c>
       <c r="C495" s="20" t="str">
@@ -19070,7 +19076,7 @@
         <v/>
       </c>
       <c r="B496" s="19" t="str">
-        <f aca="false">IF(C496="","",$C$5+A496-1)</f>
+        <f aca="false">IF(C496="","",WORKDAY($C$5-1,A496))</f>
         <v/>
       </c>
       <c r="C496" s="20" t="str">
@@ -19107,7 +19113,7 @@
         <v/>
       </c>
       <c r="B497" s="19" t="str">
-        <f aca="false">IF(C497="","",$C$5+A497-1)</f>
+        <f aca="false">IF(C497="","",WORKDAY($C$5-1,A497))</f>
         <v/>
       </c>
       <c r="C497" s="20" t="str">
@@ -19144,7 +19150,7 @@
         <v/>
       </c>
       <c r="B498" s="19" t="str">
-        <f aca="false">IF(C498="","",$C$5+A498-1)</f>
+        <f aca="false">IF(C498="","",WORKDAY($C$5-1,A498))</f>
         <v/>
       </c>
       <c r="C498" s="20" t="str">
@@ -19181,7 +19187,7 @@
         <v/>
       </c>
       <c r="B499" s="19" t="str">
-        <f aca="false">IF(C499="","",$C$5+A499-1)</f>
+        <f aca="false">IF(C499="","",WORKDAY($C$5-1,A499))</f>
         <v/>
       </c>
       <c r="C499" s="20" t="str">
@@ -19218,7 +19224,7 @@
         <v/>
       </c>
       <c r="B500" s="19" t="str">
-        <f aca="false">IF(C500="","",$C$5+A500-1)</f>
+        <f aca="false">IF(C500="","",WORKDAY($C$5-1,A500))</f>
         <v/>
       </c>
       <c r="C500" s="20" t="str">
@@ -19255,7 +19261,7 @@
         <v/>
       </c>
       <c r="B501" s="19" t="str">
-        <f aca="false">IF(C501="","",$C$5+A501-1)</f>
+        <f aca="false">IF(C501="","",WORKDAY($C$5-1,A501))</f>
         <v/>
       </c>
       <c r="C501" s="20" t="str">
@@ -19292,7 +19298,7 @@
         <v/>
       </c>
       <c r="B502" s="19" t="str">
-        <f aca="false">IF(C502="","",$C$5+A502-1)</f>
+        <f aca="false">IF(C502="","",WORKDAY($C$5-1,A502))</f>
         <v/>
       </c>
       <c r="C502" s="20" t="str">
@@ -19329,7 +19335,7 @@
         <v/>
       </c>
       <c r="B503" s="19" t="str">
-        <f aca="false">IF(C503="","",$C$5+A503-1)</f>
+        <f aca="false">IF(C503="","",WORKDAY($C$5-1,A503))</f>
         <v/>
       </c>
       <c r="C503" s="20" t="str">
@@ -19366,7 +19372,7 @@
         <v/>
       </c>
       <c r="B504" s="19" t="str">
-        <f aca="false">IF(C504="","",$C$5+A504-1)</f>
+        <f aca="false">IF(C504="","",WORKDAY($C$5-1,A504))</f>
         <v/>
       </c>
       <c r="C504" s="20" t="str">
@@ -19403,7 +19409,7 @@
         <v/>
       </c>
       <c r="B505" s="19" t="str">
-        <f aca="false">IF(C505="","",$C$5+A505-1)</f>
+        <f aca="false">IF(C505="","",WORKDAY($C$5-1,A505))</f>
         <v/>
       </c>
       <c r="C505" s="20" t="str">
@@ -19440,7 +19446,7 @@
         <v/>
       </c>
       <c r="B506" s="19" t="str">
-        <f aca="false">IF(C506="","",$C$5+A506-1)</f>
+        <f aca="false">IF(C506="","",WORKDAY($C$5-1,A506))</f>
         <v/>
       </c>
       <c r="C506" s="20" t="str">
@@ -19477,7 +19483,7 @@
         <v/>
       </c>
       <c r="B507" s="19" t="str">
-        <f aca="false">IF(C507="","",$C$5+A507-1)</f>
+        <f aca="false">IF(C507="","",WORKDAY($C$5-1,A507))</f>
         <v/>
       </c>
       <c r="C507" s="20" t="str">
@@ -19514,7 +19520,7 @@
         <v/>
       </c>
       <c r="B508" s="19" t="str">
-        <f aca="false">IF(C508="","",$C$5+A508-1)</f>
+        <f aca="false">IF(C508="","",WORKDAY($C$5-1,A508))</f>
         <v/>
       </c>
       <c r="C508" s="20" t="str">
@@ -19551,7 +19557,7 @@
         <v/>
       </c>
       <c r="B509" s="19" t="str">
-        <f aca="false">IF(C509="","",$C$5+A509-1)</f>
+        <f aca="false">IF(C509="","",WORKDAY($C$5-1,A509))</f>
         <v/>
       </c>
       <c r="C509" s="20" t="str">
@@ -19588,7 +19594,7 @@
         <v/>
       </c>
       <c r="B510" s="19" t="str">
-        <f aca="false">IF(C510="","",$C$5+A510-1)</f>
+        <f aca="false">IF(C510="","",WORKDAY($C$5-1,A510))</f>
         <v/>
       </c>
       <c r="C510" s="20" t="str">
@@ -19625,7 +19631,7 @@
         <v/>
       </c>
       <c r="B511" s="19" t="str">
-        <f aca="false">IF(C511="","",$C$5+A511-1)</f>
+        <f aca="false">IF(C511="","",WORKDAY($C$5-1,A511))</f>
         <v/>
       </c>
       <c r="C511" s="20" t="str">
@@ -19662,7 +19668,7 @@
         <v/>
       </c>
       <c r="B512" s="19" t="str">
-        <f aca="false">IF(C512="","",$C$5+A512-1)</f>
+        <f aca="false">IF(C512="","",WORKDAY($C$5-1,A512))</f>
         <v/>
       </c>
       <c r="C512" s="20" t="str">
@@ -19760,7 +19766,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C6F4AB1B-E09F-47F2-9F7E-CE3043892DC8}</x14:id>
+          <x14:id>{596ABDFB-8924-4732-8F3B-D97075E9C277}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -19791,7 +19797,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C6F4AB1B-E09F-47F2-9F7E-CE3043892DC8}">
+          <x14:cfRule type="dataBar" id="{596ABDFB-8924-4732-8F3B-D97075E9C277}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -19816,7 +19822,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -19937,6 +19943,16 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="28" t="s">
         <v>50</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="28" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="28" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: download filled Excel tracker and import from Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USJ2QdZK7Rdpo1YWsPGJTB
</commit_message>
<xml_diff>
--- a/Trading_PnL_Tracker.xlsx
+++ b/Trading_PnL_Tracker.xlsx
@@ -110,7 +110,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="95">
   <si>
     <t xml:space="preserve">Live summary of the Tracker sheet — enter results there, not here. Figures marked * are projections that assume every daily profit target is met; they are illustrations, not guarantees.</t>
   </si>
@@ -351,6 +351,18 @@
   </si>
   <si>
     <t xml:space="preserve">   • The table stops at the first day whose projected (or actual) close reaches the goal, and extends automatically after losses (up to 500 days).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sync with the website dashboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • On the website, "Download Excel" gives you this file filled with everything saved there.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • "Import from Excel" on the website reads this file's Closing Balance, Done?, Notes, Settings and NSE Holidays, and replaces the website's data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • They don't update each other live. Type in one place, then move the data across with those buttons.</t>
   </si>
   <si>
     <t xml:space="preserve">Other notes</t>
@@ -3359,11 +3371,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="71873509"/>
-        <c:axId val="29867929"/>
+        <c:axId val="89161003"/>
+        <c:axId val="26325666"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="71873509"/>
+        <c:axId val="89161003"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3429,7 +3441,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29867929"/>
+        <c:crossAx val="26325666"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3437,7 +3449,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="29867929"/>
+        <c:axId val="26325666"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3513,7 +3525,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71873509"/>
+        <c:crossAx val="89161003"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4644,11 +4656,11 @@
         </c:ser>
         <c:gapWidth val="40"/>
         <c:overlap val="100"/>
-        <c:axId val="25250192"/>
-        <c:axId val="36325388"/>
+        <c:axId val="28709444"/>
+        <c:axId val="4003282"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="25250192"/>
+        <c:axId val="28709444"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4714,7 +4726,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36325388"/>
+        <c:crossAx val="4003282"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4722,7 +4734,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36325388"/>
+        <c:axId val="4003282"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4798,7 +4810,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25250192"/>
+        <c:crossAx val="28709444"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5444,7 +5456,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1DF01534-C5DE-4079-9CE2-48A9ACE0ADD2}</x14:id>
+          <x14:id>{DCCF2CDD-89E7-417B-824B-BF3E469097F4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5481,7 +5493,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1DF01534-C5DE-4079-9CE2-48A9ACE0ADD2}">
+          <x14:cfRule type="dataBar" id="{DCCF2CDD-89E7-417B-824B-BF3E469097F4}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -24300,7 +24312,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{93FCA3E9-B7B4-4178-8D8C-F0A8175D346B}</x14:id>
+          <x14:id>{39EFEA56-12AE-4D78-A16A-D4A8DB88DAA7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24331,7 +24343,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{93FCA3E9-B7B4-4178-8D8C-F0A8175D346B}">
+          <x14:cfRule type="dataBar" id="{39EFEA56-12AE-4D78-A16A-D4A8DB88DAA7}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -25025,7 +25037,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -25139,23 +25151,46 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="47" t="s">
+      <c r="A24" s="45"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="48" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="47" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="47" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="47" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="47" t="s">
         <v>86</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="47" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="47" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="47" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="47" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -25182,19 +25217,19 @@
         <v>31</v>
       </c>
       <c r="B1" s="49" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C1" s="49" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D1" s="49" t="s">
         <v>25</v>
       </c>
       <c r="E1" s="49" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F1" s="49" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>